<commit_message>
v1.1: toast, tasa solo coma, caja banco, conceptos CC, layout 1600px, responsive móvil
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E20"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>08/03/2026</v>
+        <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:14</v>
+        <v>13:09</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -444,16 +444,322 @@
         <v>Setup</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C3" t="str">
+        <v>SQL tablas y seguridad</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Tablas negocio: clientes, tipos_movimiento_caja, ordenes, movimientos_caja, movimientos_cuenta_corriente. Seguridad: roles (Admin, Encargado, Visor), permisos abm_*, RLS, set_user_role.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C4" t="str">
+        <v>UI base y login</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Layout tipo Everfit: sidebar (Inicio, Órdenes, Cajas, Clientes, Cuenta corriente, Seguridad), login/registro, header con logo y user-bar. Auth Supabase, navegación entre vistas. Vista Seguridad: get_users_for_admin + set_user_role.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C5" t="str">
+        <v>ABM Clientes</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Vista Clientes: listado desde Supabase, botón Nuevo cliente (si abm_clientes), modal Alta/Edición con nombre, documento, email, teléfono, dirección, activo. Guardar insert/update.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Vista Cajas</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Saldos USD/EUR/ARS (cards), filtro por moneda, tabla de movimientos. Nuevo movimiento manual: modal con moneda, tipo (tipos_movimiento_caja), monto, concepto, fecha. Signo según tipo ingreso/egreso.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ABM Tipos de movimiento de caja</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Integrado en vista Cajas: listado de tipos, Nuevo tipo y Editar. Campos: nombre, dirección (Ingreso/Egreso), activo. Al cargar se define si es Ingreso o Egreso.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Iconos y regla botones</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Iconos por moneda en Cajas (USA USD, Euro EUR, bandera ARS). Regla: todo botón de acción con icono a la izquierda. Aplicado a Entrar, Crear cuenta, Cerrar sesión, Nuevo/Editar/Guardar/Cancelar en todas las vistas.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Importes y formato</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Campo monto con formato es-AR (miles con punto, decimales con coma). parseImporteInput, formatImporteDisplay, setupInputImporte en modales.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Vista Órdenes</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Listado de órdenes (fecha, cliente, estado, recibido/entregado, cotización). Nueva orden y Editar con modal (cliente, fecha, monedas y montos, estado cotización/cerrada/concertada). Al concertar se crean movimientos de caja y cuenta corriente (una sola vez por orden).</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Edición movimientos de caja</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Botón Editar en cada movimiento. Modal en modo edición: para movimientos manuales se editan moneda, tipo, monto, concepto y fecha; para movimientos por orden solo concepto y fecha.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Vista Cuenta corriente</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Selector de cliente, saldos por moneda (USD, EUR, ARS), tabla de movimientos con filtro por moneda. Convención: positivo = cliente nos debe, negativo = nosotros le debemos.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Vista Inicio</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Resumen con saldos de las 3 cajas (USD, EUR, ARS) y accesos rápidos a Órdenes, Cajas, Clientes y Cuenta corriente.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Convención cuenta corriente</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Corregidos signos al concertar: moneda recibida → monto negativo (nosotros le debemos), moneda entregada → monto positivo (cliente nos debe). Leyenda aclarada en la vista. Script sql/corregir_signos_cuenta_corriente.sql para datos existentes.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Edición movimientos cuenta corriente</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Botón Editar en tabla de movimientos de cuenta corriente (permiso abm_ordenes). Modal para editar concepto y fecha. Guardar actualiza y recarga la vista del cliente.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Responsividad móvil</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Breakpoints 768px y 480px. Touch targets mínimos 44px en botones y menú. Tablas con scroll horizontal y -webkit-overflow-scrolling: touch. Cards y modales adaptados; form dos columnas en una en móvil; inputs font-size 16px en modal para evitar zoom iOS.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Mensajería propia (toast)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Reemplazo de todos los alert() por showToast(): validaciones de órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles. Toasts con tipo success/error/info.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Tasa descuento intermediario y caja banco</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Campo tasa ARS-ARS CHEQUE: solo coma decimal (no punto), mantener coma al escribir decimales. Modal movimiento caja: selector Caja (Efectivo/Banco) para movimientos manuales; caja_tipo guardado en movimientos_caja.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Conceptos CC y layout</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Conceptos cuenta corriente más claros: Conversión de moneda (antes Conversión por tipo de cambio), Comisión del acuerdo (antes Comisión). Layout: max-width 1600px para aprovechar pantalla.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>13:09</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Responsive móvil reforzado</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Safe area insets (notch, barra gestos), body overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y popovers adaptados, form-actions en columna en 480px, títulos y paneles con menos padding.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B21"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -483,9 +789,153 @@
         <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con Log, Resumen, Ref Git y Vercel, Versiones, Tecnología.</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Tablas de negocio (Supabase)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>clientes, tipos_movimiento_caja, ordenes, movimientos_caja, movimientos_cuenta_corriente. Órdenes: cotizacion, cerrada, concertada. CC por cliente y moneda.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Seguridad (Supabase)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Roles Admin/Encargado/Visor. Permisos abm_*. RLS. RPC set_user_role.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>UI base Pandi</v>
+      </c>
+      <c r="B6" t="str">
+        <v>index.html + main.js: sidebar colapsable, login/registro, 6 vistas (Inicio, Órdenes, Cajas, Clientes, Cuenta corriente, Seguridad). Estilos Everfit. Vista Seguridad funcional (asignar rol).</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ABM Clientes</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Listado de clientes (tabla clientes), Nuevo cliente y Editar en modal. Campos: nombre, documento, email, teléfono, dirección, activo. Solo usuarios con permiso abm_clientes pueden crear/editar.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Vista Cajas</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Tres saldos (USD, EUR, ARS) calculados desde movimientos_caja. Filtro por moneda y tabla de movimientos. Alta de movimiento manual con tipo de movimiento (tipos_movimiento_caja), monto positivo; signo según ingreso/egreso.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ABM Tipos de movimiento de caja</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Integrado en Cajas: listado, Nuevo tipo, Editar. Nombre, Dirección (Ingreso/Egreso), Activo. Permiso abm_tipos_movimiento_caja.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Iconos y botones</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Iconos por moneda (USA/Euro/Argentina). Todo botón de acción con icono a la izquierda (Entrar, Guardar, Editar, Nuevo, Cancelar, etc.).</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Vista Órdenes</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Listado, Nueva orden y Editar. Estados: cotización, cerrada, concertada. Al concertar se generan movimientos de caja y cuenta corriente (evita doble concertación).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Edición movimientos de caja</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Editar movimiento: manual (todos los campos) o por orden (solo concepto y fecha).</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Vista Cuenta corriente</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Selector cliente, saldos USD/EUR/ARS, tabla de movimientos con filtro por moneda. Convención: positivo = cliente nos debe, negativo = nosotros le debemos.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Vista Inicio</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Saldos de las 3 cajas y accesos rápidos a Órdenes, Cajas, Clientes, Cuenta corriente.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Convención y corrección CC</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Signos correctos al concertar. sql/corregir_signos_cuenta_corriente.sql para corregir datos ya cargados.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Edición movimientos cuenta corriente</v>
+      </c>
+      <c r="B16" t="str">
+        <v>En vista Cuenta corriente, botón Editar por movimiento. Modal: concepto y fecha. Permiso abm_ordenes.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Responsividad móvil</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Media queries 768px y 480px. Touch 44px, tablas con scroll táctil, modales y cards adaptados, formularios en una columna en móvil.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Mensajería toast</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Todos los avisos y errores con showToast() (success/error/info) en lugar de alert(). Aplicado a órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Movimientos caja efectivo/banco</v>
+      </c>
+      <c r="B19" t="str">
+        <v>En nuevo movimiento de caja: selector Caja (Efectivo o Banco). Los movimientos manuales se guardan con caja_tipo; saldos por tipo en vista Cajas.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Conceptos cuenta corriente</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Layout y responsive</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -555,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -578,15 +1028,26 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>08/03/2026</v>
+        <v>09/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1.1</v>
+      </c>
+      <c r="B3" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.2: quitar título redundante Panel de Control en vista Inicio
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:09</v>
+        <v>13:20</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -750,9 +750,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Panel de Control sin título redundante</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Quitado el h3 "Panel de Control" duplicado dentro de la vista Inicio; el título solo se muestra en el header de la página.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -874,7 +891,7 @@
         <v>Vista Inicio</v>
       </c>
       <c r="B14" t="str">
-        <v>Saldos de las 3 cajas y accesos rápidos a Órdenes, Cajas, Clientes, Cuenta corriente.</v>
+        <v>Saldos de las 3 cajas y accesos rápidos a Órdenes, Cajas, Clientes, Cuenta corriente. Título de vista solo en el header (sin duplicado en el contenido).</v>
       </c>
     </row>
     <row r="15">
@@ -1005,7 +1022,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1045,9 +1062,20 @@
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1.2</v>
+      </c>
+      <c r="B4" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.3: Permisos granulares editar_orden y cambiar_estado_transaccion
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>13:20</v>
+        <v>14:13</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -767,16 +767,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>14:13</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Permisos editar orden y cambiar estado transacción</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Nuevos permisos editar_orden y cambiar_estado_transaccion. Migración SQL (app_permission, app_role_permission, RLS en ordenes, transacciones, mov_cc, instrumentacion, comisiones_orden). Frontend: botones Editar/Transacciones, combo pendiente/ejecutada y Editar transacción según permiso; saveOrden valida permisos.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -950,9 +967,17 @@
         <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Permisos granulares órdenes</v>
+      </c>
+      <c r="B22" t="str">
+        <v>editar_orden: editar datos de orden e instrumentación. cambiar_estado_transaccion: cambiar estado pendiente/ejecutada y editar transacción. Botones y combos en vista Órdenes, panel detalle, modal transacciones pendientes y wizard según permiso; RLS actualizado en Supabase.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1022,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1073,9 +1098,20 @@
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1.3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.4: Logo y favicon desde Emoji-de-WhatsApp-panda
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>14:13</v>
+        <v>15:30</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -784,16 +784,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Favicon y logo de app generados desde JPG del panda. Corrección cropOffset (Y X = 0 262) con sips; PNG 192x192 (logo), 32x32 y 16x16 (pestaña). Logo en círculo (contain), z-index para que sidebar no tape; ?v=2 en links favicon para cache.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -975,9 +992,17 @@
         <v>editar_orden: editar datos de orden e instrumentación. cambiar_estado_transaccion: cambiar estado pendiente/ejecutada y editar transacción. Botones y combos en vista Órdenes, panel detalle, modal transacciones pendientes y wizard según permiso; RLS actualizado en Supabase.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Logo y favicon</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1047,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1109,9 +1134,20 @@
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>1.4</v>
+      </c>
+      <c r="B6" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.5: Tipo operación define monedas (primera=recibida, segunda=entregada); selects en gris
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:30</v>
+        <v>15:57</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -801,16 +801,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>15:57</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Tipo operación define monedas en Nueva orden</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Regla: primera moneda del tipo = recibida, segunda = entregada. Selects Moneda recibida/entregada se rellenan y deshabilitan según tipo (estilo gris). ARS-USD tratado como ARS-DOLAR. Cualquier código XXX-YYY aplica.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1000,9 +1017,17 @@
         <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Tipo de operación y monedas en orden</v>
+      </c>
+      <c r="B24" t="str">
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris); ARS-USD equivalente a ARS-DOLAR.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1072,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1145,9 +1170,20 @@
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>1.5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados. ARS-USD tratado como ARS-DOLAR.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.6: Instrumentación sin intermediario (USD-USD, ARS-USD, etc.): auto-generar 2 transacciones
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +806,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:57</v>
+        <v>16:53</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -818,16 +818,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>16:53</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Transacciones auto sin intermediario</v>
+      </c>
+      <c r="D25" t="str">
+        <v>AutoCompletarInstrumentacionSinIntermediario para USD-USD, ARS-USD, ARS-DOLAR, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1025,9 +1042,17 @@
         <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris); ARS-USD equivalente a ARS-DOLAR.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Instrumentación sin intermediario</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, ARS-DOLAR, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1097,7 +1122,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1181,9 +1206,20 @@
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados. ARS-USD tratado como ARS-DOLAR.</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1.6</v>
+      </c>
+      <c r="B8" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, ARS-DOLAR, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.7: CC intermediario conciliación, transacciones por tipo operación, distribución comisión y alerta 0%
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +806,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -823,7 +823,7 @@
         <v>09/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:53</v>
+        <v>18:16</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -835,9 +835,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>18:16</v>
+      </c>
+      <c r="C26" t="str">
+        <v>v1.7: CC intermediario, transacciones y orden</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Conciliación CC intermediario: cap Debe por moneda al Haber; un solo movimiento Comisión del acuerdo cuando hay tope. Modal transacción: moneda/tipo según operación (Ingreso=moneda recibida, Egreso=entregada). Orden: distribución comisión siempre visible con intermediario; carga desde comisiones_orden al editar; alerta genérica si comisión intermediario 0% (todos los tipos); ARS-USD en split y validaciones.</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1122,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1217,9 +1234,20 @@
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, ARS-DOLAR, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>1.7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>09/03/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.8: ARS-USD/USD-ARS (montos desde TC, sin comisión), anulación de órdenes, baja de transacciones, mensajería interna (showConfirm), estado al instrumentar, ARS-DOLAR eliminado
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -446,10 +446,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -463,10 +463,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -480,10 +480,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -497,10 +497,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -514,10 +514,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -531,10 +531,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -548,10 +548,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -565,10 +565,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -582,10 +582,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -616,10 +616,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -650,10 +650,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -667,10 +667,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -684,10 +684,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -701,10 +701,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -718,10 +718,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -735,10 +735,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -752,10 +752,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -769,10 +769,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -786,10 +786,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -803,16 +803,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
       </c>
       <c r="D24" t="str">
-        <v>Regla: primera moneda del tipo = recibida, segunda = entregada. Selects Moneda recibida/entregada se rellenan y deshabilitan según tipo (estilo gris). ARS-USD tratado como ARS-DOLAR. Cualquier código XXX-YYY aplica.</v>
+        <v>Regla: primera moneda del tipo = recibida, segunda = entregada. Selects Moneda recibida/entregada se rellenan y deshabilitan según tipo (estilo gris). Cualquier código XXX-YYY aplica.</v>
       </c>
       <c r="E24" t="str">
         <v>Desarrollo</v>
@@ -820,16 +820,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
       </c>
       <c r="D25" t="str">
-        <v>AutoCompletarInstrumentacionSinIntermediario para USD-USD, ARS-USD, ARS-DOLAR, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
+        <v>AutoCompletarInstrumentacionSinIntermediario para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
       </c>
       <c r="E25" t="str">
         <v>Desarrollo</v>
@@ -837,10 +837,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>18:16</v>
+        <v>10:20</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -852,16 +852,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>10:20</v>
+      </c>
+      <c r="C27" t="str">
+        <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
+      </c>
+      <c r="D27" t="str">
+        <v>ARS-USD/USD-ARS: foco en tipo de cambio al abrir detalle, sin comisión, cálculo Monto a Recibir/Entregar desde TC (autocompletar con base 1). Anulación de órdenes: estado anulada, botón Anular en tabla y en modal. Baja de transacciones: botón Eliminar por fila. Mensajería interna: showConfirm (modal) reemplaza confirm(); regla en .cursor/rules. Estado de orden: actualizarEstadoOrden tras auto-completar instrumentación (sin intermediario y cheque con intermediario). Eliminación de ARS-DOLAR en código y catálogo.</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B27"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1056,7 +1073,7 @@
         <v>Tipo de operación y monedas en orden</v>
       </c>
       <c r="B24" t="str">
-        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris); ARS-USD equivalente a ARS-DOLAR.</v>
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
       </c>
     </row>
     <row r="25">
@@ -1064,12 +1081,28 @@
         <v>Instrumentación sin intermediario</v>
       </c>
       <c r="B25" t="str">
-        <v>Órdenes sin intermediario (USD-USD, ARS-USD, ARS-DOLAR, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Anulación de órdenes y baja de transacciones</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Estado de orden al instrumentar</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1139,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1162,7 +1195,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -1173,7 +1206,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -1184,7 +1217,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -1195,7 +1228,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -1206,7 +1239,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -1217,10 +1250,10 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C7" t="str">
-        <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados. ARS-USD tratado como ARS-DOLAR.</v>
+        <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
       </c>
     </row>
     <row r="8">
@@ -1228,10 +1261,10 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C8" t="str">
-        <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, ARS-DOLAR, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
+        <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
       </c>
     </row>
     <row r="9">
@@ -1239,15 +1272,26 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>09/03/2026</v>
+        <v>10/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>1.8</v>
+      </c>
+      <c r="B10" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.9: permisos reordenados (7 granulares, sin abm_ordenes)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +806,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -823,7 +823,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -840,7 +840,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -857,7 +857,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>10:20</v>
+        <v>10:43</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -869,9 +869,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>10:43</v>
+      </c>
+      <c r="C28" t="str">
+        <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Migración SQL: nuevos permisos ingresar_orden, editar_orden, anular_orden, editar_estado_orden, ingresar_transacciones, editar_transacciones, eliminar_transacciones; eliminados abm_ordenes, cambiar_estado_transaccion. RLS actualizado. Frontend: todos los botones y combos (Nueva orden, Editar, Anular, estado orden, Nueva transacción, Editar/Eliminar transacción) usan solo los 7 permisos; orden en Seguridad según lista acordada.</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1057,7 +1074,7 @@
         <v>Permisos granulares órdenes</v>
       </c>
       <c r="B22" t="str">
-        <v>editar_orden: editar datos de orden e instrumentación. cambiar_estado_transaccion: cambiar estado pendiente/ejecutada y editar transacción. Botones y combos en vista Órdenes, panel detalle, modal transacciones pendientes y wizard según permiso; RLS actualizado en Supabase.</v>
+        <v>Siete permisos: Ingresar/Editar/Anular Orden, Editar Estado de Orden, Ingresar/Editar/Eliminar Transacciones. Sin abm_ordenes. RLS y frontend (Órdenes, panel, wizard, transacciones pendientes, CC) usan solo estos permisos; orden en Seguridad según lista acordada.</v>
       </c>
     </row>
     <row r="23">
@@ -1172,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1289,9 +1306,20 @@
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1.9</v>
+      </c>
+      <c r="B11" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.10: Panel de Control con tarjetas Efectivo/Banco, órdenes y transacciones pendientes
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +806,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -823,7 +823,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -840,7 +840,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -857,7 +857,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -874,7 +874,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>10:43</v>
+        <v>11:28</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -886,16 +886,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>11:28</v>
+      </c>
+      <c r="C29" t="str">
+        <v>v1.10: Panel de Control rediseñado</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Tarjetas Efectivo y Banco con Saldo Inicial, Saldo Actual (resaltado), Var. por moneda (USD, ARS, EUR en Efectivo; USD, ARS en Banco); iconos por moneda y por caja; sin decimales. Cards Órdenes pendientes (por estado con ojo por fila) y Transacciones pendientes (número en círculo); mismo ancho que Efectivo. Fila Saldo Actual con fondo y negrita.</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1015,111 +1032,119 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Convención y corrección CC</v>
+        <v>Panel de Control (Inicio)</v>
       </c>
       <c r="B15" t="str">
-        <v>Signos correctos al concertar. sql/corregir_signos_cuenta_corriente.sql para corregir datos ya cargados.</v>
+        <v>Tarjetas Efectivo y Banco: Saldo Inicial, Saldo Actual (fila destacada), Var. con icono tendencia; USD/ARS/EUR (Efectivo) y USD/ARS (Banco); iconos por moneda. Cards Órdenes pendientes (por estado, ojo por fila y en título) y Transacciones pendientes (cantidad en círculo); mismo ancho que Efectivo.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Edición movimientos cuenta corriente</v>
+        <v>Convención y corrección CC</v>
       </c>
       <c r="B16" t="str">
-        <v>En vista Cuenta corriente, botón Editar por movimiento. Modal: concepto y fecha. Permiso abm_ordenes.</v>
+        <v>Signos correctos al concertar. sql/corregir_signos_cuenta_corriente.sql para corregir datos ya cargados.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Responsividad móvil</v>
+        <v>Edición movimientos cuenta corriente</v>
       </c>
       <c r="B17" t="str">
-        <v>Media queries 768px y 480px. Touch 44px, tablas con scroll táctil, modales y cards adaptados, formularios en una columna en móvil.</v>
+        <v>En vista Cuenta corriente, botón Editar por movimiento. Modal: concepto y fecha. Permiso abm_ordenes.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Mensajería toast</v>
+        <v>Responsividad móvil</v>
       </c>
       <c r="B18" t="str">
-        <v>Todos los avisos y errores con showToast() (success/error/info) en lugar de alert(). Aplicado a órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles.</v>
+        <v>Media queries 768px y 480px. Touch 44px, tablas con scroll táctil, modales y cards adaptados, formularios en una columna en móvil.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Movimientos caja efectivo/banco</v>
+        <v>Mensajería toast</v>
       </c>
       <c r="B19" t="str">
-        <v>En nuevo movimiento de caja: selector Caja (Efectivo o Banco). Los movimientos manuales se guardan con caja_tipo; saldos por tipo en vista Cajas.</v>
+        <v>Todos los avisos y errores con showToast() (success/error/info) en lugar de alert(). Aplicado a órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Conceptos cuenta corriente</v>
+        <v>Movimientos caja efectivo/banco</v>
       </c>
       <c r="B20" t="str">
-        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
+        <v>En nuevo movimiento de caja: selector Caja (Efectivo o Banco). Los movimientos manuales se guardan con caja_tipo; saldos por tipo en vista Cajas.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Layout y responsive</v>
+        <v>Conceptos cuenta corriente</v>
       </c>
       <c r="B21" t="str">
-        <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
+        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Permisos granulares órdenes</v>
+        <v>Layout y responsive</v>
       </c>
       <c r="B22" t="str">
-        <v>Siete permisos: Ingresar/Editar/Anular Orden, Editar Estado de Orden, Ingresar/Editar/Eliminar Transacciones. Sin abm_ordenes. RLS y frontend (Órdenes, panel, wizard, transacciones pendientes, CC) usan solo estos permisos; orden en Seguridad según lista acordada.</v>
+        <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Logo y favicon</v>
+        <v>Permisos granulares órdenes</v>
       </c>
       <c r="B23" t="str">
-        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
+        <v>Siete permisos: Ingresar/Editar/Anular Orden, Editar Estado de Orden, Ingresar/Editar/Eliminar Transacciones. Sin abm_ordenes. RLS y frontend (Órdenes, panel, wizard, transacciones pendientes, CC) usan solo estos permisos; orden en Seguridad según lista acordada.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Tipo de operación y monedas en orden</v>
+        <v>Logo y favicon</v>
       </c>
       <c r="B24" t="str">
-        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
+        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Instrumentación sin intermediario</v>
+        <v>Tipo de operación y monedas en orden</v>
       </c>
       <c r="B25" t="str">
-        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Anulación de órdenes y baja de transacciones</v>
+        <v>Instrumentación sin intermediario</v>
       </c>
       <c r="B26" t="str">
-        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>Anulación de órdenes y baja de transacciones</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
         <v>Estado de orden al instrumentar</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B28" t="str">
         <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1189,7 +1214,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1317,9 +1342,20 @@
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>1.10</v>
+      </c>
+      <c r="B12" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.11: Permisos de vistas por perfil, Panel parametrizable, Seguridad agrupada y roles colapsados
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +449,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +466,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +483,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +500,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +517,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +534,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +551,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +568,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +585,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +602,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +619,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +636,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +653,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +670,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +687,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +704,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +721,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +738,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +755,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +772,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +789,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +806,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -823,7 +823,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -840,7 +840,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -857,7 +857,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -874,7 +874,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -891,7 +891,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>11:28</v>
+        <v>12:13</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -903,16 +903,84 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>12:13</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Permisos de vistas por perfil</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Migración sql/migracion_permisos_vistas.sql: permisos ver_inicio, ver_ordenes, ver_cajas, ver_clientes, ver_intermediarios, ver_cuenta_corriente, ver_seguridad. Menú lateral y vista por defecto según permisos del rol; redirección si no tiene permiso.</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>12:13</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Panel de Control parametrizable</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Tres permisos: ver_inicio_efectivo, ver_inicio_banco, ver_inicio_pendientes. Tarjetas Efectivo/Banco/Pendientes visibles según permiso; por defecto visor solo tarjetas de pendientes. loadInicio muestra/oculta bloques.</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>12:13</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Seguridad: agrupación y subpermisos</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Permisos por rol agrupados en Permisos de vistas y Permisos de alta, baja o modificación. Subpermisos del Panel (Efectivo, Banco, Pendientes) con sangría y viñeta. Títulos con icono; líneas entre filas; toggles alineados.</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>12:13</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Seguridad: roles colapsados</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Cada rol (Admin, Encargado, Visor) inicia colapsado; clic en el encabezado expande/contrae los permisos. Chevron animado; accesibilidad aria-expanded/aria-controls.</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B31"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1104,47 +1172,71 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Logo y favicon</v>
+        <v>Permisos de vistas</v>
       </c>
       <c r="B24" t="str">
-        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
+        <v>Permisos ver_inicio, ver_ordenes, ver_cajas, ver_clientes, ver_intermediarios, ver_cuenta_corriente, ver_seguridad. Menú y vista por defecto según rol; redirección si no tiene permiso. Migración sql/migracion_permisos_vistas.sql.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Tipo de operación y monedas en orden</v>
+        <v>Panel de Control parametrizable</v>
       </c>
       <c r="B25" t="str">
-        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
+        <v>Tres permisos: ver_inicio_efectivo, ver_inicio_banco, ver_inicio_pendientes. En Inicio se muestran/ocultan tarjetas Efectivo, Banco y bloque Pendientes según permiso. Por defecto visor solo tarjetas de pendientes.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Instrumentación sin intermediario</v>
+        <v>Módulo Seguridad mejorado</v>
       </c>
       <c r="B26" t="str">
-        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+        <v>Permisos por rol agrupados en Permisos de vistas y Permisos de alta, baja o modificación. Subpermisos del Panel con sangría y viñeta. Títulos con icono; filas con separador; roles colapsados al cargar (expandir al clic).</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Anulación de órdenes y baja de transacciones</v>
+        <v>Logo y favicon</v>
       </c>
       <c r="B27" t="str">
-        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>Tipo de operación y monedas en orden</v>
+      </c>
+      <c r="B28" t="str">
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Instrumentación sin intermediario</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Anulación de órdenes y baja de transacciones</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
         <v>Estado de orden al instrumentar</v>
       </c>
-      <c r="B28" t="str">
+      <c r="B31" t="str">
         <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B31"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1214,7 +1306,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1353,9 +1445,20 @@
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>1.11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Guardar antes de mudar a iCloud
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -8,6 +8,7 @@
     <sheet name="Ref Git y Vercel" sheetId="3" r:id="rId3"/>
     <sheet name="Versiones" sheetId="4" r:id="rId4"/>
     <sheet name="Tecnología" sheetId="5" r:id="rId5"/>
+    <sheet name="Presupuesto" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -432,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -449,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -466,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -483,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -500,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -517,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -534,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -551,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -568,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -585,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -602,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -619,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -636,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -653,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -670,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -687,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -704,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -721,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -738,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -755,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -772,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -789,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -806,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -823,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -840,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -857,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -874,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -891,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -908,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -925,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -942,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -959,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:13</v>
+        <v>12:49</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -1007,7 +1008,7 @@
         <v>Bitácora</v>
       </c>
       <c r="B3" t="str">
-        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con Log, Resumen, Ref Git y Vercel, Versiones, Tecnología.</v>
+        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con Log, Resumen, Ref Git y Vercel, Versiones, Tecnología, Presupuesto.</v>
       </c>
     </row>
     <row r="4">
@@ -1508,7 +1509,7 @@
         <v>Bitácora</v>
       </c>
       <c r="B5" t="str">
-        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con Log, Resumen, Ref Git y Vercel, Versiones, Tecnología.</v>
+        <v>Node.js + SheetJS (xlsx). Script scripts/crear-bitacora-excel.js genera Bitacora_tareas.xlsx con Log, Resumen, Ref Git y Vercel, Versiones, Tecnología, Presupuesto.</v>
       </c>
     </row>
   </sheetData>
@@ -1516,4 +1517,231 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D15"/>
+  <cols>
+    <col min="1" max="1" width="52.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Funcionalidad</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Horas hombre</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Importe (USD)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Nuevo</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Setup y arquitectura (repo Supabase Vercel config)</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>456</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Autenticación y seguridad (Auth roles permisos RLS)</v>
+      </c>
+      <c r="B3">
+        <v>24</v>
+      </c>
+      <c r="C3">
+        <v>912</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>UI base y navegación (sidebar vistas login responsive)</v>
+      </c>
+      <c r="B4">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>760</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ABM Clientes (listado alta edición permisos)</v>
+      </c>
+      <c r="B5">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>304</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Módulo Cajas (saldos movimientos tipos Efectivo/Banco)</v>
+      </c>
+      <c r="B6">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>912</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Módulo Órdenes (CRUD estados concertación monedas)</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>1216</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Instrumentación y transacciones (intermediarios comisiones)</v>
+      </c>
+      <c r="B8">
+        <v>28</v>
+      </c>
+      <c r="C8">
+        <v>1064</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Cuenta corriente (cliente e intermediario conciliación)</v>
+      </c>
+      <c r="B9">
+        <v>24</v>
+      </c>
+      <c r="C9">
+        <v>912</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Panel de Control (saldos pendientes accesos parametrizable)</v>
+      </c>
+      <c r="B10">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>608</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Permisos granulares y control de vistas por rol</v>
+      </c>
+      <c r="B11">
+        <v>12</v>
+      </c>
+      <c r="C11">
+        <v>456</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Experiencia de usuario (toast confirm validaciones)</v>
+      </c>
+      <c r="B12">
+        <v>8</v>
+      </c>
+      <c r="C12">
+        <v>304</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Responsive y adaptación móvil (touch safe area)</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <v>456</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Documentación bitácora y despliegue continuo</v>
+      </c>
+      <c r="B14">
+        <v>12</v>
+      </c>
+      <c r="C14">
+        <v>456</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="B15">
+        <v>232</v>
+      </c>
+      <c r="C15">
+        <v>8816</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1.12: Presentación comercial (barra azul, logo transparente, paginado, interlineados)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:49</v>
+        <v>13:49</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -972,16 +972,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B34" t="str">
+        <v>13:49</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Presentación comercial PPT</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Script presentacion/crear_presentacion_pptx.py: barra azul (#0d2137), logo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Presentación</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1235,9 +1252,17 @@
         <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Presentación comercial (PPT)</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1307,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1457,9 +1482,20 @@
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>1.12</v>
+      </c>
+      <c r="B14" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.13: Filtros en Órdenes pendientes; regla de despliegue sin PPT
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>13:49</v>
+        <v>16:07</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -989,16 +989,50 @@
         <v>Presentación</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B35" t="str">
+        <v>16:07</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Filtros en Órdenes pendientes</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Modal Órdenes pendientes: filtros por Cliente, Intermediario y Estado; misma barra y estilos que el resto de la web; re-render al cambiar filtros.</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B36" t="str">
+        <v>16:07</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Regla de despliegue sin PPT</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Flujo de despliegue ya no incluye regenerar PowerPoint; commit sin Propuesta_Pandi.pptx. Reglas bitacora-tareas y reglas-pandi actualizadas.</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Reglas</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1260,9 +1294,17 @@
         <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Filtros en Órdenes pendientes</v>
+      </c>
+      <c r="B33" t="str">
+        <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1332,7 +1374,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1493,9 +1535,20 @@
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>1.13</v>
+      </c>
+      <c r="B15" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.14: Tiempo de inactividad (cierre de sesión automático); solo Admin en Seguridad
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>16:07</v>
+        <v>16:16</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1023,16 +1023,33 @@
         <v>Reglas</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B37" t="str">
+        <v>16:16</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Tiempo de inactividad</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Cierre de sesión automático tras X minutos sin actividad. Solo Admin ve y edita el parámetro en Seguridad. Tabla app_config, sql/app_config_session_timeout.sql.</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1302,9 +1319,17 @@
         <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Tiempo de inactividad</v>
+      </c>
+      <c r="B34" t="str">
+        <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1374,7 +1399,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1546,9 +1571,20 @@
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>1.14</v>
+      </c>
+      <c r="B16" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.15: Sidebar colapsado más visible (flecha, borde, botón)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>16:16</v>
+        <v>16:23</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1040,16 +1040,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B38" t="str">
+        <v>16:23</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Sidebar colapsado más visible</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Borde derecho y sombra cuando está colapsado; botón expandir con fondo, borde y flecha más grande; title/aria-label dinámicos (Expandir/Contraer menú).</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1327,9 +1344,17 @@
         <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Sidebar colapsable</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B35"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1399,7 +1424,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1582,9 +1607,20 @@
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1.15</v>
+      </c>
+      <c r="B17" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.16: iconos cash/Banco en tarjetas, carpeta assets con logos e iconos
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>16:23</v>
+        <v>17:07</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1057,16 +1057,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>17:07</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Iconos y carpeta assets</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Tarjetas Efectivo y Banco con iconos cash.png y Banco.webp. Carpeta assets/ con favicons, logos, iconos monedas y cajas; referencias /assets/ en index.html y crear_presentacion_pptx.py; regla estructura-proyecto.</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1352,9 +1369,17 @@
         <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Carpeta assets</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Logos e iconos en assets/: favicon, logo app, Icono_Dolar/ARS/Euro, cash.png, Banco.webp, SP_logo.svg. En la app se usan como /assets/nombre.ext. Script PPT usa assets/SP_logo.svg.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1424,7 +1449,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1618,9 +1643,20 @@
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>1.16</v>
+      </c>
+      <c r="B18" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.17: Cuenta corriente (filtro Cliente/Intermediario, iconos Panel, Acción); modales amplios y arrastrables
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E44"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>17:07</v>
+        <v>22:53</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1074,16 +1074,101 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B40" t="str">
+        <v>22:53</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Ajustes modal Nueva transacción</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Campo monto con etiqueta según moneda del tipo (Monto (USD/EUR/ARS)); tipo de cambio solo lectura y gris; modo de pago por defecto Ninguno con validación al guardar; mensajería interna (toast).</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B41" t="str">
+        <v>22:53</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Modal transacción: moneda del tipo y conversión inversa</v>
+      </c>
+      <c r="D41" t="str">
+        <v>En operación ARS-USD: ingresos en ARS, egresos en USD. Un solo campo Monto (moneda de la transacción); bloque conversión con tipo de cambio (solo lectura) y monto calculado = conversión inversa (ARS→÷TC otra moneda, USD/EUR→×TC ARS).</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B42" t="str">
+        <v>22:53</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
+      </c>
+      <c r="D42" t="str">
+        <v>tipos_operacion con columnas moneda_in y moneda_out; backfill desde código. Permiso abm_tipos_operacion; RLS INSERT/UPDATE/DELETE. Vista Tipos de operación en menú (solo con permiso); listado y modal Nuevo/Editar (código, nombre, moneda IN, moneda OUT, activo). adaptarFormularioOrden usa monedas del tipo.</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B43" t="str">
+        <v>22:53</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Cuenta corriente: vista Todos y modal detalle</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Vista Cuenta corriente con filtro fijo Todos: una sola tabla con Nombre (cliente/intermediario), Saldo a favor y Saldo negativo por moneda (USD, EUR, ARS) con iconos de moneda en encabezados; botón Ver detalle por fila. Modal Detalle: datos del cliente/intermediario, saldos por moneda (cards) y tabla de movimientos (Debe/Haber); Editar movimiento solo para clientes.</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B44" t="str">
+        <v>22:53</v>
+      </c>
+      <c r="C44" t="str">
+        <v>v1.17: Cuenta corriente y modales</v>
+      </c>
+      <c r="D44" t="str">
+        <v>CC: encabezado por moneda (iconos Panel), Positivo/Negativo, filtro Cliente/Intermediario, solo con saldo; columna Acción; icono Ver detalle limpio. Modales: máximo ancho/alto (95vw, 92vh), arrastrables por header; regla Modales en reglas-pandi.</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B39"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1190,196 +1275,220 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Selector cliente, saldos USD/EUR/ARS, tabla de movimientos con filtro por moneda. Convención: positivo = cliente nos debe, negativo = nosotros le debemos.</v>
+        <v>Tabla por moneda (USD, EUR, ARS) con iconos del Panel; Positivo/Negativo; filtro Cliente/Intermediario; solo entidades con saldo; columna Acción. Ver detalle abre modal con datos, saldos y movimientos. Editar movimiento solo clientes.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Vista Inicio</v>
+        <v>Modales</v>
       </c>
       <c r="B14" t="str">
-        <v>Saldos de las 3 cajas y accesos rápidos a Órdenes, Cajas, Clientes, Cuenta corriente. Título de vista solo en el header (sin duplicado en el contenido).</v>
+        <v>Tamaño amplio (95vw, 92vh). Arrastrables por el header para mover; al cerrar se resetea posición. Estructura .modal-backdrop &gt; .modal &gt; .modal-header + .modal-body.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Panel de Control (Inicio)</v>
+        <v>Vista Inicio</v>
       </c>
       <c r="B15" t="str">
-        <v>Tarjetas Efectivo y Banco: Saldo Inicial, Saldo Actual (fila destacada), Var. con icono tendencia; USD/ARS/EUR (Efectivo) y USD/ARS (Banco); iconos por moneda. Cards Órdenes pendientes (por estado, ojo por fila y en título) y Transacciones pendientes (cantidad en círculo); mismo ancho que Efectivo.</v>
+        <v>Saldos de las 3 cajas y accesos rápidos a Órdenes, Cajas, Clientes, Cuenta corriente. Título de vista solo en el header (sin duplicado en el contenido).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Convención y corrección CC</v>
+        <v>Panel de Control (Inicio)</v>
       </c>
       <c r="B16" t="str">
-        <v>Signos correctos al concertar. sql/corregir_signos_cuenta_corriente.sql para corregir datos ya cargados.</v>
+        <v>Tarjetas Efectivo y Banco: Saldo Inicial, Saldo Actual (fila destacada), Var. con icono tendencia; USD/ARS/EUR (Efectivo) y USD/ARS (Banco); iconos por moneda. Cards Órdenes pendientes (por estado, ojo por fila y en título) y Transacciones pendientes (cantidad en círculo); mismo ancho que Efectivo.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Edición movimientos cuenta corriente</v>
+        <v>Convención y corrección CC</v>
       </c>
       <c r="B17" t="str">
-        <v>En vista Cuenta corriente, botón Editar por movimiento. Modal: concepto y fecha. Permiso abm_ordenes.</v>
+        <v>Signos correctos al concertar. sql/corregir_signos_cuenta_corriente.sql para corregir datos ya cargados.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Responsividad móvil</v>
+        <v>Edición movimientos cuenta corriente</v>
       </c>
       <c r="B18" t="str">
-        <v>Media queries 768px y 480px. Touch 44px, tablas con scroll táctil, modales y cards adaptados, formularios en una columna en móvil.</v>
+        <v>En vista Cuenta corriente, botón Editar por movimiento. Modal: concepto y fecha. Permiso abm_ordenes.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Mensajería toast</v>
+        <v>Responsividad móvil</v>
       </c>
       <c r="B19" t="str">
-        <v>Todos los avisos y errores con showToast() (success/error/info) en lugar de alert(). Aplicado a órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles.</v>
+        <v>Media queries 768px y 480px. Touch 44px, tablas con scroll táctil, modales y cards adaptados, formularios en una columna en móvil.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Movimientos caja efectivo/banco</v>
+        <v>Mensajería toast</v>
       </c>
       <c r="B20" t="str">
-        <v>En nuevo movimiento de caja: selector Caja (Efectivo o Banco). Los movimientos manuales se guardan con caja_tipo; saldos por tipo en vista Cajas.</v>
+        <v>Todos los avisos y errores con showToast() (success/error/info) en lugar de alert(). Aplicado a órdenes, transacciones, movimientos caja/CC, clientes, intermediarios, tipos movimiento, roles.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Conceptos cuenta corriente</v>
+        <v>Movimientos caja efectivo/banco</v>
       </c>
       <c r="B21" t="str">
-        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
+        <v>En nuevo movimiento de caja: selector Caja (Efectivo o Banco). Los movimientos manuales se guardan con caja_tipo; saldos por tipo en vista Cajas.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Layout y responsive</v>
+        <v>Conceptos cuenta corriente</v>
       </c>
       <c r="B22" t="str">
-        <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
+        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Permisos granulares órdenes</v>
+        <v>Layout y responsive</v>
       </c>
       <c r="B23" t="str">
-        <v>Siete permisos: Ingresar/Editar/Anular Orden, Editar Estado de Orden, Ingresar/Editar/Eliminar Transacciones. Sin abm_ordenes. RLS y frontend (Órdenes, panel, wizard, transacciones pendientes, CC) usan solo estos permisos; orden en Seguridad según lista acordada.</v>
+        <v>Contenedor principal hasta 1600px. Móvil: safe area, overflow-x hidden, todos los tabla-wrap con scroll táctil, toasts y form-actions adaptados a 480px.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Permisos de vistas</v>
+        <v>Permisos granulares órdenes</v>
       </c>
       <c r="B24" t="str">
-        <v>Permisos ver_inicio, ver_ordenes, ver_cajas, ver_clientes, ver_intermediarios, ver_cuenta_corriente, ver_seguridad. Menú y vista por defecto según rol; redirección si no tiene permiso. Migración sql/migracion_permisos_vistas.sql.</v>
+        <v>Siete permisos: Ingresar/Editar/Anular Orden, Editar Estado de Orden, Ingresar/Editar/Eliminar Transacciones. Sin abm_ordenes. RLS y frontend (Órdenes, panel, wizard, transacciones pendientes, CC) usan solo estos permisos; orden en Seguridad según lista acordada.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Panel de Control parametrizable</v>
+        <v>Permisos de vistas</v>
       </c>
       <c r="B25" t="str">
-        <v>Tres permisos: ver_inicio_efectivo, ver_inicio_banco, ver_inicio_pendientes. En Inicio se muestran/ocultan tarjetas Efectivo, Banco y bloque Pendientes según permiso. Por defecto visor solo tarjetas de pendientes.</v>
+        <v>Permisos ver_inicio, ver_ordenes, ver_cajas, ver_clientes, ver_intermediarios, ver_cuenta_corriente, ver_seguridad. Menú y vista por defecto según rol; redirección si no tiene permiso. Migración sql/migracion_permisos_vistas.sql.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Módulo Seguridad mejorado</v>
+        <v>Panel de Control parametrizable</v>
       </c>
       <c r="B26" t="str">
-        <v>Permisos por rol agrupados en Permisos de vistas y Permisos de alta, baja o modificación. Subpermisos del Panel con sangría y viñeta. Títulos con icono; filas con separador; roles colapsados al cargar (expandir al clic).</v>
+        <v>Tres permisos: ver_inicio_efectivo, ver_inicio_banco, ver_inicio_pendientes. En Inicio se muestran/ocultan tarjetas Efectivo, Banco y bloque Pendientes según permiso. Por defecto visor solo tarjetas de pendientes.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Logo y favicon</v>
+        <v>Módulo Seguridad mejorado</v>
       </c>
       <c r="B27" t="str">
-        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
+        <v>Permisos por rol agrupados en Permisos de vistas y Permisos de alta, baja o modificación. Subpermisos del Panel con sangría y viñeta. Títulos con icono; filas con separador; roles colapsados al cargar (expandir al clic).</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Tipo de operación y monedas en orden</v>
+        <v>Logo y favicon</v>
       </c>
       <c r="B28" t="str">
-        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
+        <v>Logo de app y favicon de pestaña generados desde Emoji-de-WhatsApp-panda.jpg. Recorte central 675x675 (sips cropOffset 0 262), PNG 192/32/16. Logo en header y login en círculo (object-fit contain); z-index para que no lo tape el sidebar; cache-bust en favicon.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Instrumentación sin intermediario</v>
+        <v>Tipo de operación y monedas en orden</v>
       </c>
       <c r="B29" t="str">
-        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Anulación de órdenes y baja de transacciones</v>
+        <v>Instrumentación sin intermediario</v>
       </c>
       <c r="B30" t="str">
-        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Estado de orden al instrumentar</v>
+        <v>Anulación de órdenes y baja de transacciones</v>
       </c>
       <c r="B31" t="str">
-        <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
+        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Presentación comercial (PPT)</v>
+        <v>Estado de orden al instrumentar</v>
       </c>
       <c r="B32" t="str">
-        <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
+        <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Filtros en Órdenes pendientes</v>
+        <v>Presentación comercial (PPT)</v>
       </c>
       <c r="B33" t="str">
-        <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
+        <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Tiempo de inactividad</v>
+        <v>Filtros en Órdenes pendientes</v>
       </c>
       <c r="B34" t="str">
-        <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
+        <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Sidebar colapsable</v>
+        <v>Tiempo de inactividad</v>
       </c>
       <c r="B35" t="str">
-        <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
+        <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>Sidebar colapsable</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v>Carpeta assets</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B37" t="str">
         <v>Logos e iconos en assets/: favicon, logo app, Icono_Dolar/ARS/Euro, cash.png, Banco.webp, SP_logo.svg. En la app se usan como /assets/nombre.ext. Script PPT usa assets/SP_logo.svg.</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Modal Nueva/Editar transacción</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Un solo campo Monto (moneda de la transacción: ingreso = moneda recibida, egreso = moneda entregada). En operaciones con dos monedas: tipo de cambio solo lectura y monto calculado = conversión inversa (ARS→÷TC, USD/EUR→×TC). Modo de pago por defecto Ninguno con validación; mensajería interna.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B39"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1449,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1654,9 +1763,20 @@
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>1.17</v>
+      </c>
+      <c r="B19" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.18: intermediario en órdenes y transacciones; consistencia en selects
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>22:53</v>
+        <v>23:22</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1159,9 +1159,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B45" t="str">
+        <v>23:22</v>
+      </c>
+      <c r="C45" t="str">
+        <v>v1.18: Intermediario en órdenes y transacciones</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Revisión: guardado y visualización de intermediario en órdenes y modales Órdenes pendientes / Transacciones pendientes correctos. Consistencia: intermediario_id incluido en todos los selects de orden (refresco detalle, validación totales, actualizar estado).</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1558,7 +1575,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1774,9 +1791,20 @@
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.19: wizard instrumentación; seguir agregando transacciones en el mismo paso
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>23:22</v>
+        <v>23:27</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1176,9 +1176,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B46" t="str">
+        <v>23:27</v>
+      </c>
+      <c r="C46" t="str">
+        <v>v1.19: Wizard instrumentación</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Corrección: al guardar la primera transacción desde el paso de instrumentación del alta de orden, el paso dejaba de mostrar la tabla y quedaba en "Cargando…". Definición de canEditarTr en renderWizardList para evitar ReferenceError; se puede seguir agregando transacciones en el mismo paso.</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1575,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1802,9 +1819,20 @@
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>1.19</v>
+      </c>
+      <c r="B21" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.20: cuenta corriente todos los estados; Caja solo ejecutada; auto-complete CC; doc
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>10/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>23:27</v>
+        <v>23:40</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1193,9 +1193,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="B47" t="str">
+        <v>23:40</v>
+      </c>
+      <c r="C47" t="str">
+        <v>v1.20: Cuenta corriente y Caja</v>
+      </c>
+      <c r="D47" t="str">
+        <v>CC refleja todos los movimientos en cualquier estado (pendiente y ejecutada). Caja/Bancos solo cuando transacción ejecutada. Auto-completar instrumentación genera movimientos CC para cada transacción creada; helper insertarMovimientosCcParaTransaccion. Doc docs/CUENTA_CORRIENTE_Y_CAJA.md.</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E47"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1592,7 +1609,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1830,9 +1847,20 @@
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1.20</v>
+      </c>
+      <c r="B22" t="str">
+        <v>10/03/2026</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.21: Permisos por menú colapsables, Cajas Ver granular, cascada padre-hijo, Intermediarios Operar
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E56"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>23:40</v>
+        <v>02:17</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1210,9 +1210,162 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B48" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Cards Cajas como Panel de Control</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Vista Cajas: una sola card Efectivo (USD, ARS, EUR en tabla con header por moneda y fila Saldo) y una sola card Banco (USD, ARS). Misma estructura y clases que Panel (inicio-cajas-dos, inicio-caja-card, inicio-caja-tabla). IDs de saldo sin cambios; setVal mantiene clase inicio-caja-valor para estilos.</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B49" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Propuesta permisos por menú</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Doc docs/PERMISOS_POR_MENU.md: reorganizar UI de permisos para que cada opción de menú (Inicio, Órdenes, Cajas, etc.) tenga Ver y Operar on/off por rol; visibilidad y transaccionalidad de Cajas desde el mismo panel. Implementación futura.</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B50" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Permisos por opción de menú (UI)</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Seguridad: permisos reorganizados por ítem de menú (Panel de Control, Órdenes, Cajas, Clientes, Intermediarios, Tipos de operación, Cuenta corriente, Seguridad). En cada uno: Ver (acceso a la vista e información) y Operar (crear, editar o anular) con leyendas claras desde app_permission. PERMISOS_POR_MENU en main.js; mismo modelo de datos.</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Cajas: Ver granular y mensajes al desactivar</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Permisos ver_cajas_efectivo y ver_cajas_banco (sql/migracion_ver_cajas_efectivo_banco.sql). Vista Cajas muestra tarjeta Efectivo/Banco según permisos. En Seguridad, Ver Efectivo/Banco como subopciones con viñeta. Al desactivar un permiso de Cajas (Ver u Operar) se muestra mensaje aclaratorio (MENSAJE_AL_DESACTIVAR_PERMISO).</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B52" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Seguridad: anclaje y toggles</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Encabezado del rol sticky al hacer scroll; input del toggle con área clicable (position absolute, z-index) para que los on/off respondan al clic.</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Seguridad: menús colapsables</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Cada ítem de menú (Panel, Órdenes, Cajas, etc.) es colapsable/expandible; por defecto colapsado. Mantiene anclaje del rol (padre).</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B54" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Cajas: tarjeta solo por permiso específico</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Tarjetas Efectivo/Banco visibles solo con ver_cajas_efectivo y ver_cajas_banco (quitado fallback ver_cajas) para que Encargado con Banco en off no vea la tarjeta.</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B55" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Intermediarios: Operar en permisos</v>
+      </c>
+      <c r="D55" t="str">
+        <v>abm_intermediarios agregado a PERMISOS_POR_MENU para que aparezca en Operar del ítem Intermediarios en Seguridad.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B56" t="str">
+        <v>02:17</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Seguridad: cascada al desactivar padre</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Al desactivar el permiso padre (acceso al menú) se desactivan también los hijos (resto Ver y Operar) de ese ítem y se actualizan los toggles.</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1286,7 +1439,7 @@
         <v>Vista Cajas</v>
       </c>
       <c r="B8" t="str">
-        <v>Tres saldos (USD, EUR, ARS) calculados desde movimientos_caja. Filtro por moneda y tabla de movimientos. Alta de movimiento manual con tipo de movimiento (tipos_movimiento_caja), monto positivo; signo según ingreso/egreso.</v>
+        <v>Dos cards como Panel: Efectivo y Banco (visibles según ver_cajas_efectivo y ver_cajas_banco). Permisos granulares Ver Efectivo / Ver Banco; al desactivar Ver u Operar en Seguridad se muestra mensaje aclaratorio. Filtro por moneda y tabla de movimientos; ABM movimientos y tipos según permisos.</v>
       </c>
     </row>
     <row r="9">
@@ -1438,7 +1591,7 @@
         <v>Módulo Seguridad mejorado</v>
       </c>
       <c r="B27" t="str">
-        <v>Permisos por rol agrupados en Permisos de vistas y Permisos de alta, baja o modificación. Subpermisos del Panel con sangría y viñeta. Títulos con icono; filas con separador; roles colapsados al cargar (expandir al clic).</v>
+        <v>Permisos por rol agrupados por opción de menú; cada ítem colapsable (por defecto cerrado). Encabezado del rol sticky; toggles on/off clicables. Ver/Operar con leyendas desde app_permission. Al desactivar el acceso al menú (padre) se desactivan también los hijos de ese ítem. Intermediarios incluye Operar (abm_intermediarios).</v>
       </c>
     </row>
     <row r="28">
@@ -1609,7 +1762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -1632,7 +1785,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -1643,7 +1796,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -1654,7 +1807,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -1665,7 +1818,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -1676,7 +1829,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -1687,7 +1840,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -1698,7 +1851,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -1709,7 +1862,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -1720,7 +1873,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -1731,7 +1884,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -1742,7 +1895,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -1753,7 +1906,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -1764,7 +1917,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -1775,7 +1928,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -1786,7 +1939,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -1797,7 +1950,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -1808,7 +1961,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -1819,7 +1972,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -1830,7 +1983,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -1841,7 +1994,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -1852,15 +2005,26 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>10/03/2026</v>
+        <v>11/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>1.21</v>
+      </c>
+      <c r="B23" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.22: CC compromiso solo no ejecutadas, Refrescar, lista completa, misma lógica intermediario
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E59"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>02:17</v>
+        <v>03:11</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1363,9 +1363,60 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B57" t="str">
+        <v>03:11</v>
+      </c>
+      <c r="C57" t="str">
+        <v>CC: refresh con nueva lógica y botón Refrescar</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Tras guardar movimiento CC o cerrar transacción, el modal de detalle actualiza saldos y tabla Operaciones que participan (no solo movimientos). Botón Refrescar en vista Cuenta corriente para recalcular saldos (compromiso − movimientos).</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B58" t="str">
+        <v>03:11</v>
+      </c>
+      <c r="C58" t="str">
+        <v>CC: compromiso solo órdenes no ejecutadas</v>
+      </c>
+      <c r="D58" t="str">
+        <v>El compromiso para el saldo de CC solo incluye órdenes que no están en estado orden_ejecutada. Las órdenes cerradas no suman al compromiso; la ganancia según tipo de operación queda solo en movimientos, evitando que aparezca como saldo a favor en la CC del cliente. Leyenda y docs actualizados.</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B59" t="str">
+        <v>03:11</v>
+      </c>
+      <c r="C59" t="str">
+        <v>v1.22 Despliegue</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Versión 1.22: Cuenta corriente (compromiso solo no ejecutadas, Refrescar, lista completa y misma lógica intermediario).</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1479,7 +1530,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Tabla por moneda (USD, EUR, ARS) con iconos del Panel; Positivo/Negativo; filtro Cliente/Intermediario; solo entidades con saldo; columna Acción. Ver detalle abre modal con datos, saldos y movimientos. Editar movimiento solo clientes.</v>
+        <v>Saldo = compromiso por órdenes no ejecutadas menos movimientos. Órdenes cerradas no suman al compromiso (la ganancia queda solo en movimientos). Tabla por moneda; filtro Cliente/Intermediario; botón Refrescar. Modal detalle: saldos, movimientos y Operaciones que participan.</v>
       </c>
     </row>
     <row r="14">
@@ -1762,7 +1813,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2022,9 +2073,20 @@
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>1.22</v>
+      </c>
+      <c r="B24" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.23: CC sin doble conteo de pendientes
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,21 +1402,55 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:11</v>
+        <v>03:33</v>
       </c>
       <c r="C59" t="str">
+        <v>CC: evitar doble conteo pendientes</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Ajuste saldo CC: los movimientos con concepto "Transacción pendiente" no se restan del compromiso (solo se restan ejecutados/cierre y manuales). Así al ejecutar una pata y quedar la otra pendiente, la CC no se "anula" por doble conteo y concilia correctamente por moneda.</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B60" t="str">
+        <v>03:33</v>
+      </c>
+      <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
       </c>
-      <c r="D59" t="str">
+      <c r="D60" t="str">
         <v>Versión 1.22: Cuenta corriente (compromiso solo no ejecutadas, Refrescar, lista completa y misma lógica intermediario).</v>
       </c>
-      <c r="E59" t="str">
+      <c r="E60" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B61" t="str">
+        <v>03:33</v>
+      </c>
+      <c r="C61" t="str">
+        <v>v1.23 Despliegue</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Versión 1.23: CC concilia sin doble conteo (pendientes no se restan del compromiso); saldos negativos/positivos visibles aunque haya patas pendientes. Actualiza leyenda y doc.</v>
+      </c>
+      <c r="E61" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1813,7 +1847,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2084,9 +2118,20 @@
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>1.23</v>
+      </c>
+      <c r="B25" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.24: ayuda expandible y regla help
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E63"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>03:33</v>
+        <v>03:42</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1448,9 +1448,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B62" t="str">
+        <v>03:42</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Help: popovers expandibles y texto CC</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Los botones de ayuda ahora soportan contenido largo (scroll), se cierran con Escape y la ayuda de Cuenta corriente muestra la explicación completa del cálculo de saldo.</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B63" t="str">
+        <v>03:42</v>
+      </c>
+      <c r="C63" t="str">
+        <v>v1.24 Despliegue</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Versión 1.24: patrón estándar para helps (popover expandible/scroll, cierre con Escape). Regla .cursor/rules/help-popovers.mdc.</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E63"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1847,7 +1881,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2129,9 +2163,20 @@
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>1.24</v>
+      </c>
+      <c r="B26" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.25: help en modal
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E66"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,21 +1470,72 @@
         <v>11/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>03:42</v>
+        <v>03:54</v>
       </c>
       <c r="C63" t="str">
+        <v>Help: leyendas colapsadas por defecto</v>
+      </c>
+      <c r="D63" t="str">
+        <v>La explicación larga ya no se muestra fija en las vistas; queda colapsada por defecto y se ve solo al hacer clic en el icono de ayuda (help).</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B64" t="str">
+        <v>03:54</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Help: modal en toda la app</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Los íconos de ayuda ahora abren un modal de Help (en lugar de popover). Se actualizó la regla .cursor/rules/help-popovers.mdc para el nuevo patrón.</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B65" t="str">
+        <v>03:54</v>
+      </c>
+      <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
       </c>
-      <c r="D63" t="str">
+      <c r="D65" t="str">
         <v>Versión 1.24: patrón estándar para helps (popover expandible/scroll, cierre con Escape). Regla .cursor/rules/help-popovers.mdc.</v>
       </c>
-      <c r="E63" t="str">
+      <c r="E65" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B66" t="str">
+        <v>03:54</v>
+      </c>
+      <c r="C66" t="str">
+        <v>v1.25 Despliegue</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Versión 1.25: ayudas (help) se muestran en modal (no popover) para mejor lectura. El modal se cierra con Escape y click en el backdrop.</v>
+      </c>
+      <c r="E66" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E66"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1881,7 +1932,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2174,9 +2225,20 @@
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>1.25</v>
+      </c>
+      <c r="B27" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.26: Cargar orden por chat (Panel, TC, auto transacciones, redirección)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E71"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>03:54</v>
+        <v>12:16</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1533,16 +1533,101 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B67" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Cargar orden por chat (MVP local)</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Botón "Cargar por chat" en vista Órdenes. Modal con input de texto; interpretación por reglas (montos con moneda, cliente "para X", fecha hoy/mañana). Preview y botón "Confirmar y abrir orden" que rellena el formulario de nueva orden y abre el modal. Solo usuarios con ingresar_orden.</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B68" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Chat orden: tipo de cambio y alta directa</v>
+      </c>
+      <c r="D68" t="str">
+        <v>En ARS-USD/USD-ARS el parser acepta tipo de cambio ("a 1500", "tc 1500", "cotización 1500"). Al confirmar se crean la orden y la instrumentación en Supabase (sin abrir el modal); toast de éxito y recarga del listado.</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B69" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Chat orden: un monto + TC calcula el otro</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Si escribís "recibo 3000 USD a tc 1500 y entrego ARS" el parser calcula los ARS (3000×1500). Soporta "recibo X moneda" y "entrego moneda" sin monto cuando hay tipo de cambio.</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B70" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Botón Cargar por chat: estilo y Panel de Control</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Botón con clase btn-chat (mismo estilo que Nueva orden, color azul #0c6ea8). Cargar por chat también en Panel de Control (Accesos rápidos), visible solo con permiso ingresar_orden.</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B71" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Chat orden: auto-generar transacciones al confirmar</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Al confirmar desde el chat se llama a autoCompletarInstrumentacionSinIntermediario tras crear la instrumentación, para generar las dos transacciones (ingreso/egreso) según tipo de operación.</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E71"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1860,9 +1945,17 @@
         <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Cargar orden por chat</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Botón Cargar por chat (estilo btn-chat, azul) en vista Órdenes y en Panel de Control (Accesos rápidos); visible solo con permiso ingresar_orden. Mensaje en lenguaje natural; con un monto y TC se calcula el otro. Al confirmar se crean orden e instrumentación.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1932,7 +2025,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2236,9 +2329,20 @@
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>1.26</v>
+      </c>
+      <c r="B28" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.27: Modal chat con icono en título y Enviar a la derecha del input
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E72"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>12:16</v>
+        <v>12:32</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1618,9 +1618,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B72" t="str">
+        <v>12:32</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Modal chat: icono en título, Enviar a la derecha del input</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Título del modal con icono de chat; botón Enviar con mismo estilo que el resto (btn-primary); input y Enviar en la misma fila (Enviar a la derecha).</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E72"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2025,7 +2042,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2340,9 +2357,20 @@
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>1.27</v>
+      </c>
+      <c r="B29" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.28: Filtros vista Órdenes, combos select-filtro, quitar Cotización/Concertada del estado
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E73"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>11/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>12:32</v>
+        <v>12:46</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1635,9 +1635,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="B73" t="str">
+        <v>12:46</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Filtros vista Órdenes y estilo combos</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Clase select-filtro para combos de filtros (puntas redondeadas, estilo moderno). Quitar Cotización y Concertada del filtro Estado.</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2042,7 +2059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -2368,9 +2385,20 @@
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>1.28</v>
+      </c>
+      <c r="B30" t="str">
+        <v>11/03/2026</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
WIP: estado actual — reglas configurables, docs, SQL; main.js con error de sintaxis pendiente de corregir en copia local
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E154"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>12:46</v>
+        <v>03:20</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1652,16 +1652,1393 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B74" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
+      </c>
+      <c r="D74" t="str">
+        <v>No se cuentan en CC las transacciones pendientes: solo se insertan movimientos al pasar a ejecutada; al crear transacciones (auto-completar) no se impacta CC. La relación cliente-intermediario no tiene CC propia: los flujos cliente↔intermediario se reflejan en la cuenta Pandy-Intermediario (insertarMovimientosCcParaTransaccion y cambiarEstadoTransaccion).</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B75" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Los compromisos del acuerdo (órdenes no ejecutadas) no participan del saldo: no se suman ni restan. El saldo se calcula solo con movimientos ya ejecutados (loadCuentaCorriente, fetchMovimientosCcPorEntidad, modal detalle). Leyenda y ayuda actualizadas.</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B76" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
+      </c>
+      <c r="D76" t="str">
+        <v>El saldo incluye el efecto de transacciones pendientes (mismo criterio de signos). Ej.: si el cliente pagó 3000 (ejecutada) y Pandy debe pagar 2940 (pendiente), el neto es 60 a favor de Pandy (comisión), no 3000 a favor. loadCuentaCorriente y fetchMovimientosCcPorEntidad actualizados; buildCcResumenRows.</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B77" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Split ingreso cliente→Pandy: ganancia explícita</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Al pasar a ejecutada un ingreso donde cobrador=Pandy y pagador=cliente, si la orden tiene misma moneda y monto_recibido &gt; monto_entregado, se divide: la original pasa a monto_entregado (ej. 2940) y se crea una transacción de ingreso con concepto "Ganancia del acuerdo" por la diferencia (60), ya ejecutada. CC y caja se impactan para ambas.</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B78" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C78" t="str">
+        <v>CC: cuando una parte cumplió, el resto participa</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Propósito de la CC: que Pandy sepa quién le debe o a quién le debe. Si una parte ya cumplió (ej. cliente pagó), la obligación pendiente de Pandy entra en el saldo: se muestra como Negativo (Pandy le debe). Regla: si lo ejecutado del cliente &gt;= lo pendiente que Pandy le debe, saldo = -pendiente (deuda de Pandy). loadCuentaCorriente (pendientePandyDebeCli) y fetchMovimientosCcPorEntidad.</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B79" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Conceptos CC y columnas Pagador/Cobrador</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Movimientos de cuenta corriente con concepto descriptivo: Pago por [moneda] [importe], Cobro por [moneda] [importe], Pago por comisión [moneda] [importe] (helper conceptoCcMovimiento). Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y guardado desde modal transacción. En modal y tablas de transacciones: orden de columnas invertido a Pagador, Cobrador.</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B80" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Orden: numero legible y orden_id obligatorio en CC</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Tabla ordenes: columna numero (integer UNIQUE NOT NULL, secuencia ordenes_numero_seq) como id legible para el cliente. Se muestra en tabla de órdenes (columna Nº), modal Editar orden #X, detalle de orden (Orden #X), transacciones pendientes y detalle CC. Movimientos de cuenta corriente (cliente e intermediario): orden_id obligatorio (NOT NULL); migración backfill desde transaccion→instrumentacion y borrado de huérfanos. Todos los inserts de CC en main.js incluyen orden_id. sql/migracion_orden_numero_y_cc_orden_id.sql.</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B81" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Si la columna ordenes.numero no existe (migración no ejecutada), loadOrdenes y demás selects de ordenes usan fallback: primer error con "numero" pone ordenesTieneNumeroColumn = false y se reintenta sin numero; la vista no muestra error. Nueva orden: al abrir el modal se crea una orden borrador en DB (crearOrdenBorrador); si el usuario cierra sin guardar se elimina en closeModalOrden; al guardar o ir a Instrumentación se deja de considerar borrador. Modal orden: cuando el tipo de operación tiene dos monedas (ARS-USD, USD-ARS, etc.) se oculta el botón Guardar y solo se muestra Instrumentación como acción principal.</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B82" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Cuando el tipo de operación tiene dos monedas: primer campo "El cliente compra [moneda] *" (monto entregado) con foco al abrir el paso detalles; segundo "Tipo de cambio *"; "El cliente vende [moneda] (calculado)" en solo lectura. Fecha y Estado no editables. Orden en DOM: entregado, cotización, recibido. setRestoOrdenEditable respeta monto recibido siempre readOnly en tipos dos monedas; al cambiar a tipo de una moneda se restaura visibilidad de selects de moneda.</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B83" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Órdenes: número visible al volver; carga instrumentación</v>
+      </c>
+      <c r="D83" t="str">
+        <v>loadOrdenes siempre intenta primero con columna numero (selectConNumero) para que al volver a la vista Órdenes el número interno aparezca; solo si falla por columna inexistente se usa selectBase. Paso instrumentación del wizard: mensaje "Cargando instrumentación…" visible al entrar (al hacer clic en Instrumentación y mientras se cargan datos).</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B84" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
+      </c>
+      <c r="D84" t="str">
+        <v>CC simplificada: solo moneda y signo. Conceptos "Cobro por [moneda] [importe]" (Pandy cobró, movimiento positivo) y "Deuda por [moneda] [importe]" (Pandy debe, negativo). Tabla detalle: Fecha, Concepto, Moneda, Importe (con signo); sin columnas Debe/Haber. Resumen: una columna por moneda con importe con signo (+/–). Se generan movimientos sintéticos "Deuda por…" para egresos pendientes (Pandy debe entregar) en el detalle; el saldo incluye lo pendiente. insertarMovimientosCc y guardado desde modal transacción alineados con la convención.</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B85" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C85" t="str">
+        <v>CC momento cero: registros pendientes por moneda</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Al instrumentar orden sin intermediario se insertan 2 registros en movimientos_cuenta_corriente (Deuda del cliente / Deuda de Pandy) con estado pendiente y monto_usd, monto_ars, monto_eur con signo. Al ejecutar una transacción se actualiza el registro existente a cerrado (no se borra ni se inserta nuevo). Saldo = suma solo de filas cerradas; detalle con columnas USD, ARS, EUR y Estado. Migración sql/migracion_cc_monto_por_moneda_y_pendiente.sql; insertarMovimientosCcMomentoCero, cambiarEstadoTransaccion y vista CC actualizadas.</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B86" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C86" t="str">
+        <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Al pasar transacción a ejecutada se actualiza el movimiento de CC a cerrado invirtiendo el signo de monto_usd, monto_ars, monto_eur (y monto si aplica). Al volver a pendiente se invierte de nuevo. El saldo se calcula siempre como suma de toda la tabla (sin filtrar por estado); en momento cero las dos filas se compensan y suma 0.</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B87" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C87" t="str">
+        <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Momento cero: monedas del cliente (lo que entrega = moneda_recibida) con signo negativo; monedas de Pandy (lo que entrega = moneda_entregada) con signo positivo; una columna por fila. Al ejecutar una transacción se invierte solo el signo en la moneda de esa transacción (en la fila correspondiente); la otra moneda no cambia para que el saldo se calcule bien.</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B88" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Editar transacción y CC: respetar momento cero</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Al guardar una transacción editada (saveTransaccion): no se borran las filas de momento cero (las que tienen monto_usd/ars/eur); solo se borran movimientos CC legacy. Si la transacción ya tiene fila de momento cero, no se insertan filas legacy de CC (cobro/deuda); la CC se maneja con la nueva lógica en cambiarEstadoTransaccion.</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B89" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C89" t="str">
+        <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Momento cero: dos filas con ambas monedas (Debe X monR de nro orden N con -mr/-me; Compensación de nro orden N con +mr/+me). Al ejecutar: se marca la fila correspondiente cerrado (sin invertir signos) y se inserta movimiento Cancelación de deuda con + o - según cliente o Pandy pague, usando cotización para la otra moneda. Al volver a pendiente: se borran Cancelación de deuda de esa transacción y la fila vuelve a pendiente. Legacy CC solo para transacciones que no son del momento cero (ej. comisión en debeDividir).</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B90" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C90" t="str">
+        <v>CC momento cero: concepto con número interno de orden</v>
+      </c>
+      <c r="D90" t="str">
+        <v>En insertarMovimientosCcMomentoCero el concepto (Debe / Compensación) usa siempre el número interno de orden (orden.numero); si no viene en el objeto se obtiene con select a ordenes. No se graba el id de Supabase en el concepto.</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B91" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Script truncado y reset secuencia orden</v>
+      </c>
+      <c r="D91" t="str">
+        <v>sql/truncar_ordenes_transacciones.sql: tras truncar tablas transaccionales se ejecuta setval(ordenes_numero_seq, 1, false) para que la próxima orden sea la nº 1.</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B92" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C92" t="str">
+        <v>CC: sin movimientos Conversión de moneda</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Con la nueva lógica de CC (momento cero + Cancelación de deuda) no se generan movimientos con concepto "Conversión de moneda". Eliminadas llamadas a generarMovimientoConversionCc y generarMovimientoConversionCcIntermediario en cambiarEstadoTransaccion y al guardar transacción. Script sql/borrar_movimientos_conversion_moneda.sql para limpiar datos legacy.</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B93" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C93" t="str">
+        <v>CC Cancelación: ambos montos por orden</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Regla CC: al ejecutar una pata se inserta un movimiento "Salda deuda" con ambos montos (ARS/USD/EUR según orden): si ejecuta Cliente → +monto_recibido en moneda_recibida y +monto_entregado en moneda_entregada; si ejecuta Pandy → mismos montos en negativo. La fila de origen solo cambia de estado.</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B94" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C94" t="str">
+        <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Implementada la regla_cc: el resumen de cuenta corriente se calcula solo desde movimientos (cliente vs Pandy e intermediario vs Pandy). Por cada orden, si la suma es positiva → Pandy debe → se muestra solo en la moneda del compromiso (Compensación) en rojo; si la suma es negativa → cliente/intermediario debe → se muestra solo en la moneda del Debe en verde. Sin mostrar +/-.</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B95" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C95" t="str">
+        <v>CC: revisión regla en todos los flujos</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Saldo: se excluyen movimientos con estado anulado (cliente e intermediario). Eliminar transacción: no se permite si tiene movimientos de momento cero (Debe/Compensación); mensaje indica usar Anular orden. Intermediario: solo se revierte (flip monto) al pasar a pendiente, no al ejecutar. Doc docs/FLUJOS_CC_REGLA.md con inventario de flujos que escriben CC.</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B96" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C96" t="str">
+        <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Si en momento cero el usuario guarda un monto distinto al de la orden (ej. 500 en vez de 1000) y pasa a ejecutada: la app cierra la transacción por el monto ejecutado, crea una nueva transacción por la diferencia (pendiente), inserta Cancelación por el monto ejecutado y actualiza filas Debe/Compensación al resto. Saldo correcto (ej. Pandy debe 500). Mismo criterio si se ajusta el egreso.</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B97" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
+      </c>
+      <c r="D97" t="str">
+        <v>En la tabla de transacciones (wizard instrumentación y panel orden) Monto es input editable (blur), Estado y Modo de pago son combos (change). El botón Editar queda para concepto y demás campos. Modo de pago editable coherente con caja/banco. Evita duplicación y permite cambiar monto + estado + modo sin abrir el modal.</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B98" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Al ejecutar la segunda transacción (la creada por el split por 500) el sistema aplicaba de nuevo la lógica de split y creaba otra duplicada. Corrección: solo hacer split cuando la fila Debe (ingreso) o Compensación (egreso) representa más que el monto de la transacción (|monto fila| &gt; monto transacción). Así la transacción "diferencia" al pasarla a ejecutada solo cierra y no genera otra. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B99" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C99" t="str">
+        <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Función insertarMovimientosCcParaTransaccion actualizada con la misma regla que cambiarEstadoTransaccion/saveTransaccion: Int→Pandy cierra Compensación con montos en 0 e inserta solo Cobro; Egreso Pandy→Int cierra Debe con montos en 0, inserta Deuda -montoEfectivoInt y Comisión del acuerdo +monto, más asegurarComisionIntermediario. Usa orden.tasa_descuento_intermediario y orden.moneda_recibida para monto efectivo.</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B100" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C100" t="str">
+        <v>CC intermediario y truncate: número de orden y setval</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Conceptos CC intermediario (Debe/Compensación momento cero) usan siempre el número interno de orden: resolverOrdenLabel en insertarMovimientosCcMomentoCeroIntermediario (orden.numero o select a ordenes); fallback "nro orden ?" si no hay numero. Script sql/truncar_ordenes_transacciones.sql: tras TRUNCATE ordenes se ejecuta setval de la secuencia numero (ordenes_numero_seq o pg_get_serial_sequence) para que la próxima orden sea nº 1.</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B101" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Cancelación de deuda en órdenes misma moneda (monR === monE): usar solo el monto de la transacción (ej. -48.750 cuando Pandy paga al cliente), no la proporción mr/me que daba -50.000 o -51.282. montosCancelacionDesdeOrden, montosCancelacion (cambiarEstadoTransaccion), montosCancelacionItem (guardarSoloMontoTransaccion) y bloques split egreso/ingreso con monR === monE. En ARS-ARS con intermediario: no insertar movimiento CC "Ganancia del acuerdo" ni actualizar la fila del ingreso reducido (asegurarGananciaPandy y revertirGananciaPandy); solo un movimiento positivo por el pago al cliente.</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B102" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C102" t="str">
+        <v>CC cliente: comisión como resultado del split y saldo 0</v>
+      </c>
+      <c r="D102" t="str">
+        <v>La comisión Pandy (1.250) debe ser resultado del split del ingreso 50.000 en dos transacciones (48.750 + 1.250). En misma moneda: no se inserta fila CC "Ganancia"; sí se actualiza la fila Cancelación del ingreso restando la comisión (50.000 → 48.750) en monto_usd/ars/eur según monR. Así la CC muestra +48.750 (ingreso) y -48.750 (egreso) = 0. Revertir: sumar de nuevo la comisión a la fila del ingreso y restaurar monto transacción. asegurarGananciaPandy y revertirGananciaPandy actualizados (update por moneda).</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B103" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C103" t="str">
+        <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Regla sagrada: no tocar los originales (Debe y Compensación). En guardarSoloMontoTransaccion cuando newRestoMonto &lt; 1e-6 solo se actualiza estado a cerrado (no monto_usd/ars/eur a 0). En misma moneda (ARS-ARS): al hacer split se actualiza la Cancelación del ingreso 50.000→48.750; se insertan dos movimientos CC para que la comisión figure y la cuenta cierre en 0: Ganancia del acuerdo +1.250 y Comisión Pandy -1.250. Revertir borra ambos por transaccion_id.</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B104" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Sincronización CC y caja desde orden + transacciones</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Modelo: orden e instrumentación (transacciones) son la fuente de verdad; CC y caja se derivan por conciliación. Función sincronizarCcYCajaDesdeOrden(ordenId): borra movimientos CC (cliente e intermediario) y caja de la orden, recalcula desde todas las transacciones (cobro/deuda, Ganancia del acuerdo, comisión intermediario) e inserta. Invocada al cambiar estado de transacción (cambiarEstadoTransaccion), al guardar monto (guardarSoloMontoTransaccion), al guardar desde modal transacción (saveTransaccion → hacerCierre) y al auto-completar ARS-ARS con intermediario (en lugar de momento cero 2 filas).</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B105" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Al hacer split de egreso (ej. 1000→500 ejecutado, 500 pendiente) la diferencia está en monE (USD). La fila Debe (monR) debe llevar el equivalente en monR (mr*diferencia/me), no -diferencia en monR. Corregido difUsd/difArs/difEur y remUsd/remArs/remEur en ambos bloques (cambiarEstadoTransaccion y saveTransaccion) para que la CC muestre "Pandy debe USD" y no ARS.</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B106" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C106" t="str">
+        <v>CC resumen: agrupar por orden_id para una sola moneda</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Al pasar una operación a pendiente el saldo debe mostrar solo la moneda que corresponde (ej. solo +2000 ARS). Se agrupa por orden_id en loadCuentaCorriente (select con orden_id) y en saldosDesdeMovimientosPorOrden se usa orden_id como clave de agrupación (fallback a parseOrdenNumero en concepto) para que todos los movimientos de la misma orden entren en un solo grupo y el saldo muestre una sola moneda.</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B107" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C107" t="str">
+        <v>CC Cancelación por monto de la transacción</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Al ejecutar una transacción (sin split) se insertaba Cancelación con mr/me (totales de la orden), generando saldo erróneo (ej. 1500 en vez de 1000). Corrección: montosCancelacion(item) usa item.monto; ingreso → +monto en monR y proporcional en monE; egreso → -monto en monE y proporcional en monR. Regla en docs y .cursor/rules: CC siempre debe cerrar con la regla conceptual; si no cierra, preguntar.</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B108" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Split CC: diferencia desde fila, no desde orden</v>
+      </c>
+      <c r="D108" t="str">
+        <v>En el segundo (o n) split se usaba mr/me para la diferencia, generando pendiente erróneo (ej. 800 en vez de 200). Corrección: diferencia = resto en fila Debe/Comp − monto ejecutado. Aplicado en cambiarEstadoTransaccion y saveTransaccion. Así pagos parciales encadenados (500, luego 300) generan 200 pendiente.</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B109" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Tarea de análisis: modal transacción con ejecutadas</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Con transacciones ya ejecutadas, el modal de Editar transacción sigue permitiendo editar todos los campos. Analizar si debe restringirse (solo lectura o bloquear edición cuando hay ejecutadas) para que la regla conceptual de CC se cumpla siempre. Revisar qué hace hoy el guardado y qué sería lo más seguro.</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Análisis pendiente</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B110" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Modal transacción ejecutada: solo concepto editable</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Análisis en docs/ANALISIS_MODAL_TRANSACCION_EJECUTADA.md. Si la transacción está ejecutada, se deshabilitan tipo, modo de pago, moneda, monto, cobrador, pagador, estado y tipo de cambio; solo concepto se puede editar. Mensaje "Transacción cerrada. Solo puede editarse el concepto…". Regla conceptual preservada.</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B111" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Se revierte la restricción del modal: modo de pago, importe y estado siguen editables (tabla y modal) también para ejecutadas. Principio: siempre re-estructurar la regla de CC cuando el usuario edita para que no se rompa. Estado editable para correcciones. Doc ANALISIS actualizado.</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B112" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Reajuste CC y caja al editar monto o modo de pago</v>
+      </c>
+      <c r="D112" t="str">
+        <v>guardarSoloModoPagoTransaccion: si transacción ejecutada, borra mov_caja anterior e inserta uno con el nuevo modo. guardarSoloMontoTransaccion: si ejecutada, revierte Cancelación y caja, actualiza monto y transacción resto (o crea nueva pendiente), inserta nueva Cancelación y caja. saveTransaccion: al editar (id) revierte Cancelación/caja; en split actualiza transacción resto existente en vez de crear otra. Regla conceptual siempre re-estructurada.</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B113" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Si el usuario cambia el monto en la tabla (ej. 500) y luego pasa a Ejecutada sin hacer blur, el sistema usaba el monto en DB (1000) y no creaba la transacción pendiente por 500. En cambiarEstadoTransaccion, antes de ejecutar se lee el valor del input de monto de la fila; si difiere del monto en DB se llama guardarSoloMontoTransaccion y luego se re-ejecuta el cambio de estado, de modo que el split use siempre el monto que ve el usuario.</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B114" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C114" t="str">
+        <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Algunos inserts a movimientos_cuenta_corriente (legacy Cobro/Deuda, Conversión, Comisión) enviaban solo moneda y monto; las columnas monto_usd, monto_ars, monto_eur quedaban null y el saldo se rompía (ej. "Pandy debe 700 USD y 300 ARS" en vez de 1000 USD). Helper montosCcPorMoneda(moneda, valor); todos los inserts a mov_cc ahora incluyen ...montosCcPorMoneda. Script sql/corregir_mov_cc_montos_null.sql para backfill de filas existentes.</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B115" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C115" t="str">
+        <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
+      </c>
+      <c r="D115" t="str">
+        <v>En órdenes ARS-ARS (CHEQUE) con intermediario la ganancia (ej. 1000 ARS) se insertaba como "Cobro por" en CC cliente y el resumen mostraba "cliente debe 1000". Esa suma es la comisión que el cliente ya pagó, no un saldo. Se consulta comisiones_orden (beneficiario=pandy); si la transacción es ingreso cliente→Pandy con monto = comisión Pandy, no se inserta el Cobro en CC cliente. Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B116" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Tasas de descuento: reconocer coma decimal</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Las tasas (cliente e intermediario %) no conservaban la coma al escribir (ej. "2," se convertía en "2"). En formatImporteInputOnType: cuando tieneDecimal, siempre se muestra la coma en el resultado (aunque parteDecimalStr esté vacía). Además con soloComaDecimal se acepta punto como decimal y se convierte a coma ("2.5" → "2,5"). Las tasas usan setupInputImporte(..., 2, true).</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B117" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Modal orden más ancho</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Clase modal-orden con max-width min(95vw, 1400px) para que la tabla de transacciones (Tipo, Modo pago, Moneda, Monto, Pagador, Cobrador, Estado, Editar) tenga más espacio horizontal.</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B118" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
+      </c>
+      <c r="D118" t="str">
+        <v>En órdenes con intermediario (ej. ARS-ARS CHEQUE) no hay filas Debe/Compensación (momento cero), por lo que al editar el importe y pasar a ejecutada no se creaba la transacción "resto" y se rompía instrumentación y CC. Se añade splitSinMomentoCero: al ejecutar con monto menor al compromiso (ingreso pagador=cliente mr&gt;monto, egreso cobrador=cliente me&gt;monto) se crea una transacción pendiente por la diferencia. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo).</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B119" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Split + CC + caja para cualquier tipo de operación</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Verificación: (1) Caja con signo correcto (ingreso/egreso) en cambiarEstadoTransaccion y guardarSoloMontoTransaccion (signoCaja = cobrador===pandy ? 1 : -1). (2) guardarSoloMontoTransaccion sin momento cero: al bajar el monto ejecutado se crea transacción resto pendiente para mantener coherencia. (3) Doc FLUJOS_CC_REGLA.md actualizado con sección "Regla de split en sintonía con CC y caja".</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B120" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
+      </c>
+      <c r="D120" t="str">
+        <v>En ARS-ARS (CHEQUE) las transacciones generadas con modo de pago Cheque no pueden cambiarse a otro modo. guardarSoloModoPagoTransaccion rechaza con toast y onFailure (revierte combo). Tabla wizard y panel: celda modo de pago en solo lectura para esas transacciones. Modal: select modo de pago deshabilitado cuando es orden CHEQUE y la transacción tiene modo cheque.</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B121" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C121" t="str">
+        <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Al ejecutar la última parte que cumple el cliente (suma de ingresos cliente ejecutados &gt;= mr y egresos a cliente ejecutados &gt;= me), se crea automáticamente la transacción "Ganancia del acuerdo" (monto = comisión Pandy de comisiones_orden), estado ejecutada, y su movimiento de caja. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo). Sincroniza instrumentación y CC con la comisión de Pandy.</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B122" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Al ejecutar la transacción de 10k (resto del split 40k→30k) el sistema generaba erróneamente otra transacción de 30k pendiente. Corrección: solo crear transacción "resto" cuando la suma de ingresos/egresos cliente ejecutados (tras esta ejecución) sigue siendo menor que mr/me. Se carga la lista de transacciones y se calculan sumIngresosClienteEjecutados y sumEgresosClienteEjecutados; faltaIngreso/faltaEgreso y diferencia = mr−suma (no mr−montoActual). En cambiarEstadoTransaccion la carga de transacciones se hace después del update para incluir esta transacción ya ejecutada. Aplicado en cambiarEstadoTransaccion, saveTransaccion (continuarFlujo) y guardarSoloMontoTransaccion.</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B123" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Al crear la transacción "Ganancia del acuerdo" (comisión Pandy) en ARS-ARS CHEQUE cuando el cliente completa, la instrumentación quedaba en 41k (30k+10k+1k) y rompía "A recibir 40.000". Se descuenta la comisión de una de las ingresos cliente→Pandy ejecutadas: se elige una con monto&gt;=comisión, se actualiza su monto (ej. 30k→29k), el movimiento de caja y el movimiento de CC (Cancelación) de esa transacción. Así instrumentación suma mr (40k). Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B124" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C124" t="str">
+        <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
+      </c>
+      <c r="D124" t="str">
+        <v>El saldo de cuenta corriente intermediario solo consideraba movimientos ejecutados, por lo que no se mostraba la deuda pendiente (ej. 40.000 del cheque Pandy→Intermediario). Para que la regla sea la misma que con el cliente (saldo real): se cargan transacciones pendientes Pandy→Intermediario por intermediario y moneda; el saldo por moneda es el máximo entre lo que sale de movimientos y lo pendiente. loadCuentaCorriente con fetchPendingPandyIntermediario; buildCcResumenRows con saldosIntermediarioConPendientes; fetchMovimientosCcPorEntidad para intermediario también incorpora pendientes en el saldo del modal detalle.</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B125" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C125" t="str">
+        <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Para igualar la regla con cliente: al instrumentar CHEQUE con intermediario se inserta la fila de momento cero (Debe … nro orden N, monto negativo, pendiente). Al ejecutar el egreso Pandy→Intermediario (cheque) no se inserta una fila nueva; se busca si existe fila con ese transaccion_id y se actualiza a estado cerrado. Si no existe (órdenes sin momento cero), se inserta como antes. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B126" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C126" t="str">
+        <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Reversa ejecutada→pendiente intermediario: ya no se hace flip monto en todas las filas. Solo filas de la transacción revocada: Debe (monto&lt;0) → UPDATE estado pendiente; cobro (monto&gt;0) → DELETE. Aplicado en cambiarEstadoTransaccion y saveTransaccion (revertCcInt). Relojería: dismissAllToasts() al cerrar modal orden y modal transacción; al cerrar modal orden se sincronizan montos de la tabla de instrumentación (guardarSoloMontoTransaccion por input) para no perder cambios sin blur. Doc DIAGNOSTICO_SINCRONIZACION_CC_Y_MODAL.md.</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B127" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Al instrumentar ARS-ARS (CHEQUE) con intermediario no se insertaban registros de momento cero en CC cliente; solo en CC intermediario. La regla debe ser única: en momento cero se cargan ambas cuentas corrientes (cliente con Pandy e intermediario con Pandy). En autoCompletarInstrumentacionChequeConIntermediario se llama ahora también a insertarMovimientosCcMomentoCero(ordenId, orden, ingresoClienteId, egresoClienteId) con las transacciones 1 y 2 (ingreso cliente→Pandy, egreso Pandy→cliente), además de insertarMovimientosCcMomentoCeroIntermediario.</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B128" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C128" t="str">
+        <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
+      </c>
+      <c r="D128" t="str">
+        <v>El INSERT de momento cero fallaba por CHECK estado solo cerrado/anulado. Migración migracion_cc_intermediario_estado_pendiente.sql permite pendiente. Ejecutar en Supabase SQL Editor.</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B129" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Reglas CC, caja e instrucciones: mejoras finales</v>
+      </c>
+      <c r="D129" t="str">
+        <v>eliminarTransaccion: verificación de momento cero también en movimientos_cuenta_corriente_intermediario (no permitir baja si la transacción forma parte del momento cero en CC intermediario). Caja: comentarios que documentan que el saldo solo cuenta movimientos con estado cerrado (anulados no cuentan). guardarSoloModoPagoTransaccion: signo de caja correcto (signoCaja = cobrador===pandy ? 1 : -1) al reinsertar movimiento de caja. Regla conceptual de CC, caja e instrucciones alineada en todos los flujos.</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B130" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C130" t="str">
+        <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Las tablas de CC cliente e intermediario deben ser idénticas. Migración añade monto_usd, monto_ars, monto_eur a movimientos_cuenta_corriente_intermediario. insertarMovimientosCcMomentoCeroIntermediario inserta con esas columnas; loadCuentaCorriente y fetchMovimientosCcPorEntidad las incluyen en el select. Reversa identifica momento cero por monto_usd/ars/eur no null.</v>
+      </c>
+      <c r="E130" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B131" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C131" t="str">
+        <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Al pasar a ejecutada el ingreso Intermediario→Pandy (efectivo) se debe marcar la fila Compensación de momento cero como cerrada y luego insertar el cobro. En insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion se hace primero UPDATE estado cerrado donde transaccion_id y estado pendiente, después INSERT del cobro.</v>
+      </c>
+      <c r="E131" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B132" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C132" t="str">
+        <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
+      </c>
+      <c r="D132" t="str">
+        <v>En momento cero las dos filas (Debe y Compensación) ya suman 0. Se quitó la capa de obligaciones pendientes (transacciones Pandy→Intermediario pendientes) que forzaba mostrar Pandy debe X. Resumen y modal detalle usan solo la suma de movimientos, igual que cliente. Eliminados fetchPendingPandyIntermediario y saldosIntermediarioConPendientes.</v>
+      </c>
+      <c r="E132" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B133" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C133" t="str">
+        <v>CC cliente: Cancelación alineada con monto de la transacción</v>
+      </c>
+      <c r="D133" t="str">
+        <v>La Cancelación de deuda debe usar siempre el monto de la transacción (item.monto), no el total de la orden. Helper montosCancelacionDesdeOrden(item, orden). Al aplicar Ganancia del acuerdo se sincroniza la fila Cancelación del egreso Pandy→cliente con el monto actual de esa transacción. Script sql/corregir_cancelacion_cc_egreso_monto.sql para corregir datos existentes.</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B134" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C134" t="str">
+        <v>CC intermediario: alta de comisión del intermediario</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Al completar el cliente (Ganancia del acuerdo) se inserta en movimientos_cuenta_corriente_intermediario un movimiento "Comisión del acuerdo" por la comisión con beneficiario=intermediario (comisiones_orden), con monto negativo (Pandy paga al intermediario). Una sola vez por orden. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B135" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C135" t="str">
+        <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Al crear la transacción Ganancia del acuerdo se inserta también en movimientos_cuenta_corriente un movimiento con ese concepto y monto (montosCcPorMoneda) para que la CC cliente cierre correctamente. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+      </c>
+      <c r="E135" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B136" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C136" t="str">
+        <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Todos los inserts en movimientos_cuenta_corriente_intermediario incluyen ...montosCcPorMoneda. Al ejecutar el ingreso Int→Pandy se asegura Comisión del acuerdo (comisiones_orden) si no existe. Script sql/corregir_cc_intermediario_montos_null.sql para datos existentes.</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B137" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C137" t="str">
+        <v>CC intermediario: descuento y comisión al entregar cheques</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Al ejecutar ingreso Int→Pandy: se inserta movimiento "Descuento sobre cheque" (-monto) para que la CC cierre (nominal cheque vs efectivo recibido). Al ejecutar egreso Pandy→Int: se crea transacción "Comisión del acuerdo" (egreso Pandy→intermediario), movimiento de caja y movimiento en CC intermediario. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion.</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B138" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C138" t="str">
+        <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
+      </c>
+      <c r="D138" t="str">
+        <v>En saveTransaccion, esOrdenCheque se obtiene desde la orden (tipos_operacion.codigo === ARS-ARS) en lugar del DOM, para que al crear la transacción Ganancia del acuerdo se ejecute siempre el insert en movimientos_cuenta_corriente (movimiento positivo por la comisión) y cierre la CC con el cliente.</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B139" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Nueva tabla orden_comisiones_generadas (orden_id, tipo ganancia_pandy|comision_intermediario, transaccion_id, transaccion_id_reducida). Helpers asegurarGananciaPandy, revertirGananciaPandy, asegurarComisionIntermediario, revertirComisionIntermediario. Al crear: solo si no existe fila. Al pasar ejecutada→pendiente: se revierte comisión (borrar transacción, caja, CC, fila); ingreso Int→Pandy se revierte cobro+descuento y Compensación; si el cliente deja de completar se revierte Ganancia y se restaura ingreso reducido. Migración sql/migracion_orden_comisiones_generadas.sql. Doc FLUJOS_CC_REGLA.md §8.</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B140" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C140" t="str">
+        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
+      </c>
+      <c r="E140" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B141" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B142" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Evitar updates de monto 0 en transacciones</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B143" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C143" t="str">
+        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B144" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C144" t="str">
+        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
+      </c>
+      <c r="E144" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B145" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C145" t="str">
+        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
+      </c>
+      <c r="E145" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B146" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C146" t="str">
+        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
+      </c>
+      <c r="E146" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B147" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C147" t="str">
+        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
+      </c>
+      <c r="E147" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B148" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C148" t="str">
+        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B149" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C149" t="str">
+        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
+      </c>
+      <c r="D149" t="str">
+        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B150" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C150" t="str">
+        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
+      </c>
+      <c r="E150" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B151" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C151" t="str">
+        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
+      </c>
+      <c r="E151" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B152" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C152" t="str">
+        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
+      </c>
+      <c r="D152" t="str">
+        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
+      </c>
+      <c r="E152" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B153" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C153" t="str">
+        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
+      </c>
+      <c r="E153" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B154" t="str">
+        <v>03:20</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Reversar a pendiente: solo una vez por transacción</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
+      </c>
+      <c r="E154" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E154"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B43"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -1768,7 +3145,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Saldo = compromiso por órdenes no ejecutadas menos movimientos. Órdenes cerradas no suman al compromiso (la ganancia queda solo en movimientos). Tabla por moneda; filtro Cliente/Intermediario; botón Refrescar. Modal detalle: saldos, movimientos y Operaciones que participan.</v>
+        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de toda la tabla. Al editar transacción se respetan filas momento cero. Tabla detalle: Fecha, Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
       </c>
     </row>
     <row r="14">
@@ -1840,7 +3217,7 @@
         <v>Conceptos cuenta corriente</v>
       </c>
       <c r="B22" t="str">
-        <v>Textos más claros en CC: Conversión de moneda (ajuste por cotización), Comisión del acuerdo. Incluye compatibilidad con textos legacy al borrar/regenerar.</v>
+        <v>Nueva lógica: solo Debe, Compensación y Cancelación de deuda (sin movimientos "Conversión de moneda"). Script sql/borrar_movimientos_conversion_moneda.sql para limpiar datos legacy.</v>
       </c>
     </row>
     <row r="23">
@@ -1901,95 +3278,119 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Instrumentación sin intermediario</v>
+        <v>Modal orden con dos monedas</v>
       </c>
       <c r="B30" t="str">
-        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
+        <v>En tipos ARS-USD, USD-ARS, etc.: primer campo "El cliente compra [moneda] *" con foco; segundo "Tipo de cambio *"; "El cliente vende [moneda] (calculado)" en solo lectura. Fecha y Estado no editables. Resto de montos calculado automáticamente y no editable.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Anulación de órdenes y baja de transacciones</v>
+        <v>Instrumentación sin intermediario</v>
       </c>
       <c r="B31" t="str">
-        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
+        <v>Órdenes sin intermediario (USD-USD, ARS-USD, USD-ARS, ARS-ARS): al abrir instrumentación vacía se generan automáticamente dos transacciones (ingreso y egreso en efectivo).</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Estado de orden al instrumentar</v>
+        <v>Anulación de órdenes y baja de transacciones</v>
       </c>
       <c r="B32" t="str">
-        <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
+        <v>Estado anulada en órdenes. Botón Anular en tabla y en modal de orden. Botón Eliminar por transacción (dar de baja). No se permite baja si la transacción tiene momento cero en CC cliente o CC intermediario; mensaje indica usar Anular orden. Mensajería interna: showConfirm (modal) en lugar de confirm(); regla en .cursor/rules.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Presentación comercial (PPT)</v>
+        <v>Reglas CC, caja e instrucciones</v>
       </c>
       <c r="B33" t="str">
-        <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
+        <v>Saldo caja: solo movimientos con estado cerrado (anulados no cuentan). Movimientos de caja por transacción ejecutada con signo correcto (Pandy cobra = +, Pandy paga = −) en todos los flujos, incluido guardar solo modo de pago.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Filtros en Órdenes pendientes</v>
+        <v>Estado de orden al instrumentar</v>
       </c>
       <c r="B34" t="str">
-        <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
+        <v>Al auto-completar instrumentación (sin intermediario o cheque con intermediario) se llama actualizarEstadoOrden: la orden pasa de Pendiente Instrumentar a Instrumentación Parcial o Cerrada en Ejecución.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Tiempo de inactividad</v>
+        <v>Presentación comercial (PPT)</v>
       </c>
       <c r="B35" t="str">
-        <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
+        <v>Script presentacion/crear_presentacion_pptx.py genera Propuesta_Pandi.pptx desde Bitácora Presupuesto. Barra azul (#0d2137), logo transparente con contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Sidebar colapsable</v>
+        <v>Filtros en Órdenes pendientes</v>
       </c>
       <c r="B36" t="str">
-        <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
+        <v>En el modal Órdenes pendientes (Panel de Control): filtros por Cliente, Intermediario y Estado; misma vista-toolbar y estilos que Transacciones pendientes; filtrado en memoria y re-render al cambiar.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Carpeta assets</v>
+        <v>Tiempo de inactividad</v>
       </c>
       <c r="B37" t="str">
-        <v>Logos e iconos en assets/: favicon, logo app, Icono_Dolar/ARS/Euro, cash.png, Banco.webp, SP_logo.svg. En la app se usan como /assets/nombre.ext. Script PPT usa assets/SP_logo.svg.</v>
+        <v>En Seguridad (solo Admin): parámetro en minutos. Tras X minutos sin actividad (clic, teclado, scroll) se cierra la sesión automáticamente. Tabla app_config; script sql/app_config_session_timeout.sql.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Modal Nueva/Editar transacción</v>
+        <v>Sidebar colapsable</v>
       </c>
       <c r="B38" t="str">
-        <v>Un solo campo Monto (moneda de la transacción: ingreso = moneda recibida, egreso = moneda entregada). En operaciones con dos monedas: tipo de cambio solo lectura y monto calculado = conversión inversa (ARS→÷TC, USD/EUR→×TC). Modo de pago por defecto Ninguno con validación; mensajería interna.</v>
+        <v>Menú lateral colapsable. Cuando está colapsado: borde derecho y sombra; botón con fondo, borde y flecha grande para expandir; al expandir, botón con flecha para contraer. Aria-label y title dinámicos.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
+        <v>Carpeta assets</v>
       </c>
       <c r="B39" t="str">
-        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
+        <v>Logos e iconos en assets/: favicon, logo app, Icono_Dolar/ARS/Euro, cash.png, Banco.webp, SP_logo.svg. En la app se usan como /assets/nombre.ext. Script PPT usa assets/SP_logo.svg.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v>Modal Nueva/Editar transacción</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Un solo campo Monto (moneda de la transacción: ingreso = moneda recibida, egreso = moneda entregada). En operaciones con dos monedas: tipo de cambio solo lectura y monto calculado = conversión inversa (ARS→÷TC, USD/EUR→×TC). Modo de pago por defecto Ninguno con validación; mensajería interna.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Transacciones: Monto, Estado y Modo de pago en tabla</v>
+      </c>
+      <c r="B41" t="str">
+        <v>En la tabla de transacciones (wizard instrumentación y panel de orden): Monto editable (input, guardado al blur), Estado y Modo de pago como combos (guardado al change). Coherente con caja/banco. Botón Editar solo para concepto y demás campos.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
         <v>Cargar orden por chat</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B43" t="str">
         <v>Botón Cargar por chat (estilo btn-chat, azul) en vista Órdenes y en Panel de Control (Accesos rápidos); visible solo con permiso ingresar_orden. Mensaje en lenguaje natural; con un monto y TC se calcula el otro. Al confirmar se crean orden e instrumentación.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2082,7 +3483,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -2093,7 +3494,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -2104,7 +3505,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -2115,7 +3516,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -2126,7 +3527,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -2137,7 +3538,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -2148,7 +3549,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -2159,7 +3560,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -2170,7 +3571,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -2181,7 +3582,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -2192,7 +3593,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -2203,7 +3604,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -2214,7 +3615,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -2225,7 +3626,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -2236,7 +3637,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -2247,7 +3648,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -2258,7 +3659,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -2269,7 +3670,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -2280,7 +3681,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -2291,7 +3692,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -2302,7 +3703,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -2313,7 +3714,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -2324,7 +3725,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -2335,7 +3736,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -2346,7 +3747,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -2357,7 +3758,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -2368,7 +3769,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -2379,7 +3780,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -2390,7 +3791,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>11/03/2026</v>
+        <v>14/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>

</xml_diff>

<commit_message>
v1.29: Tipos de operación usa_intermediario, switches como Seguridad
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E161"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2558,7 +2558,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C127" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2575,7 +2575,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C128" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2592,7 +2592,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C129" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2609,7 +2609,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C130" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2626,7 +2626,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2643,7 +2643,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C132" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2660,7 +2660,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C133" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2677,7 +2677,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2694,7 +2694,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C135" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2711,7 +2711,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2728,7 +2728,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2745,7 +2745,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2762,7 +2762,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C139" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2779,7 +2779,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C140" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2796,7 +2796,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C141" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2813,7 +2813,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C142" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2830,7 +2830,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C143" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2847,7 +2847,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C144" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -2864,7 +2864,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C145" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -2881,7 +2881,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C146" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -2898,7 +2898,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C147" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -2915,7 +2915,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C148" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -2932,7 +2932,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C149" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -2949,7 +2949,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C150" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -2966,7 +2966,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C151" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -2983,7 +2983,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C152" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3000,7 +3000,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3017,7 +3017,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>03:20</v>
+        <v>18:53</v>
       </c>
       <c r="C154" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3029,16 +3029,135 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B155" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
+      </c>
+      <c r="E155" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B156" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C156" t="str">
+        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
+      </c>
+      <c r="D156" t="str">
+        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
+      </c>
+      <c r="E156" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B157" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Número de transacción interno y convención movimientos de caja</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
+      </c>
+      <c r="E157" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B158" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B159" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+      </c>
+      <c r="E159" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B160" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+      </c>
+      <c r="D160" t="str">
+        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+      </c>
+      <c r="E160" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B161" t="str">
+        <v>18:53</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Tipos de operación: Intermediario Sí/No</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+      </c>
+      <c r="E161" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E154"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E161"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B49"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3388,9 +3507,57 @@
         <v>Botón Cargar por chat (estilo btn-chat, azul) en vista Órdenes y en Panel de Control (Accesos rápidos); visible solo con permiso ingresar_orden. Mensaje en lenguaje natural; con un monto y TC se calcula el otro. Al confirmar se crean orden e instrumentación.</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Tests E2E (Playwright)</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Tests en tests/e2e/: login (pantalla login, login con usuario de prueba, navegación a Panel). Orden ARS-ARS y cuenta corriente: flujo completo (nueva orden tipo ARS-ARS, cliente, importe cheque + tasa, instrumentación, ejecutar las dos transacciones) y verificación de que la CC refleja cada paso. Requisitos: tipo ARS-ARS activo, al menos un cliente, usuario con permisos. Guía docs/TESTING_E2E_GUIA.md.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Número de transacción y convención caja</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Transacciones tienen número interno (transacciones.numero, secuencia) para trazabilidad. Movimientos de caja originados por transacción usan concepto: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Panel de transacciones muestra columna Nro. sql/migracion_transacciones_numero.sql.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Log E2E hoja Caja</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Hoja Caja en Excel: una fila por transacción (y una final) con columnas Saldo_Caja_EF/BA por moneda (Esp, App, Resultado). irACajasYLeerSaldos espera fin de carga para que los saldos no queden en blanco. tests/e2e/orden-cc.spec.js y e2e-log-excel.js.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Movimientos de caja estructurados</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Tabla movimientos_caja con orden_numero y transaccion_numero; vista Cajas: columnas Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Caja, Concepto. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Caja: movimiento por comisión Pandy</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Cuando hay comisión Pandy (misma moneda, sin transacción Ganancia) la sincronización agrega un movimiento de caja (ingreso efectivo por la comisión) para que la caja cierre en cero en operaciones de cobro de cheques. transaccion_id null; al re-sincronizar se borran esos movimientos por orden.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Tipos de operación: Intermediario Sí/No</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3460,7 +3627,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3797,9 +3964,20 @@
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>1.29</v>
+      </c>
+      <c r="B31" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.30: número de orden atómico (MAX+1 con lock en DB)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:E162"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2558,7 +2558,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C127" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2575,7 +2575,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C128" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2592,7 +2592,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C129" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2609,7 +2609,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C130" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2626,7 +2626,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2643,7 +2643,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C132" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2660,7 +2660,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C133" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2677,7 +2677,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2694,7 +2694,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C135" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2711,7 +2711,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2728,7 +2728,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2745,7 +2745,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2762,7 +2762,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C139" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2779,7 +2779,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C140" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2796,7 +2796,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C141" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2813,7 +2813,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C142" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2830,7 +2830,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C143" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2847,7 +2847,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C144" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -2864,7 +2864,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C145" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -2881,7 +2881,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C146" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -2898,7 +2898,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C147" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -2915,7 +2915,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C148" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -2932,7 +2932,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C149" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -2949,7 +2949,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C150" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -2966,7 +2966,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C151" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -2983,7 +2983,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C152" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3000,7 +3000,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3017,7 +3017,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C154" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3034,7 +3034,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C155" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3051,7 +3051,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C156" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3068,7 +3068,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C157" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3085,7 +3085,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C158" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3102,7 +3102,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C159" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3119,7 +3119,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C160" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3136,7 +3136,7 @@
         <v>14/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>18:53</v>
+        <v>21:23</v>
       </c>
       <c r="C161" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3148,16 +3148,33 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="B162" t="str">
+        <v>21:23</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Número de orden MAX+1 atómico en DB</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Función ordenes_insertar_con_proximo_numero en Supabase: asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones. La app llama a la RPC al crear orden nueva (wizard, saveOrden, chat); fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+      </c>
+      <c r="E162" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E161"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E162"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B50"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3555,9 +3572,17 @@
         <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Número de orden atómico (MAX+1)</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B50"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3627,7 +3652,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3975,9 +4000,20 @@
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>1.30</v>
+      </c>
+      <c r="B32" t="str">
+        <v>14/03/2026</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.31: tests E2E reajustados, signos CC regla simple, refresh sin colapsar secciones expandidas
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E167"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2215,10 +2215,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2266,10 +2266,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2283,10 +2283,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2402,10 +2402,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2419,10 +2419,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2436,10 +2436,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2470,10 +2470,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2487,10 +2487,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2521,10 +2521,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2538,16 +2538,16 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C126" t="str">
-        <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
+        <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
       </c>
       <c r="D126" t="str">
-        <v>Reversa ejecutada→pendiente intermediario: ya no se hace flip monto en todas las filas. Solo filas de la transacción revocada: Debe (monto&lt;0) → UPDATE estado pendiente; cobro (monto&gt;0) → DELETE. Aplicado en cambiarEstadoTransaccion y saveTransaccion (revertCcInt). Relojería: dismissAllToasts() al cerrar modal orden y modal transacción; al cerrar modal orden se sincronizan montos de la tabla de instrumentación (guardarSoloMontoTransaccion por input) para no perder cambios sin blur. Doc DIAGNOSTICO_SINCRONIZACION_CC_Y_MODAL.md.</v>
+        <v>Operaciones dos monedas (monR ≠ monE): cuando el cliente paga (ingreso ejecutada), se insertan dos movimientos CC: Cancelación de deuda (+monto en monR) y Contraparte cancelación (-monto en monR, -enMonE en monE). La suma da 0 en USD y solo queda Pandy debe ARS. Aplicado en guardarSoloMontoTransaccion, sincronizarCcYCajaDesdeOrden (Refrescar), saveTransaccion (!tieneMomentoCero). Al revertir se borran ambos conceptos (Cancelación y Contraparte cancelación) en saveTransaccion, guardarSoloMontoTransaccion y cambiarEstadoTransaccion.</v>
       </c>
       <c r="E126" t="str">
         <v>Desarrollo</v>
@@ -2555,16 +2555,16 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C127" t="str">
-        <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
+        <v>CC regla simple: Compromiso y Compromiso Saldado</v>
       </c>
       <c r="D127" t="str">
-        <v>Al instrumentar ARS-ARS (CHEQUE) con intermediario no se insertaban registros de momento cero en CC cliente; solo en CC intermediario. La regla debe ser única: en momento cero se cargan ambas cuentas corrientes (cliente con Pandy e intermediario con Pandy). En autoCompletarInstrumentacionChequeConIntermediario se llama ahora también a insertarMovimientosCcMomentoCero(ordenId, orden, ingresoClienteId, egresoClienteId) con las transacciones 1 y 2 (ingreso cliente→Pandy, egreso Pandy→cliente), además de insertarMovimientosCcMomentoCeroIntermediario.</v>
+        <v>Un registro por evento y por moneda. Momento cero: 2 filas Compromiso (una por moneda, solo esa moneda con valor); concepto "Compromiso - Orden Nro X y Trans Nro Y". Al ejecutar: 1 fila "Compromiso Saldado" por moneda pagada (una moneda por fila). Sin uso de estado para saldo (solo se excluye anulado). transaccion_numero en mov_cc y mov_cc_int (migración sql/migracion_cc_transaccion_numero_y_regla_simple.sql). Doc docs/REGLA_CC_SIMPLE.md. insertarMovimientosCcMomentoCero e Intermediario; sincronizarCcYCajaDesdeOrden con usarReglaSimpleCliente.</v>
       </c>
       <c r="E127" t="str">
         <v>Desarrollo</v>
@@ -2572,16 +2572,16 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C128" t="str">
-        <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
+        <v>CC vista: saldo solo transacciones ejecutadas</v>
       </c>
       <c r="D128" t="str">
-        <v>El INSERT de momento cero fallaba por CHECK estado solo cerrado/anulado. Migración migracion_cc_intermediario_estado_pendiente.sql permite pendiente. Ejecutar en Supabase SQL Editor.</v>
+        <v>En la vista de Cuenta corriente (resumen y modal detalle) el saldo se calcula solo con movimientos que corresponden a transacciones ejecutadas. Si todas están pendientes, nadie le debe nada a nadie. Regla: Compromiso Saldado siempre cuenta; Compromiso solo si la transacción está ejecutada o la orden tiene al menos una ejecutada. loadCuentaCorriente y fetchMovimientosCcPorEntidad cargan transacciones e instrumentación para filtrar antes de sumar.</v>
       </c>
       <c r="E128" t="str">
         <v>Desarrollo</v>
@@ -2589,16 +2589,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C129" t="str">
-        <v>Reglas CC, caja e instrucciones: mejoras finales</v>
+        <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
       </c>
       <c r="D129" t="str">
-        <v>eliminarTransaccion: verificación de momento cero también en movimientos_cuenta_corriente_intermediario (no permitir baja si la transacción forma parte del momento cero en CC intermediario). Caja: comentarios que documentan que el saldo solo cuenta movimientos con estado cerrado (anulados no cuentan). guardarSoloModoPagoTransaccion: signo de caja correcto (signoCaja = cobrador===pandy ? 1 : -1) al reinsertar movimiento de caja. Regla conceptual de CC, caja e instrucciones alineada en todos los flujos.</v>
+        <v>Reversa ejecutada→pendiente intermediario: ya no se hace flip monto en todas las filas. Solo filas de la transacción revocada: Debe (monto&lt;0) → UPDATE estado pendiente; cobro (monto&gt;0) → DELETE. Aplicado en cambiarEstadoTransaccion y saveTransaccion (revertCcInt). Relojería: dismissAllToasts() al cerrar modal orden y modal transacción; al cerrar modal orden se sincronizan montos de la tabla de instrumentación (guardarSoloMontoTransaccion por input) para no perder cambios sin blur. Doc DIAGNOSTICO_SINCRONIZACION_CC_Y_MODAL.md.</v>
       </c>
       <c r="E129" t="str">
         <v>Desarrollo</v>
@@ -2606,16 +2606,16 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C130" t="str">
-        <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
+        <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
       </c>
       <c r="D130" t="str">
-        <v>Las tablas de CC cliente e intermediario deben ser idénticas. Migración añade monto_usd, monto_ars, monto_eur a movimientos_cuenta_corriente_intermediario. insertarMovimientosCcMomentoCeroIntermediario inserta con esas columnas; loadCuentaCorriente y fetchMovimientosCcPorEntidad las incluyen en el select. Reversa identifica momento cero por monto_usd/ars/eur no null.</v>
+        <v>Al instrumentar ARS-ARS (CHEQUE) con intermediario no se insertaban registros de momento cero en CC cliente; solo en CC intermediario. La regla debe ser única: en momento cero se cargan ambas cuentas corrientes (cliente con Pandy e intermediario con Pandy). En autoCompletarInstrumentacionChequeConIntermediario se llama ahora también a insertarMovimientosCcMomentoCero(ordenId, orden, ingresoClienteId, egresoClienteId) con las transacciones 1 y 2 (ingreso cliente→Pandy, egreso Pandy→cliente), además de insertarMovimientosCcMomentoCeroIntermediario.</v>
       </c>
       <c r="E130" t="str">
         <v>Desarrollo</v>
@@ -2623,16 +2623,16 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C131" t="str">
-        <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
+        <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
       </c>
       <c r="D131" t="str">
-        <v>Al pasar a ejecutada el ingreso Intermediario→Pandy (efectivo) se debe marcar la fila Compensación de momento cero como cerrada y luego insertar el cobro. En insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion se hace primero UPDATE estado cerrado donde transaccion_id y estado pendiente, después INSERT del cobro.</v>
+        <v>El INSERT de momento cero fallaba por CHECK estado solo cerrado/anulado. Migración migracion_cc_intermediario_estado_pendiente.sql permite pendiente. Ejecutar en Supabase SQL Editor.</v>
       </c>
       <c r="E131" t="str">
         <v>Desarrollo</v>
@@ -2640,16 +2640,16 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C132" t="str">
-        <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
+        <v>Reglas CC, caja e instrucciones: mejoras finales</v>
       </c>
       <c r="D132" t="str">
-        <v>En momento cero las dos filas (Debe y Compensación) ya suman 0. Se quitó la capa de obligaciones pendientes (transacciones Pandy→Intermediario pendientes) que forzaba mostrar Pandy debe X. Resumen y modal detalle usan solo la suma de movimientos, igual que cliente. Eliminados fetchPendingPandyIntermediario y saldosIntermediarioConPendientes.</v>
+        <v>eliminarTransaccion: verificación de momento cero también en movimientos_cuenta_corriente_intermediario (no permitir baja si la transacción forma parte del momento cero en CC intermediario). Caja: comentarios que documentan que el saldo solo cuenta movimientos con estado cerrado (anulados no cuentan). guardarSoloModoPagoTransaccion: signo de caja correcto (signoCaja = cobrador===pandy ? 1 : -1) al reinsertar movimiento de caja. Regla conceptual de CC, caja e instrucciones alineada en todos los flujos.</v>
       </c>
       <c r="E132" t="str">
         <v>Desarrollo</v>
@@ -2657,16 +2657,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C133" t="str">
-        <v>CC cliente: Cancelación alineada con monto de la transacción</v>
+        <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
       </c>
       <c r="D133" t="str">
-        <v>La Cancelación de deuda debe usar siempre el monto de la transacción (item.monto), no el total de la orden. Helper montosCancelacionDesdeOrden(item, orden). Al aplicar Ganancia del acuerdo se sincroniza la fila Cancelación del egreso Pandy→cliente con el monto actual de esa transacción. Script sql/corregir_cancelacion_cc_egreso_monto.sql para corregir datos existentes.</v>
+        <v>Las tablas de CC cliente e intermediario deben ser idénticas. Migración añade monto_usd, monto_ars, monto_eur a movimientos_cuenta_corriente_intermediario. insertarMovimientosCcMomentoCeroIntermediario inserta con esas columnas; loadCuentaCorriente y fetchMovimientosCcPorEntidad las incluyen en el select. Reversa identifica momento cero por monto_usd/ars/eur no null.</v>
       </c>
       <c r="E133" t="str">
         <v>Desarrollo</v>
@@ -2674,16 +2674,16 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C134" t="str">
-        <v>CC intermediario: alta de comisión del intermediario</v>
+        <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
       </c>
       <c r="D134" t="str">
-        <v>Al completar el cliente (Ganancia del acuerdo) se inserta en movimientos_cuenta_corriente_intermediario un movimiento "Comisión del acuerdo" por la comisión con beneficiario=intermediario (comisiones_orden), con monto negativo (Pandy paga al intermediario). Una sola vez por orden. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>Al pasar a ejecutada el ingreso Intermediario→Pandy (efectivo) se debe marcar la fila Compensación de momento cero como cerrada y luego insertar el cobro. En insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion se hace primero UPDATE estado cerrado donde transaccion_id y estado pendiente, después INSERT del cobro.</v>
       </c>
       <c r="E134" t="str">
         <v>Desarrollo</v>
@@ -2691,16 +2691,16 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C135" t="str">
-        <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
+        <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
       </c>
       <c r="D135" t="str">
-        <v>Al crear la transacción Ganancia del acuerdo se inserta también en movimientos_cuenta_corriente un movimiento con ese concepto y monto (montosCcPorMoneda) para que la CC cliente cierre correctamente. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>En momento cero las dos filas (Debe y Compensación) ya suman 0. Se quitó la capa de obligaciones pendientes (transacciones Pandy→Intermediario pendientes) que forzaba mostrar Pandy debe X. Resumen y modal detalle usan solo la suma de movimientos, igual que cliente. Eliminados fetchPendingPandyIntermediario y saldosIntermediarioConPendientes.</v>
       </c>
       <c r="E135" t="str">
         <v>Desarrollo</v>
@@ -2708,16 +2708,16 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C136" t="str">
-        <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
+        <v>CC cliente: Cancelación alineada con monto de la transacción</v>
       </c>
       <c r="D136" t="str">
-        <v>Todos los inserts en movimientos_cuenta_corriente_intermediario incluyen ...montosCcPorMoneda. Al ejecutar el ingreso Int→Pandy se asegura Comisión del acuerdo (comisiones_orden) si no existe. Script sql/corregir_cc_intermediario_montos_null.sql para datos existentes.</v>
+        <v>La Cancelación de deuda debe usar siempre el monto de la transacción (item.monto), no el total de la orden. Helper montosCancelacionDesdeOrden(item, orden). Al aplicar Ganancia del acuerdo se sincroniza la fila Cancelación del egreso Pandy→cliente con el monto actual de esa transacción. Script sql/corregir_cancelacion_cc_egreso_monto.sql para corregir datos existentes.</v>
       </c>
       <c r="E136" t="str">
         <v>Desarrollo</v>
@@ -2725,16 +2725,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C137" t="str">
-        <v>CC intermediario: descuento y comisión al entregar cheques</v>
+        <v>CC intermediario: alta de comisión del intermediario</v>
       </c>
       <c r="D137" t="str">
-        <v>Al ejecutar ingreso Int→Pandy: se inserta movimiento "Descuento sobre cheque" (-monto) para que la CC cierre (nominal cheque vs efectivo recibido). Al ejecutar egreso Pandy→Int: se crea transacción "Comisión del acuerdo" (egreso Pandy→intermediario), movimiento de caja y movimiento en CC intermediario. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>Al completar el cliente (Ganancia del acuerdo) se inserta en movimientos_cuenta_corriente_intermediario un movimiento "Comisión del acuerdo" por la comisión con beneficiario=intermediario (comisiones_orden), con monto negativo (Pandy paga al intermediario). Una sola vez por orden. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E137" t="str">
         <v>Desarrollo</v>
@@ -2742,16 +2742,16 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C138" t="str">
-        <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
+        <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
       </c>
       <c r="D138" t="str">
-        <v>En saveTransaccion, esOrdenCheque se obtiene desde la orden (tipos_operacion.codigo === ARS-ARS) en lugar del DOM, para que al crear la transacción Ganancia del acuerdo se ejecute siempre el insert en movimientos_cuenta_corriente (movimiento positivo por la comisión) y cierre la CC con el cliente.</v>
+        <v>Al crear la transacción Ganancia del acuerdo se inserta también en movimientos_cuenta_corriente un movimiento con ese concepto y monto (montosCcPorMoneda) para que la CC cliente cierre correctamente. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E138" t="str">
         <v>Desarrollo</v>
@@ -2759,16 +2759,16 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C139" t="str">
-        <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
+        <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
       </c>
       <c r="D139" t="str">
-        <v>Nueva tabla orden_comisiones_generadas (orden_id, tipo ganancia_pandy|comision_intermediario, transaccion_id, transaccion_id_reducida). Helpers asegurarGananciaPandy, revertirGananciaPandy, asegurarComisionIntermediario, revertirComisionIntermediario. Al crear: solo si no existe fila. Al pasar ejecutada→pendiente: se revierte comisión (borrar transacción, caja, CC, fila); ingreso Int→Pandy se revierte cobro+descuento y Compensación; si el cliente deja de completar se revierte Ganancia y se restaura ingreso reducido. Migración sql/migracion_orden_comisiones_generadas.sql. Doc FLUJOS_CC_REGLA.md §8.</v>
+        <v>Todos los inserts en movimientos_cuenta_corriente_intermediario incluyen ...montosCcPorMoneda. Al ejecutar el ingreso Int→Pandy se asegura Comisión del acuerdo (comisiones_orden) si no existe. Script sql/corregir_cc_intermediario_montos_null.sql para datos existentes.</v>
       </c>
       <c r="E139" t="str">
         <v>Desarrollo</v>
@@ -2776,16 +2776,16 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C140" t="str">
-        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
+        <v>CC intermediario: descuento y comisión al entregar cheques</v>
       </c>
       <c r="D140" t="str">
-        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
+        <v>Al ejecutar ingreso Int→Pandy: se inserta movimiento "Descuento sobre cheque" (-monto) para que la CC cierre (nominal cheque vs efectivo recibido). Al ejecutar egreso Pandy→Int: se crea transacción "Comisión del acuerdo" (egreso Pandy→intermediario), movimiento de caja y movimiento en CC intermediario. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E140" t="str">
         <v>Desarrollo</v>
@@ -2793,16 +2793,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C141" t="str">
-        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
+        <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
       </c>
       <c r="D141" t="str">
-        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
+        <v>En saveTransaccion, esOrdenCheque se obtiene desde la orden (tipos_operacion.codigo === ARS-ARS) en lugar del DOM, para que al crear la transacción Ganancia del acuerdo se ejecute siempre el insert en movimientos_cuenta_corriente (movimiento positivo por la comisión) y cierre la CC con el cliente.</v>
       </c>
       <c r="E141" t="str">
         <v>Desarrollo</v>
@@ -2810,16 +2810,16 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C142" t="str">
-        <v>Evitar updates de monto 0 en transacciones</v>
+        <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
       </c>
       <c r="D142" t="str">
-        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
+        <v>Nueva tabla orden_comisiones_generadas (orden_id, tipo ganancia_pandy|comision_intermediario, transaccion_id, transaccion_id_reducida). Helpers asegurarGananciaPandy, revertirGananciaPandy, asegurarComisionIntermediario, revertirComisionIntermediario. Al crear: solo si no existe fila. Al pasar ejecutada→pendiente: se revierte comisión (borrar transacción, caja, CC, fila); ingreso Int→Pandy se revierte cobro+descuento y Compensación; si el cliente deja de completar se revierte Ganancia y se restaura ingreso reducido. Migración sql/migracion_orden_comisiones_generadas.sql. Doc FLUJOS_CC_REGLA.md §8.</v>
       </c>
       <c r="E142" t="str">
         <v>Desarrollo</v>
@@ -2827,16 +2827,16 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C143" t="str">
-        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
+        <v>Reajuste tests E2E y signos CC regla simple</v>
       </c>
       <c r="D143" t="str">
-        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
+        <v>Tests orden-cc.spec.js: timeouts aumentados para vista CC (cc-loading hidden 45s, tbody primera fila 15s) por las consultas extra de transacciones e instrumentación. App: signos CC regla simple corregidos: Compromiso monE (Pandy debe) se guarda con -me; Compromiso Saldado egreso con +monto para que "Pandy debe" se muestre como valor negativo. Ejecutar npx playwright install si falta; app en marcha y .env.test para correr tests.</v>
       </c>
       <c r="E143" t="str">
         <v>Desarrollo</v>
@@ -2844,16 +2844,16 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C144" t="str">
-        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
+        <v>Refresh sin colapsar secciones expandidas</v>
       </c>
       <c r="D144" t="str">
-        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
+        <v>El refresco automático (cada 30 s) y el criterio de no refrescar con modal abierto se extiende: si hay una sección expandida en la vista actual no se ejecuta el refresh para no colapsarla. Órdenes: detalle de transacciones expandido (transaccionesOrdenIdActual). Seguridad: menú o rol expandido. hasExpandedSectionInCurrentView(); refreshCurrentViewData() retorna sin recargar cuando hay expansión.</v>
       </c>
       <c r="E144" t="str">
         <v>Desarrollo</v>
@@ -2861,16 +2861,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C145" t="str">
-        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
+        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
       </c>
       <c r="D145" t="str">
-        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
+        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
       </c>
       <c r="E145" t="str">
         <v>Desarrollo</v>
@@ -2878,16 +2878,16 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C146" t="str">
-        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
+        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
       </c>
       <c r="D146" t="str">
-        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
+        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
       </c>
       <c r="E146" t="str">
         <v>Desarrollo</v>
@@ -2895,16 +2895,16 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C147" t="str">
-        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
+        <v>Evitar updates de monto 0 en transacciones</v>
       </c>
       <c r="D147" t="str">
-        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
+        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
       </c>
       <c r="E147" t="str">
         <v>Desarrollo</v>
@@ -2912,16 +2912,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C148" t="str">
-        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
+        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
       </c>
       <c r="D148" t="str">
-        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
+        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
       </c>
       <c r="E148" t="str">
         <v>Desarrollo</v>
@@ -2929,16 +2929,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C149" t="str">
-        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
+        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
       </c>
       <c r="D149" t="str">
-        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
+        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
       </c>
       <c r="E149" t="str">
         <v>Desarrollo</v>
@@ -2946,16 +2946,16 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C150" t="str">
-        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
+        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
       </c>
       <c r="D150" t="str">
-        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
+        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
       </c>
       <c r="E150" t="str">
         <v>Desarrollo</v>
@@ -2963,16 +2963,16 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C151" t="str">
-        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
+        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
       </c>
       <c r="D151" t="str">
-        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
+        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
       </c>
       <c r="E151" t="str">
         <v>Desarrollo</v>
@@ -2980,16 +2980,16 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C152" t="str">
-        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
+        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
       </c>
       <c r="D152" t="str">
-        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
+        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
       </c>
       <c r="E152" t="str">
         <v>Desarrollo</v>
@@ -2997,16 +2997,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C153" t="str">
-        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
+        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
       </c>
       <c r="D153" t="str">
-        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
+        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
       </c>
       <c r="E153" t="str">
         <v>Desarrollo</v>
@@ -3014,16 +3014,16 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C154" t="str">
-        <v>Reversar a pendiente: solo una vez por transacción</v>
+        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
       </c>
       <c r="D154" t="str">
-        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
+        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
       </c>
       <c r="E154" t="str">
         <v>Desarrollo</v>
@@ -3031,16 +3031,16 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C155" t="str">
-        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
+        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
       </c>
       <c r="D155" t="str">
-        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
+        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
       </c>
       <c r="E155" t="str">
         <v>Desarrollo</v>
@@ -3048,16 +3048,16 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C156" t="str">
-        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
+        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
       </c>
       <c r="D156" t="str">
-        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
+        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
       </c>
       <c r="E156" t="str">
         <v>Desarrollo</v>
@@ -3065,16 +3065,16 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C157" t="str">
-        <v>Número de transacción interno y convención movimientos de caja</v>
+        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
       </c>
       <c r="D157" t="str">
-        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
+        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
       </c>
       <c r="E157" t="str">
         <v>Desarrollo</v>
@@ -3082,16 +3082,16 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C158" t="str">
-        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
+        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
       </c>
       <c r="D158" t="str">
-        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
       </c>
       <c r="E158" t="str">
         <v>Desarrollo</v>
@@ -3099,16 +3099,16 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C159" t="str">
-        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+        <v>Reversar a pendiente: solo una vez por transacción</v>
       </c>
       <c r="D159" t="str">
-        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
       </c>
       <c r="E159" t="str">
         <v>Desarrollo</v>
@@ -3116,16 +3116,16 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C160" t="str">
-        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
       </c>
       <c r="D160" t="str">
-        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
       </c>
       <c r="E160" t="str">
         <v>Desarrollo</v>
@@ -3133,16 +3133,16 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C161" t="str">
-        <v>Tipos de operación: Intermediario Sí/No</v>
+        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
       </c>
       <c r="D161" t="str">
-        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
       </c>
       <c r="E161" t="str">
         <v>Desarrollo</v>
@@ -3150,24 +3150,109 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>21:23</v>
+        <v>12:31</v>
       </c>
       <c r="C162" t="str">
+        <v>Número de transacción interno y convención movimientos de caja</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
+      </c>
+      <c r="E162" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B163" t="str">
+        <v>12:31</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
+      </c>
+      <c r="D163" t="str">
+        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+      </c>
+      <c r="E163" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B164" t="str">
+        <v>12:31</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+      </c>
+      <c r="E164" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B165" t="str">
+        <v>12:31</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+      </c>
+      <c r="D165" t="str">
+        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+      </c>
+      <c r="E165" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B166" t="str">
+        <v>12:31</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Tipos de operación: Intermediario Sí/No</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+      </c>
+      <c r="E166" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B167" t="str">
+        <v>12:31</v>
+      </c>
+      <c r="C167" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
       </c>
-      <c r="D162" t="str">
+      <c r="D167" t="str">
         <v>Función ordenes_insertar_con_proximo_numero en Supabase: asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones. La app llama a la RPC al crear orden nueva (wizard, saveOrden, chat); fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
-      <c r="E162" t="str">
+      <c r="E167" t="str">
         <v>Desarrollo</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E162"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E167"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3652,7 +3737,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3675,7 +3760,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -3686,7 +3771,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -3697,7 +3782,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -3708,7 +3793,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -3719,7 +3804,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -3730,7 +3815,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -3741,7 +3826,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -3752,7 +3837,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -3763,7 +3848,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -3774,7 +3859,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -3785,7 +3870,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -3796,7 +3881,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -3807,7 +3892,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -3818,7 +3903,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -3829,7 +3914,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -3840,7 +3925,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -3851,7 +3936,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -3862,7 +3947,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -3873,7 +3958,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -3884,7 +3969,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -3895,7 +3980,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -3906,7 +3991,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -3917,7 +4002,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -3928,7 +4013,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -3939,7 +4024,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -3950,7 +4035,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -3961,7 +4046,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -3972,7 +4057,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -3983,7 +4068,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
@@ -3994,7 +4079,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
@@ -4005,15 +4090,26 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>14/03/2026</v>
+        <v>15/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>1.31</v>
+      </c>
+      <c r="B33" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.32: switch Activo en tablas y modales, centrado botón y título, truncate y tests E2E
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E170"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>15/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,13 +2864,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C145" t="str">
-        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
+        <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
       </c>
       <c r="D145" t="str">
-        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
+        <v>En órdenes ARS-USD, USD-ARS y USD-USD (sin intermediario) el tipo tiene usa_intermediario=false y el wrap #orden-wrap-intermediario se oculta; el test intentaba selectOption en #orden-intermediario y fallaba por "element is not visible". Se espera a que el wrap esté hidden tras elegir el tipo y solo se selecciona intermediario cuando el wrap es visible.</v>
       </c>
       <c r="E145" t="str">
         <v>Desarrollo</v>
@@ -2881,13 +2881,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C146" t="str">
-        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
+        <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
       </c>
       <c r="D146" t="str">
-        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
+        <v>En los modales de Cliente e Intermediario el campo Activo pasa de checkbox a toggle switch (mismo estilo que en Tipos de operación). Clases form-group-toggle y label-with-toggle; mismo .toggle-switch con .slider. IDs cliente-activo e intermediario-activo sin cambios.</v>
       </c>
       <c r="E146" t="str">
         <v>Desarrollo</v>
@@ -2898,13 +2898,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C147" t="str">
-        <v>Evitar updates de monto 0 en transacciones</v>
+        <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
       </c>
       <c r="D147" t="str">
-        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
+        <v>En la tabla de Clientes y en la de Intermediarios la columna Activo muestra un toggle switch (como en Tipos de operación). Al cambiar el switch se actualiza activo en Supabase sin abrir el modal. Sin SQL: los datos ya están; solo cambia la UI.</v>
       </c>
       <c r="E147" t="str">
         <v>Desarrollo</v>
@@ -2915,13 +2915,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C148" t="str">
-        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
+        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
       </c>
       <c r="D148" t="str">
-        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
+        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
       </c>
       <c r="E148" t="str">
         <v>Desarrollo</v>
@@ -2932,13 +2932,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C149" t="str">
-        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
+        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
       </c>
       <c r="D149" t="str">
-        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
+        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
       </c>
       <c r="E149" t="str">
         <v>Desarrollo</v>
@@ -2949,13 +2949,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C150" t="str">
-        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
+        <v>Evitar updates de monto 0 en transacciones</v>
       </c>
       <c r="D150" t="str">
-        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
+        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
       </c>
       <c r="E150" t="str">
         <v>Desarrollo</v>
@@ -2966,13 +2966,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C151" t="str">
-        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
+        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
       </c>
       <c r="D151" t="str">
-        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
+        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
       </c>
       <c r="E151" t="str">
         <v>Desarrollo</v>
@@ -2983,13 +2983,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C152" t="str">
-        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
+        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
       </c>
       <c r="D152" t="str">
-        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
+        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
       </c>
       <c r="E152" t="str">
         <v>Desarrollo</v>
@@ -3000,13 +3000,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C153" t="str">
-        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
+        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
       </c>
       <c r="D153" t="str">
-        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
+        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
       </c>
       <c r="E153" t="str">
         <v>Desarrollo</v>
@@ -3017,13 +3017,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C154" t="str">
-        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
+        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
       </c>
       <c r="D154" t="str">
-        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
+        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
       </c>
       <c r="E154" t="str">
         <v>Desarrollo</v>
@@ -3034,13 +3034,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C155" t="str">
-        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
+        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
       </c>
       <c r="D155" t="str">
-        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
+        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
       </c>
       <c r="E155" t="str">
         <v>Desarrollo</v>
@@ -3051,13 +3051,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C156" t="str">
-        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
+        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
       </c>
       <c r="D156" t="str">
-        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
+        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
       </c>
       <c r="E156" t="str">
         <v>Desarrollo</v>
@@ -3068,13 +3068,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C157" t="str">
-        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
+        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
       </c>
       <c r="D157" t="str">
-        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
+        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
       </c>
       <c r="E157" t="str">
         <v>Desarrollo</v>
@@ -3085,13 +3085,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C158" t="str">
-        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
+        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
       </c>
       <c r="D158" t="str">
-        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
+        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
       </c>
       <c r="E158" t="str">
         <v>Desarrollo</v>
@@ -3102,13 +3102,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C159" t="str">
-        <v>Reversar a pendiente: solo una vez por transacción</v>
+        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
       </c>
       <c r="D159" t="str">
-        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
+        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
       </c>
       <c r="E159" t="str">
         <v>Desarrollo</v>
@@ -3119,13 +3119,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C160" t="str">
-        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
+        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
       </c>
       <c r="D160" t="str">
-        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
+        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
       </c>
       <c r="E160" t="str">
         <v>Desarrollo</v>
@@ -3136,13 +3136,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C161" t="str">
-        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
+        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
       </c>
       <c r="D161" t="str">
-        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
+        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
       </c>
       <c r="E161" t="str">
         <v>Desarrollo</v>
@@ -3153,13 +3153,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C162" t="str">
-        <v>Número de transacción interno y convención movimientos de caja</v>
+        <v>Reversar a pendiente: solo una vez por transacción</v>
       </c>
       <c r="D162" t="str">
-        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
+        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
       </c>
       <c r="E162" t="str">
         <v>Desarrollo</v>
@@ -3170,13 +3170,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C163" t="str">
-        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
+        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
       </c>
       <c r="D163" t="str">
-        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
       </c>
       <c r="E163" t="str">
         <v>Desarrollo</v>
@@ -3187,13 +3187,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C164" t="str">
-        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
       </c>
       <c r="D164" t="str">
-        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
       </c>
       <c r="E164" t="str">
         <v>Desarrollo</v>
@@ -3204,13 +3204,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C165" t="str">
-        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+        <v>Número de transacción interno y convención movimientos de caja</v>
       </c>
       <c r="D165" t="str">
-        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
       </c>
       <c r="E165" t="str">
         <v>Desarrollo</v>
@@ -3221,13 +3221,13 @@
         <v>15/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C166" t="str">
-        <v>Tipos de operación: Intermediario Sí/No</v>
+        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
       </c>
       <c r="D166" t="str">
-        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
       </c>
       <c r="E166" t="str">
         <v>Desarrollo</v>
@@ -3238,21 +3238,72 @@
         <v>15/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>12:31</v>
+        <v>12:47</v>
       </c>
       <c r="C167" t="str">
+        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+      </c>
+      <c r="D167" t="str">
+        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+      </c>
+      <c r="E167" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B168" t="str">
+        <v>12:47</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+      </c>
+      <c r="D168" t="str">
+        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+      </c>
+      <c r="E168" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B169" t="str">
+        <v>12:47</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Tipos de operación: Intermediario Sí/No</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+      </c>
+      <c r="E169" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="B170" t="str">
+        <v>12:47</v>
+      </c>
+      <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
       </c>
-      <c r="D167" t="str">
+      <c r="D170" t="str">
         <v>Función ordenes_insertar_con_proximo_numero en Supabase: asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones. La app llama a la RPC al crear orden nueva (wizard, saveOrden, chat); fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
-      <c r="E167" t="str">
+      <c r="E170" t="str">
         <v>Desarrollo</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E167"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E170"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3737,7 +3788,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4107,9 +4158,20 @@
         <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>1.32</v>
+      </c>
+      <c r="B34" t="str">
+        <v>15/03/2026</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Switch Activo en tablas Clientes e Intermediarios; modales Cliente/Intermediario con toggle; centrado de botón y título en todas las pantallas con switch. Script truncar: orden correcto y orden_comisiones_generadas opcional. Tests E2E: intermediario solo si visible (tipos sin intermediario).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.33: CC ARS-ARS con intermediario momento cero; mensajes E2E y guía TEST_BASE_URL
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E170"/>
+  <dimension ref="A1:E171"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2215,10 +2215,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2266,10 +2266,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2283,10 +2283,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2402,10 +2402,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2419,10 +2419,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2436,10 +2436,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2470,10 +2470,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2487,10 +2487,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2521,10 +2521,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2538,10 +2538,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2572,10 +2572,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2589,10 +2589,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2606,10 +2606,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2623,10 +2623,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2640,10 +2640,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2657,10 +2657,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2674,10 +2674,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2691,10 +2691,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2708,10 +2708,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2725,10 +2725,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2742,10 +2742,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2759,10 +2759,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2776,10 +2776,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2793,10 +2793,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2810,10 +2810,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2827,10 +2827,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2844,10 +2844,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2861,10 +2861,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2878,10 +2878,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2895,10 +2895,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2912,10 +2912,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2946,10 +2946,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2963,10 +2963,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2980,10 +2980,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -2997,10 +2997,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3014,10 +3014,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3031,10 +3031,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3048,10 +3048,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3065,10 +3065,10 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3082,10 +3082,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3099,10 +3099,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3116,10 +3116,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3133,10 +3133,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3150,10 +3150,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3167,10 +3167,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3184,10 +3184,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3201,10 +3201,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3218,10 +3218,10 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3235,10 +3235,10 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3252,10 +3252,10 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3269,10 +3269,10 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3286,10 +3286,10 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>12:47</v>
+        <v>14:58</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3301,9 +3301,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B171" t="str">
+        <v>14:58</v>
+      </c>
+      <c r="C171" t="str">
+        <v>v1.33 Despliegue</v>
+      </c>
+      <c r="D171" t="str">
+        <v>CC ARS-ARS con intermediario: momento cero cliente (Compromiso -mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía TEST_BASE_URL cuando Vite usa otro puerto.</v>
+      </c>
+      <c r="E171" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E170"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E171"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3788,7 +3805,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -3811,7 +3828,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -3822,7 +3839,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -3833,7 +3850,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -3844,7 +3861,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -3855,7 +3872,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -3866,7 +3883,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -3877,7 +3894,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -3888,7 +3905,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -3899,7 +3916,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -3910,7 +3927,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -3921,7 +3938,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -3932,7 +3949,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -3943,7 +3960,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -3954,7 +3971,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -3965,7 +3982,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -3976,7 +3993,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -3987,7 +4004,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -3998,7 +4015,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -4009,7 +4026,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -4020,7 +4037,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -4031,7 +4048,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -4042,7 +4059,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -4053,7 +4070,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -4064,7 +4081,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -4075,7 +4092,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -4086,7 +4103,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -4097,7 +4114,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -4108,7 +4125,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -4119,7 +4136,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
@@ -4130,7 +4147,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
@@ -4141,7 +4158,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
@@ -4152,7 +4169,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
@@ -4163,15 +4180,26 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>15/03/2026</v>
+        <v>16/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Switch Activo en tablas Clientes e Intermediarios; modales Cliente/Intermediario con toggle; centrado de botón y título en todas las pantallas con switch. Script truncar: orden correcto y orden_comisiones_generadas opcional. Tests E2E: intermediario solo si visible (tipos sin intermediario).</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>1.33</v>
+      </c>
+      <c r="B35" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C35" t="str">
+        <v>CC ARS-ARS con intermediario: momento cero cliente (-mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía testing con TEST_BASE_URL cuando Vite usa otro puerto.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.34: CC regla simple ambas pendientes = saldo 0
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E172"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>14:58</v>
+        <v>15:05</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3318,9 +3318,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B172" t="str">
+        <v>15:05</v>
+      </c>
+      <c r="C172" t="str">
+        <v>v1.34 Despliegue</v>
+      </c>
+      <c r="D172" t="str">
+        <v>CC regla simple: compromisos solo si al menos una transacción ejecutada; ambas pendientes → saldo 0.</v>
+      </c>
+      <c r="E172" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E171"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E172"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3805,7 +3822,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4197,9 +4214,20 @@
         <v>CC ARS-ARS con intermediario: momento cero cliente (-mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía testing con TEST_BASE_URL cuando Vite usa otro puerto.</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>1.34</v>
+      </c>
+      <c r="B36" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C36" t="str">
+        <v>CC regla simple (USD-USD, 2 transacciones): compromisos solo cuando al menos una transacción está ejecutada; si ambas pendientes, saldo 0 (no figura deuda).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.35: regla estilos botones LyP (icono a la izquierda, mismo estilo con/sin leyenda)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E172"/>
+  <dimension ref="A1:E175"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3323,7 +3323,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>15:05</v>
+        <v>16:36</v>
       </c>
       <c r="C172" t="str">
         <v>v1.34 Despliegue</v>
@@ -3335,16 +3335,67 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B173" t="str">
+        <v>16:36</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
+      </c>
+      <c r="D173" t="str">
+        <v>utils.js en raíz: formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda; main.js importa desde ./utils.js. RPC sync_cc_caja_orden en Supabase: front construye rows y llama RPC para delete+insert atómico; fallback a delete+insert en cliente si RPC no existe. sql/rpc_sync_cc_caja_orden.sql. Doc docs/FUNCIONES_CRITICAS_SUPABASE_VS_FRONT.md actualizado.</v>
+      </c>
+      <c r="E173" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B174" t="str">
+        <v>16:36</v>
+      </c>
+      <c r="C174" t="str">
+        <v>RPC transacciones_cambiar_estado</v>
+      </c>
+      <c r="D174" t="str">
+        <v>Función PostgreSQL transacciones_cambiar_estado(p_transaccion_id, p_estado, p_fecha_ejecucion, p_usuario_id, p_revertida_una_vez). El front llama la RPC al cambiar pendiente↔ejecutada; si la RPC no existe usa UPDATE directo. sql/rpc_transacciones_cambiar_estado.sql. Sin Edge Functions: solo RPC (funciones en la DB).</v>
+      </c>
+      <c r="E174" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B175" t="str">
+        <v>16:36</v>
+      </c>
+      <c r="C175" t="str">
+        <v>v1.35 Despliegue</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Regla de estilos de botones LyP: mismo estilo en toda la app; con leyenda icono a la izquierda; solo icono mismo estilo. Regla .cursor/rules/estilos-botones.mdc en Pandi y replicada en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
+      </c>
+      <c r="E175" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E175"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3750,9 +3801,17 @@
         <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Utils y RPC sync CC/caja</v>
+      </c>
+      <c r="B51" t="str">
+        <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B51"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3822,7 +3881,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4225,9 +4284,20 @@
         <v>CC regla simple (USD-USD, 2 transacciones): compromisos solo cuando al menos una transacción está ejecutada; si ambas pendientes, saldo 0 (no figura deuda).</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>1.35</v>
+      </c>
+      <c r="B37" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Regla de estilos de botones LyP: mismo estilo (border-radius 8px, min-height); con leyenda = icono a la izquierda; solo icono mismo estilo; botón Excel verde. Regla estilos-botones.mdc en Pandi y en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.36: reglas bitácora, RPC y tests no pueden omitirse; CC Originante y leyendas concepto
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E178"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3323,7 +3323,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C172" t="str">
         <v>v1.34 Despliegue</v>
@@ -3340,7 +3340,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C173" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3357,7 +3357,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C174" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3374,7 +3374,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>16:36</v>
+        <v>17:06</v>
       </c>
       <c r="C175" t="str">
         <v>v1.35 Despliegue</v>
@@ -3386,9 +3386,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B176" t="str">
+        <v>17:06</v>
+      </c>
+      <c r="C176" t="str">
+        <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Vista Detalle de movimientos: se quitó el filtro Tipo "Todos"; solo Cliente e Intermediario. Columna Originante siempre visible: encabezado "Cliente" o "Intermediario" según el filtro y en cada fila el nombre del originante del movimiento. Export Excel incluye esa columna con el mismo criterio.</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B177" t="str">
+        <v>17:06</v>
+      </c>
+      <c r="C177" t="str">
+        <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Originante en cada movimiento = Pagador de la transacción (nombre resuelto desde cliente/intermediario/Pandy). Leyendas concepto unificadas: Pago Realizado - Orden x y Trans x, Cobro Realizado - Orden x y Trans x, Compromiso de Pago - Orden x y Trans x, Compromiso a Cobrar - Orden x y Trans x. Vista Detalle: columnas Orden y Trans. (sin "Nro"); columnas Cliente/Intermediario y Originante. Helper conceptoCcLeyenda; sync e insertar momento cero usan nuevas leyendas.</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B178" t="str">
+        <v>17:06</v>
+      </c>
+      <c r="C178" t="str">
+        <v>v1.36 Despliegue</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. bitacora-tareas.mdc y reglas-pandi.mdc actualizados con revisión RPC y adaptación de tests obligatorias.</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E175"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E178"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3881,7 +3932,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4295,9 +4346,20 @@
         <v>Regla de estilos de botones LyP: mismo estilo (border-radius 8px, min-height); con leyenda = icono a la izquierda; solo icono mismo estilo; botón Excel verde. Regla estilos-botones.mdc en Pandi y en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>1.36</v>
+      </c>
+      <c r="B38" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. Al completar tareas hay que actualizar bitácora, revisar RPC en sql/ si aplica y adaptar tests si afectan. bitacora-tareas.mdc y reglas-pandi.mdc.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.37: modales backdrop real click, sesión mousemove, CC tipo op. sticky y export
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E185"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3323,7 +3323,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C172" t="str">
         <v>v1.34 Despliegue</v>
@@ -3340,7 +3340,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C173" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3357,7 +3357,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C174" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3374,7 +3374,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C175" t="str">
         <v>v1.35 Despliegue</v>
@@ -3391,7 +3391,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C176" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3408,7 +3408,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C177" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3425,7 +3425,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>17:06</v>
+        <v>18:07</v>
       </c>
       <c r="C178" t="str">
         <v>v1.36 Despliegue</v>
@@ -3437,16 +3437,135 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B179" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C179" t="str">
+        <v>CC: unificación de conceptos y transaccion_numero</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Conceptos CC intermediario y derivados unificados con conceptoCcLeyenda: Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo (tipo comision_acuerdo), siempre con " - Orden x y Trans x". transaccion_numero en todos los rows/inserts de CC (cliente e intermediario). asegurarComisionIntermediario con parámetro ordenNumero; filtros de reversa actualizados a "Compromiso a Cobrar". Doc REVISION_CC_INTERMEDIARIO_CONCEPTOS_Y_NRO_TRANS.md §4.</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B180" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C180" t="str">
+        <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Eliminado duplicado: una sola fila "Compromiso a Cobrar" por transacción (cuantasQueremos = 1). Doc FLUJOS_CC_REGLA.md: sección Revisión de impacto (RCA) y Objetivo actuar por transacción (no borrar/repoblar toda la orden). Regla en reglas-pandi.mdc: revisión de impacto RCA y regla por transacción (movimientos ligados a transacción; no depender de sync completo).</v>
+      </c>
+      <c r="E180" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B181" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C181" t="str">
+        <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
+      </c>
+      <c r="D181" t="str">
+        <v>loadCuentaCorriente: solo lee mov_cc y mov_cc_int (sin sync previo). guardarSoloMontoTransaccion y hacerCierre: sin llamar a sincronizarCcYCajaDesdeOrden. autoCompletarInstrumentacionChequeConIntermediario: inserta momento cero (insertarMovimientosCcMomentoCero e Intermediario) en lugar de sync. cambiarEstadoTransaccion: actualizarEstadoSinSync (solo actualizarEstadoOrden). saveTransaccion revert: revertirCcYCajaPorTransaccion (borrar/actualizar solo movimientos de esa transacción) en lugar de sync. Base siempre bien relacionada; eficiente con alto volumen.</v>
+      </c>
+      <c r="E181" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B182" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C182" t="str">
+        <v>CC detalle movimientos: columna Tipo de operación</v>
+      </c>
+      <c r="D182" t="str">
+        <v>En el modal Detalle de movimientos (cliente/intermediario) se agrega la columna Tipo op. con el código del tipo de operación de la orden (tipos_operacion.codigo). fetchMovimientosCcPorEntidad incluye tipo_operacion_id y tipos_operacion(codigo) en el select de órdenes; se enriquece cada movimiento con tipo_operacion; ordenamiento por esa columna. Trazabilidad visual completa (Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado).</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B183" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C183" t="str">
+        <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Tipo de operación visible en vista Detalle (página), modal detalle y export. Orden de columnas: Fecha, Tipo op., Orden, Trans., Concepto, … Columnas Fecha y Tipo op. ancladas en scroll horizontal (sticky left) en modal y vista detalle. loadCuentaCorriente carga tipos_operacion(codigo) en órdenes; buildCcResumenRows agrega tipo_operacion a detalleList. Export Excel incluye columna Tipo op. tras Fecha.</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B184" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Modales: no cerrar al elegir opción de menú/select</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Al abrir un desplegable (select o menú) y mover el mouse para elegir, el click a veces se reportaba en el backdrop y cerraba el modal. Helper setupBackdropCloseOnlyOnRealClick: solo cerrar si tanto mousedown como click fueron sobre el backdrop. Aplicado a todos los modales (órdenes, transacciones, CC, cliente, intermediario, tipo op., confirm, help, etc.).</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B185" t="str">
+        <v>18:07</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
+      </c>
+      <c r="D185" t="str">
+        <v>El cierre por inactividad se disparaba al solo mover el mouse o el trackpad (sin clic) porque mousemove no actualizaba lastActivityTime. Se agregó mousemove a los eventos que llaman a updateSessionActivity (throttle 30 s); así mover el cursor mantiene la sesión viva y no se cierra la app al abrir un menú.</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E178"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E185"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -3553,7 +3672,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de toda la tabla. Al editar transacción se respetan filas momento cero. Tabla detalle: Fecha, Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
+        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de toda la tabla. Al editar transacción se respetan filas momento cero. Tabla detalle: Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
       </c>
     </row>
     <row r="14">
@@ -3860,9 +3979,17 @@
         <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Conceptos CC unificados y número de transacción</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Todos los movimientos CC (cliente e intermediario) usan leyendas unificadas (Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo) con sufijo " - Orden x y Trans x". transaccion_numero se guarda en todos los inserts/rows para que la columna Trans. del detalle nunca quede en blanco cuando hay transacción de referencia. Incluye movimientos derivados (pago/cobro de comisiones).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B52"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3932,7 +4059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4357,9 +4484,20 @@
         <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. Al completar tareas hay que actualizar bitácora, revisar RPC en sql/ si aplica y adaptar tests si afectan. bitacora-tareas.mdc y reglas-pandi.mdc.</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>1.37</v>
+      </c>
+      <c r="B39" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Modales: no cerrar al elegir en select (mousedown+click en backdrop). Sesión: mousemove cuenta como actividad para no cerrar por inactividad al mover mouse/trackpad. CC: Tipo op. después de Fecha, sticky y export Excel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.38: XLSX desde CDN para producción Vercel (fix module specifier)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E186"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3323,7 +3323,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C172" t="str">
         <v>v1.34 Despliegue</v>
@@ -3340,7 +3340,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C173" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3357,7 +3357,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C174" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3374,7 +3374,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C175" t="str">
         <v>v1.35 Despliegue</v>
@@ -3391,7 +3391,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C176" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3408,7 +3408,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C177" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3425,7 +3425,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C178" t="str">
         <v>v1.36 Despliegue</v>
@@ -3442,7 +3442,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C179" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3459,7 +3459,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C180" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3476,7 +3476,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C181" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3493,7 +3493,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C182" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3510,7 +3510,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C183" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3527,7 +3527,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C184" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3544,7 +3544,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>18:07</v>
+        <v>18:24</v>
       </c>
       <c r="C185" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3556,9 +3556,26 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B186" t="str">
+        <v>18:24</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Despliegue v1.38</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Producción Vercel: XLSX desde CDN en index.html y main.js usa window.XLSX para que funcione sin bundler (fix "Failed to resolve module specifier xlsx").</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E186"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4059,7 +4076,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4495,9 +4512,20 @@
         <v>Modales: no cerrar al elegir en select (mousedown+click en backdrop). Sesión: mousemove cuenta como actividad para no cerrar por inactividad al mover mouse/trackpad. CC: Tipo op. después de Fecha, sticky y export Excel.</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>1.38</v>
+      </c>
+      <c r="B40" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Producción Vercel: XLSX cargado desde CDN (script en index.html); main.js usa window.XLSX para evitar error "Failed to resolve module specifier xlsx" sin bundler.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.39: CC regla infalible (me/mr, ingreso pendiente muestra deuda cliente)
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E186"/>
+  <dimension ref="A1:E195"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2099,7 +2099,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C100" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2116,7 +2116,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C101" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2133,7 +2133,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C102" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2150,7 +2150,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C103" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2167,7 +2167,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C104" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2184,7 +2184,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C105" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2201,7 +2201,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C106" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2218,7 +2218,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C107" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2235,7 +2235,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C108" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2252,7 +2252,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C109" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2269,7 +2269,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C110" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2286,7 +2286,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C111" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2303,7 +2303,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C112" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2320,7 +2320,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C113" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2337,7 +2337,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C114" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2354,7 +2354,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C115" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2371,7 +2371,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C116" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2388,7 +2388,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C117" t="str">
         <v>Modal orden más ancho</v>
@@ -2405,7 +2405,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C118" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2422,7 +2422,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C119" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2439,7 +2439,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C120" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2456,7 +2456,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C121" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2473,7 +2473,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C122" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2490,7 +2490,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C123" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2507,7 +2507,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C124" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2524,7 +2524,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C125" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2541,7 +2541,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C126" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2558,7 +2558,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C127" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2575,7 +2575,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C128" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2592,7 +2592,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C129" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2609,7 +2609,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C130" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2626,7 +2626,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C131" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2643,7 +2643,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C132" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2660,7 +2660,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2677,7 +2677,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C134" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2694,7 +2694,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2711,7 +2711,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C136" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2728,7 +2728,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2745,7 +2745,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2762,7 +2762,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2779,7 +2779,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C140" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2796,7 +2796,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C141" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2813,7 +2813,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C142" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2830,7 +2830,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C143" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2847,7 +2847,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C144" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2864,7 +2864,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C145" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2881,7 +2881,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C146" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2898,7 +2898,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C147" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2915,7 +2915,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C148" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2932,7 +2932,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C149" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2949,7 +2949,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C150" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2966,7 +2966,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C151" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -2983,7 +2983,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C152" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3000,7 +3000,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C153" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3017,7 +3017,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3034,7 +3034,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C155" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3051,7 +3051,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C156" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3068,7 +3068,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3085,7 +3085,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3102,7 +3102,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C159" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3119,7 +3119,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C160" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3136,7 +3136,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C161" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3153,7 +3153,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C162" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3170,7 +3170,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C163" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3187,7 +3187,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C164" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3204,7 +3204,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C165" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3221,7 +3221,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C166" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3238,7 +3238,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C167" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3255,7 +3255,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C168" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3272,7 +3272,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C169" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3289,7 +3289,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C170" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3306,7 +3306,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C171" t="str">
         <v>v1.33 Despliegue</v>
@@ -3323,7 +3323,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C172" t="str">
         <v>v1.34 Despliegue</v>
@@ -3340,7 +3340,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C173" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3357,7 +3357,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C174" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3374,7 +3374,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C175" t="str">
         <v>v1.35 Despliegue</v>
@@ -3391,7 +3391,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C176" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3408,7 +3408,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C177" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3425,7 +3425,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C178" t="str">
         <v>v1.36 Despliegue</v>
@@ -3442,7 +3442,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C179" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3459,7 +3459,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C180" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3476,7 +3476,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C181" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3493,7 +3493,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C182" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3510,7 +3510,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C183" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3527,7 +3527,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C184" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3544,7 +3544,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C185" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3561,7 +3561,7 @@
         <v>16/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>18:24</v>
+        <v>22:57</v>
       </c>
       <c r="C186" t="str">
         <v>Despliegue v1.38</v>
@@ -3573,9 +3573,162 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B187" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Tras cambiar transacción a "ejecutada" en el wizard, el test cerraba el modal y navegaba a Cuenta corriente antes de que el backend terminara; la transacción no se persistía y los asserts fallaban. Se agregó esperarActualizacionEstadoOrden(page): espera a que #orden-inst-actualizando-msg desaparezca (hasta 35 s) en los cuatro flujos (ARS-ARS, ARS-USD, USD-ARS, USD-USD).</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B188" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C188" t="str">
+        <v>CC intermediario: estado pendiente en momento cero</v>
+      </c>
+      <c r="D188" t="str">
+        <v>En ARS-ARS con intermediario, insertarMovimientosCcMomentoCeroIntermediario no guardaba estado en las filas Debe/Compensación; si la tabla tiene estado NULL, el UPDATE en cambiarEstadoTransaccion (.eq(estado, pendiente)) no coincidía y la fila no se cerraba, dejando la CC del intermediario en cero tras ejecutar la 3.ª transacción. Se agrega estado: "pendiente" en ambas filas al insertar.</v>
+      </c>
+      <c r="E188" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B189" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Regla simple e infalible CC y caja</v>
+      </c>
+      <c r="D189" t="str">
+        <v>Docs REGLA_CC_SIMPLE_INFALIBLE.md y actualización FLUJOS_CC_REGLA.md. Solo transacciones ejecutadas generan movimientos; signo por pagador/cobrador (pagador entidad → +monto, cobrador entidad → -monto); caja Pandy cobra + / paga -. Sin momento cero: no se insertan movimientos al crear la instrumentación; sync (sincronizarCcYCajaDesdeOrden) construye rows solo desde transacciones ejecutadas. cambiarEstadoTransaccion: tras RPC, reversas de ganancia/comisión si aplica y siempre sincronizarCcYCajaDesdeOrden(ordenId). App, tests y RPC alineados a la misma regla.</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B190" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C190" t="str">
+        <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
+      </c>
+      <c r="D190" t="str">
+        <v>En órdenes ARS-USD/USD-ARS el saldo debe cerrar en 0 tras ejecutar ambas transacciones. RPC sync_cc_caja_orden: COALESCE((r-&gt;&gt;'monto_usd')::numeric, 0) (y monto_ars, monto_eur) en inserts CC cliente e intermediario para no guardar NULL. Front: en sincronizarCcYCajaDesdeOrden los rows CC cliente llevan monto_usd, monto_ars, monto_eur explícitos con numCc(montos.*) en lugar de ...montos. sql/rpc_sync_cc_caja_orden.sql y main.js.</v>
+      </c>
+      <c r="E190" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B191" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C191" t="str">
+        <v>CC: un movimiento = una moneda (la de la transacción)</v>
+      </c>
+      <c r="D191" t="str">
+        <v>No puede haber valor en más de una moneda por movimiento. Sync: se usa montosCcPorMoneda(mon, monto) en lugar de montosCcPorOrden en todos los flujos (sincronizarCcYCajaDesdeOrden, insertarMovimientosCcParaTransaccion y fallbacks). Vista Detalle de movimientos: se muestra solo la columna de la moneda del movimiento (m.moneda); las demás "–". Aplica a vista principal y modal detalle.</v>
+      </c>
+      <c r="E191" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B192" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C192" t="str">
+        <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Por misma orden no puede haber resumen de CC con saldo en más de una moneda. Para órdenes en dos monedas (ARS-USD, USD-ARS) sin intermediario: cuando ingreso Cliente→Pandy y egreso Pandy→Cliente están ejecutados, se añaden dos movimientos de cierre en sync (concepto "Cierre orden N"): -monto recibido en monR y +monto entregado en monE. Así el saldo del cliente para esa orden queda 0 en cada moneda. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B193" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Regla CC: 4 premisas clave documentadas</v>
+      </c>
+      <c r="D193" t="str">
+        <v>Doc REGLA_CC_SIMPLE_INFALIBLE.md reordenado con las 4 premisas como base: (1) Siempre pagador y cobrador; (2) Siempre una única moneda; (3) Estado Pendiente o Ejecutada, solo Ejecutada genera movimientos; (4) Comisión implícita se administra según estado. Secciones del doc referencian cada premisa.</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B194" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C194" t="str">
+        <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Cliente pagó → movimiento -monto (saldo negativo = Pandy debe entregar). Pandy pagó al cliente → +monto. Así una sola transacción ejecutada (cliente pagó 3700) muestra -3700 (Pandy debe), no +3700. Ajustados sync, cierre dos monedas, ganancia Pandy e insertarMovimientosCcParaTransaccion. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="B195" t="str">
+        <v>22:57</v>
+      </c>
+      <c r="C195" t="str">
+        <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Cuando solo el egreso está ejecutada (Pandy pagó me) y el ingreso Cliente→Pandy está pendiente, el resumen debe mostrar lo que el cliente debe (mr), no me. En sync: egreso misma moneda con ingreso pendiente → movimiento +mr en CC cliente. Así ALFIE con ingreso 4933 pendiente y egreso 4849,14 ejecutada muestra "cliente debe 4933". Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E186"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E195"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4076,7 +4229,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4523,9 +4676,20 @@
         <v>Producción Vercel: XLSX cargado desde CDN (script en index.html); main.js usa window.XLSX para evitar error "Failed to resolve module specifier xlsx" sin bundler.</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>1.39</v>
+      </c>
+      <c r="B41" t="str">
+        <v>16/03/2026</v>
+      </c>
+      <c r="C41" t="str">
+        <v>CC regla infalible: ingreso misma moneda aporta -me (Pandy debe su transacción); egreso con ingreso pendiente aporta +mr (resumen muestra deuda del cliente). Sin movimiento extra ganancia Pandy en CC. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.40: validación egreso cheques y color CC a favor/en contra de Pandy
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E199"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2079,16 +2079,16 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C99" t="str">
-        <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
+        <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
       </c>
       <c r="D99" t="str">
-        <v>Función insertarMovimientosCcParaTransaccion actualizada con la misma regla que cambiarEstadoTransaccion/saveTransaccion: Int→Pandy cierra Compensación con montos en 0 e inserta solo Cobro; Egreso Pandy→Int cierra Debe con montos en 0, inserta Deuda -montoEfectivoInt y Comisión del acuerdo +monto, más asegurarComisionIntermediario. Usa orden.tasa_descuento_intermediario y orden.moneda_recibida para monto efectivo.</v>
+        <v>Pendientes Pandy→Intermediario: carga desde instrumentación primero, luego órdenes por orden_id (evita RLS). Filas para intermediarios que solo tienen pendiente (sin movimientos en CC), igual que cliente. Cliente: misma estrategia (instrumentación primero) para simetría. Regla de oro: todo cambio en CC intermediario se replica en cliente y viceversa.</v>
       </c>
       <c r="E99" t="str">
         <v>Desarrollo</v>
@@ -2096,16 +2096,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C100" t="str">
-        <v>CC intermediario y truncate: número de orden y setval</v>
+        <v>CC: regla unificada y una sola carga de pendientes</v>
       </c>
       <c r="D100" t="str">
-        <v>Conceptos CC intermediario (Debe/Compensación momento cero) usan siempre el número interno de orden: resolverOrdenLabel en insertarMovimientosCcMomentoCeroIntermediario (orden.numero o select a ordenes); fallback "nro orden ?" si no hay numero. Script sql/truncar_ordenes_transacciones.sql: tras TRUNCATE ordenes se ejecuta setval de la secuencia numero (ordenes_numero_seq o pg_get_serial_sequence) para que la próxima orden sea nº 1.</v>
+        <v>contribucionPendienteCcUnificada(t, orden, transaccionesOrden): una sola función con estado, pagador, cobrador, moneda, monto; devuelve contribución para cliente e intermediario. Una sola promesa promPendientesCcGlobal: instrumentación → órdenes → transacciones .eq(estado,pendiente), filtro en JS por instrumentacion_id; aplica regla unificada para ambos mapas. Carga de transacciones sin .in(instrumentacion_id) para no depender de órdenes con movimientos; CC intermediario debe verse siempre.</v>
       </c>
       <c r="E100" t="str">
         <v>Desarrollo</v>
@@ -2113,16 +2113,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C101" t="str">
-        <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
+        <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
       </c>
       <c r="D101" t="str">
-        <v>Cancelación de deuda en órdenes misma moneda (monR === monE): usar solo el monto de la transacción (ej. -48.750 cuando Pandy paga al cliente), no la proporción mr/me que daba -50.000 o -51.282. montosCancelacionDesdeOrden, montosCancelacion (cambiarEstadoTransaccion), montosCancelacionItem (guardarSoloMontoTransaccion) y bloques split egreso/ingreso con monR === monE. En ARS-ARS con intermediario: no insertar movimiento CC "Ganancia del acuerdo" ni actualizar la fila del ingreso reducido (asegurarGananciaPandy y revertirGananciaPandy); solo un movimiento positivo por el pago al cliente.</v>
+        <v>Función insertarMovimientosCcParaTransaccion actualizada con la misma regla que cambiarEstadoTransaccion/saveTransaccion: Int→Pandy cierra Compensación con montos en 0 e inserta solo Cobro; Egreso Pandy→Int cierra Debe con montos en 0, inserta Deuda -montoEfectivoInt y Comisión del acuerdo +monto, más asegurarComisionIntermediario. Usa orden.tasa_descuento_intermediario y orden.moneda_recibida para monto efectivo.</v>
       </c>
       <c r="E101" t="str">
         <v>Desarrollo</v>
@@ -2130,16 +2130,16 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C102" t="str">
-        <v>CC cliente: comisión como resultado del split y saldo 0</v>
+        <v>CC intermediario y truncate: número de orden y setval</v>
       </c>
       <c r="D102" t="str">
-        <v>La comisión Pandy (1.250) debe ser resultado del split del ingreso 50.000 en dos transacciones (48.750 + 1.250). En misma moneda: no se inserta fila CC "Ganancia"; sí se actualiza la fila Cancelación del ingreso restando la comisión (50.000 → 48.750) en monto_usd/ars/eur según monR. Así la CC muestra +48.750 (ingreso) y -48.750 (egreso) = 0. Revertir: sumar de nuevo la comisión a la fila del ingreso y restaurar monto transacción. asegurarGananciaPandy y revertirGananciaPandy actualizados (update por moneda).</v>
+        <v>Conceptos CC intermediario (Debe/Compensación momento cero) usan siempre el número interno de orden: resolverOrdenLabel en insertarMovimientosCcMomentoCeroIntermediario (orden.numero o select a ordenes); fallback "nro orden ?" si no hay numero. Script sql/truncar_ordenes_transacciones.sql: tras TRUNCATE ordenes se ejecuta setval de la secuencia numero (ordenes_numero_seq o pg_get_serial_sequence) para que la próxima orden sea nº 1.</v>
       </c>
       <c r="E102" t="str">
         <v>Desarrollo</v>
@@ -2147,16 +2147,16 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C103" t="str">
-        <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
+        <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
       </c>
       <c r="D103" t="str">
-        <v>Regla sagrada: no tocar los originales (Debe y Compensación). En guardarSoloMontoTransaccion cuando newRestoMonto &lt; 1e-6 solo se actualiza estado a cerrado (no monto_usd/ars/eur a 0). En misma moneda (ARS-ARS): al hacer split se actualiza la Cancelación del ingreso 50.000→48.750; se insertan dos movimientos CC para que la comisión figure y la cuenta cierre en 0: Ganancia del acuerdo +1.250 y Comisión Pandy -1.250. Revertir borra ambos por transaccion_id.</v>
+        <v>Cancelación de deuda en órdenes misma moneda (monR === monE): usar solo el monto de la transacción (ej. -48.750 cuando Pandy paga al cliente), no la proporción mr/me que daba -50.000 o -51.282. montosCancelacionDesdeOrden, montosCancelacion (cambiarEstadoTransaccion), montosCancelacionItem (guardarSoloMontoTransaccion) y bloques split egreso/ingreso con monR === monE. En ARS-ARS con intermediario: no insertar movimiento CC "Ganancia del acuerdo" ni actualizar la fila del ingreso reducido (asegurarGananciaPandy y revertirGananciaPandy); solo un movimiento positivo por el pago al cliente.</v>
       </c>
       <c r="E103" t="str">
         <v>Desarrollo</v>
@@ -2164,16 +2164,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C104" t="str">
-        <v>Sincronización CC y caja desde orden + transacciones</v>
+        <v>CC cliente: comisión como resultado del split y saldo 0</v>
       </c>
       <c r="D104" t="str">
-        <v>Modelo: orden e instrumentación (transacciones) son la fuente de verdad; CC y caja se derivan por conciliación. Función sincronizarCcYCajaDesdeOrden(ordenId): borra movimientos CC (cliente e intermediario) y caja de la orden, recalcula desde todas las transacciones (cobro/deuda, Ganancia del acuerdo, comisión intermediario) e inserta. Invocada al cambiar estado de transacción (cambiarEstadoTransaccion), al guardar monto (guardarSoloMontoTransaccion), al guardar desde modal transacción (saveTransaccion → hacerCierre) y al auto-completar ARS-ARS con intermediario (en lugar de momento cero 2 filas).</v>
+        <v>La comisión Pandy (1.250) debe ser resultado del split del ingreso 50.000 en dos transacciones (48.750 + 1.250). En misma moneda: no se inserta fila CC "Ganancia"; sí se actualiza la fila Cancelación del ingreso restando la comisión (50.000 → 48.750) en monto_usd/ars/eur según monR. Así la CC muestra +48.750 (ingreso) y -48.750 (egreso) = 0. Revertir: sumar de nuevo la comisión a la fila del ingreso y restaurar monto transacción. asegurarGananciaPandy y revertirGananciaPandy actualizados (update por moneda).</v>
       </c>
       <c r="E104" t="str">
         <v>Desarrollo</v>
@@ -2181,16 +2181,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C105" t="str">
-        <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
+        <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
       </c>
       <c r="D105" t="str">
-        <v>Al hacer split de egreso (ej. 1000→500 ejecutado, 500 pendiente) la diferencia está en monE (USD). La fila Debe (monR) debe llevar el equivalente en monR (mr*diferencia/me), no -diferencia en monR. Corregido difUsd/difArs/difEur y remUsd/remArs/remEur en ambos bloques (cambiarEstadoTransaccion y saveTransaccion) para que la CC muestre "Pandy debe USD" y no ARS.</v>
+        <v>Regla sagrada: no tocar los originales (Debe y Compensación). En guardarSoloMontoTransaccion cuando newRestoMonto &lt; 1e-6 solo se actualiza estado a cerrado (no monto_usd/ars/eur a 0). En misma moneda (ARS-ARS): al hacer split se actualiza la Cancelación del ingreso 50.000→48.750; se insertan dos movimientos CC para que la comisión figure y la cuenta cierre en 0: Ganancia del acuerdo +1.250 y Comisión Pandy -1.250. Revertir borra ambos por transaccion_id.</v>
       </c>
       <c r="E105" t="str">
         <v>Desarrollo</v>
@@ -2198,16 +2198,16 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C106" t="str">
-        <v>CC resumen: agrupar por orden_id para una sola moneda</v>
+        <v>Sincronización CC y caja desde orden + transacciones</v>
       </c>
       <c r="D106" t="str">
-        <v>Al pasar una operación a pendiente el saldo debe mostrar solo la moneda que corresponde (ej. solo +2000 ARS). Se agrupa por orden_id en loadCuentaCorriente (select con orden_id) y en saldosDesdeMovimientosPorOrden se usa orden_id como clave de agrupación (fallback a parseOrdenNumero en concepto) para que todos los movimientos de la misma orden entren en un solo grupo y el saldo muestre una sola moneda.</v>
+        <v>Modelo: orden e instrumentación (transacciones) son la fuente de verdad; CC y caja se derivan por conciliación. Función sincronizarCcYCajaDesdeOrden(ordenId): borra movimientos CC (cliente e intermediario) y caja de la orden, recalcula desde todas las transacciones (cobro/deuda, Ganancia del acuerdo, comisión intermediario) e inserta. Invocada al cambiar estado de transacción (cambiarEstadoTransaccion), al guardar monto (guardarSoloMontoTransaccion), al guardar desde modal transacción (saveTransaccion → hacerCierre) y al auto-completar ARS-ARS con intermediario (en lugar de momento cero 2 filas).</v>
       </c>
       <c r="E106" t="str">
         <v>Desarrollo</v>
@@ -2215,16 +2215,16 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C107" t="str">
-        <v>CC Cancelación por monto de la transacción</v>
+        <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
       </c>
       <c r="D107" t="str">
-        <v>Al ejecutar una transacción (sin split) se insertaba Cancelación con mr/me (totales de la orden), generando saldo erróneo (ej. 1500 en vez de 1000). Corrección: montosCancelacion(item) usa item.monto; ingreso → +monto en monR y proporcional en monE; egreso → -monto en monE y proporcional en monR. Regla en docs y .cursor/rules: CC siempre debe cerrar con la regla conceptual; si no cierra, preguntar.</v>
+        <v>Al hacer split de egreso (ej. 1000→500 ejecutado, 500 pendiente) la diferencia está en monE (USD). La fila Debe (monR) debe llevar el equivalente en monR (mr*diferencia/me), no -diferencia en monR. Corregido difUsd/difArs/difEur y remUsd/remArs/remEur en ambos bloques (cambiarEstadoTransaccion y saveTransaccion) para que la CC muestre "Pandy debe USD" y no ARS.</v>
       </c>
       <c r="E107" t="str">
         <v>Desarrollo</v>
@@ -2232,16 +2232,16 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C108" t="str">
-        <v>Split CC: diferencia desde fila, no desde orden</v>
+        <v>CC resumen: agrupar por orden_id para una sola moneda</v>
       </c>
       <c r="D108" t="str">
-        <v>En el segundo (o n) split se usaba mr/me para la diferencia, generando pendiente erróneo (ej. 800 en vez de 200). Corrección: diferencia = resto en fila Debe/Comp − monto ejecutado. Aplicado en cambiarEstadoTransaccion y saveTransaccion. Así pagos parciales encadenados (500, luego 300) generan 200 pendiente.</v>
+        <v>Al pasar una operación a pendiente el saldo debe mostrar solo la moneda que corresponde (ej. solo +2000 ARS). Se agrupa por orden_id en loadCuentaCorriente (select con orden_id) y en saldosDesdeMovimientosPorOrden se usa orden_id como clave de agrupación (fallback a parseOrdenNumero en concepto) para que todos los movimientos de la misma orden entren en un solo grupo y el saldo muestre una sola moneda.</v>
       </c>
       <c r="E108" t="str">
         <v>Desarrollo</v>
@@ -2249,33 +2249,33 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C109" t="str">
-        <v>Tarea de análisis: modal transacción con ejecutadas</v>
+        <v>CC Cancelación por monto de la transacción</v>
       </c>
       <c r="D109" t="str">
-        <v>Con transacciones ya ejecutadas, el modal de Editar transacción sigue permitiendo editar todos los campos. Analizar si debe restringirse (solo lectura o bloquear edición cuando hay ejecutadas) para que la regla conceptual de CC se cumpla siempre. Revisar qué hace hoy el guardado y qué sería lo más seguro.</v>
+        <v>Al ejecutar una transacción (sin split) se insertaba Cancelación con mr/me (totales de la orden), generando saldo erróneo (ej. 1500 en vez de 1000). Corrección: montosCancelacion(item) usa item.monto; ingreso → +monto en monR y proporcional en monE; egreso → -monto en monE y proporcional en monR. Regla en docs y .cursor/rules: CC siempre debe cerrar con la regla conceptual; si no cierra, preguntar.</v>
       </c>
       <c r="E109" t="str">
-        <v>Análisis pendiente</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C110" t="str">
-        <v>Modal transacción ejecutada: solo concepto editable</v>
+        <v>Split CC: diferencia desde fila, no desde orden</v>
       </c>
       <c r="D110" t="str">
-        <v>Análisis en docs/ANALISIS_MODAL_TRANSACCION_EJECUTADA.md. Si la transacción está ejecutada, se deshabilitan tipo, modo de pago, moneda, monto, cobrador, pagador, estado y tipo de cambio; solo concepto se puede editar. Mensaje "Transacción cerrada. Solo puede editarse el concepto…". Regla conceptual preservada.</v>
+        <v>En el segundo (o n) split se usaba mr/me para la diferencia, generando pendiente erróneo (ej. 800 en vez de 200). Corrección: diferencia = resto en fila Debe/Comp − monto ejecutado. Aplicado en cambiarEstadoTransaccion y saveTransaccion. Así pagos parciales encadenados (500, luego 300) generan 200 pendiente.</v>
       </c>
       <c r="E110" t="str">
         <v>Desarrollo</v>
@@ -2283,33 +2283,33 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C111" t="str">
-        <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
+        <v>Tarea de análisis: modal transacción con ejecutadas</v>
       </c>
       <c r="D111" t="str">
-        <v>Se revierte la restricción del modal: modo de pago, importe y estado siguen editables (tabla y modal) también para ejecutadas. Principio: siempre re-estructurar la regla de CC cuando el usuario edita para que no se rompa. Estado editable para correcciones. Doc ANALISIS actualizado.</v>
+        <v>Con transacciones ya ejecutadas, el modal de Editar transacción sigue permitiendo editar todos los campos. Analizar si debe restringirse (solo lectura o bloquear edición cuando hay ejecutadas) para que la regla conceptual de CC se cumpla siempre. Revisar qué hace hoy el guardado y qué sería lo más seguro.</v>
       </c>
       <c r="E111" t="str">
-        <v>Desarrollo</v>
+        <v>Análisis pendiente</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C112" t="str">
-        <v>Reajuste CC y caja al editar monto o modo de pago</v>
+        <v>Modal transacción ejecutada: solo concepto editable</v>
       </c>
       <c r="D112" t="str">
-        <v>guardarSoloModoPagoTransaccion: si transacción ejecutada, borra mov_caja anterior e inserta uno con el nuevo modo. guardarSoloMontoTransaccion: si ejecutada, revierte Cancelación y caja, actualiza monto y transacción resto (o crea nueva pendiente), inserta nueva Cancelación y caja. saveTransaccion: al editar (id) revierte Cancelación/caja; en split actualiza transacción resto existente en vez de crear otra. Regla conceptual siempre re-estructurada.</v>
+        <v>Análisis en docs/ANALISIS_MODAL_TRANSACCION_EJECUTADA.md. Si la transacción está ejecutada, se deshabilitan tipo, modo de pago, moneda, monto, cobrador, pagador, estado y tipo de cambio; solo concepto se puede editar. Mensaje "Transacción cerrada. Solo puede editarse el concepto…". Regla conceptual preservada.</v>
       </c>
       <c r="E112" t="str">
         <v>Desarrollo</v>
@@ -2317,16 +2317,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C113" t="str">
-        <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
+        <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
       </c>
       <c r="D113" t="str">
-        <v>Si el usuario cambia el monto en la tabla (ej. 500) y luego pasa a Ejecutada sin hacer blur, el sistema usaba el monto en DB (1000) y no creaba la transacción pendiente por 500. En cambiarEstadoTransaccion, antes de ejecutar se lee el valor del input de monto de la fila; si difiere del monto en DB se llama guardarSoloMontoTransaccion y luego se re-ejecuta el cambio de estado, de modo que el split use siempre el monto que ve el usuario.</v>
+        <v>Se revierte la restricción del modal: modo de pago, importe y estado siguen editables (tabla y modal) también para ejecutadas. Principio: siempre re-estructurar la regla de CC cuando el usuario edita para que no se rompa. Estado editable para correcciones. Doc ANALISIS actualizado.</v>
       </c>
       <c r="E113" t="str">
         <v>Desarrollo</v>
@@ -2334,16 +2334,16 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C114" t="str">
-        <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
+        <v>Reajuste CC y caja al editar monto o modo de pago</v>
       </c>
       <c r="D114" t="str">
-        <v>Algunos inserts a movimientos_cuenta_corriente (legacy Cobro/Deuda, Conversión, Comisión) enviaban solo moneda y monto; las columnas monto_usd, monto_ars, monto_eur quedaban null y el saldo se rompía (ej. "Pandy debe 700 USD y 300 ARS" en vez de 1000 USD). Helper montosCcPorMoneda(moneda, valor); todos los inserts a mov_cc ahora incluyen ...montosCcPorMoneda. Script sql/corregir_mov_cc_montos_null.sql para backfill de filas existentes.</v>
+        <v>guardarSoloModoPagoTransaccion: si transacción ejecutada, borra mov_caja anterior e inserta uno con el nuevo modo. guardarSoloMontoTransaccion: si ejecutada, revierte Cancelación y caja, actualiza monto y transacción resto (o crea nueva pendiente), inserta nueva Cancelación y caja. saveTransaccion: al editar (id) revierte Cancelación/caja; en split actualiza transacción resto existente en vez de crear otra. Regla conceptual siempre re-estructurada.</v>
       </c>
       <c r="E114" t="str">
         <v>Desarrollo</v>
@@ -2351,16 +2351,16 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C115" t="str">
-        <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
+        <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
       </c>
       <c r="D115" t="str">
-        <v>En órdenes ARS-ARS (CHEQUE) con intermediario la ganancia (ej. 1000 ARS) se insertaba como "Cobro por" en CC cliente y el resumen mostraba "cliente debe 1000". Esa suma es la comisión que el cliente ya pagó, no un saldo. Se consulta comisiones_orden (beneficiario=pandy); si la transacción es ingreso cliente→Pandy con monto = comisión Pandy, no se inserta el Cobro en CC cliente. Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+        <v>Si el usuario cambia el monto en la tabla (ej. 500) y luego pasa a Ejecutada sin hacer blur, el sistema usaba el monto en DB (1000) y no creaba la transacción pendiente por 500. En cambiarEstadoTransaccion, antes de ejecutar se lee el valor del input de monto de la fila; si difiere del monto en DB se llama guardarSoloMontoTransaccion y luego se re-ejecuta el cambio de estado, de modo que el split use siempre el monto que ve el usuario.</v>
       </c>
       <c r="E115" t="str">
         <v>Desarrollo</v>
@@ -2368,16 +2368,16 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C116" t="str">
-        <v>Tasas de descuento: reconocer coma decimal</v>
+        <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
       </c>
       <c r="D116" t="str">
-        <v>Las tasas (cliente e intermediario %) no conservaban la coma al escribir (ej. "2," se convertía en "2"). En formatImporteInputOnType: cuando tieneDecimal, siempre se muestra la coma en el resultado (aunque parteDecimalStr esté vacía). Además con soloComaDecimal se acepta punto como decimal y se convierte a coma ("2.5" → "2,5"). Las tasas usan setupInputImporte(..., 2, true).</v>
+        <v>Algunos inserts a movimientos_cuenta_corriente (legacy Cobro/Deuda, Conversión, Comisión) enviaban solo moneda y monto; las columnas monto_usd, monto_ars, monto_eur quedaban null y el saldo se rompía (ej. "Pandy debe 700 USD y 300 ARS" en vez de 1000 USD). Helper montosCcPorMoneda(moneda, valor); todos los inserts a mov_cc ahora incluyen ...montosCcPorMoneda. Script sql/corregir_mov_cc_montos_null.sql para backfill de filas existentes.</v>
       </c>
       <c r="E116" t="str">
         <v>Desarrollo</v>
@@ -2385,16 +2385,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C117" t="str">
-        <v>Modal orden más ancho</v>
+        <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
       </c>
       <c r="D117" t="str">
-        <v>Clase modal-orden con max-width min(95vw, 1400px) para que la tabla de transacciones (Tipo, Modo pago, Moneda, Monto, Pagador, Cobrador, Estado, Editar) tenga más espacio horizontal.</v>
+        <v>En órdenes ARS-ARS (CHEQUE) con intermediario la ganancia (ej. 1000 ARS) se insertaba como "Cobro por" en CC cliente y el resumen mostraba "cliente debe 1000". Esa suma es la comisión que el cliente ya pagó, no un saldo. Se consulta comisiones_orden (beneficiario=pandy); si la transacción es ingreso cliente→Pandy con monto = comisión Pandy, no se inserta el Cobro en CC cliente. Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
       </c>
       <c r="E117" t="str">
         <v>Desarrollo</v>
@@ -2402,16 +2402,16 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C118" t="str">
-        <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
+        <v>Tasas de descuento: reconocer coma decimal</v>
       </c>
       <c r="D118" t="str">
-        <v>En órdenes con intermediario (ej. ARS-ARS CHEQUE) no hay filas Debe/Compensación (momento cero), por lo que al editar el importe y pasar a ejecutada no se creaba la transacción "resto" y se rompía instrumentación y CC. Se añade splitSinMomentoCero: al ejecutar con monto menor al compromiso (ingreso pagador=cliente mr&gt;monto, egreso cobrador=cliente me&gt;monto) se crea una transacción pendiente por la diferencia. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo).</v>
+        <v>Las tasas (cliente e intermediario %) no conservaban la coma al escribir (ej. "2," se convertía en "2"). En formatImporteInputOnType: cuando tieneDecimal, siempre se muestra la coma en el resultado (aunque parteDecimalStr esté vacía). Además con soloComaDecimal se acepta punto como decimal y se convierte a coma ("2.5" → "2,5"). Las tasas usan setupInputImporte(..., 2, true).</v>
       </c>
       <c r="E118" t="str">
         <v>Desarrollo</v>
@@ -2419,16 +2419,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C119" t="str">
-        <v>Split + CC + caja para cualquier tipo de operación</v>
+        <v>Modal orden más ancho</v>
       </c>
       <c r="D119" t="str">
-        <v>Verificación: (1) Caja con signo correcto (ingreso/egreso) en cambiarEstadoTransaccion y guardarSoloMontoTransaccion (signoCaja = cobrador===pandy ? 1 : -1). (2) guardarSoloMontoTransaccion sin momento cero: al bajar el monto ejecutado se crea transacción resto pendiente para mantener coherencia. (3) Doc FLUJOS_CC_REGLA.md actualizado con sección "Regla de split en sintonía con CC y caja".</v>
+        <v>Clase modal-orden con max-width min(95vw, 1400px) para que la tabla de transacciones (Tipo, Modo pago, Moneda, Monto, Pagador, Cobrador, Estado, Editar) tenga más espacio horizontal.</v>
       </c>
       <c r="E119" t="str">
         <v>Desarrollo</v>
@@ -2436,16 +2436,16 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C120" t="str">
-        <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
+        <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
       </c>
       <c r="D120" t="str">
-        <v>En ARS-ARS (CHEQUE) las transacciones generadas con modo de pago Cheque no pueden cambiarse a otro modo. guardarSoloModoPagoTransaccion rechaza con toast y onFailure (revierte combo). Tabla wizard y panel: celda modo de pago en solo lectura para esas transacciones. Modal: select modo de pago deshabilitado cuando es orden CHEQUE y la transacción tiene modo cheque.</v>
+        <v>En órdenes con intermediario (ej. ARS-ARS CHEQUE) no hay filas Debe/Compensación (momento cero), por lo que al editar el importe y pasar a ejecutada no se creaba la transacción "resto" y se rompía instrumentación y CC. Se añade splitSinMomentoCero: al ejecutar con monto menor al compromiso (ingreso pagador=cliente mr&gt;monto, egreso cobrador=cliente me&gt;monto) se crea una transacción pendiente por la diferencia. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo).</v>
       </c>
       <c r="E120" t="str">
         <v>Desarrollo</v>
@@ -2453,16 +2453,16 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C121" t="str">
-        <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
+        <v>Split + CC + caja para cualquier tipo de operación</v>
       </c>
       <c r="D121" t="str">
-        <v>Al ejecutar la última parte que cumple el cliente (suma de ingresos cliente ejecutados &gt;= mr y egresos a cliente ejecutados &gt;= me), se crea automáticamente la transacción "Ganancia del acuerdo" (monto = comisión Pandy de comisiones_orden), estado ejecutada, y su movimiento de caja. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo). Sincroniza instrumentación y CC con la comisión de Pandy.</v>
+        <v>Verificación: (1) Caja con signo correcto (ingreso/egreso) en cambiarEstadoTransaccion y guardarSoloMontoTransaccion (signoCaja = cobrador===pandy ? 1 : -1). (2) guardarSoloMontoTransaccion sin momento cero: al bajar el monto ejecutado se crea transacción resto pendiente para mantener coherencia. (3) Doc FLUJOS_CC_REGLA.md actualizado con sección "Regla de split en sintonía con CC y caja".</v>
       </c>
       <c r="E121" t="str">
         <v>Desarrollo</v>
@@ -2470,16 +2470,16 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C122" t="str">
-        <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
+        <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
       </c>
       <c r="D122" t="str">
-        <v>Al ejecutar la transacción de 10k (resto del split 40k→30k) el sistema generaba erróneamente otra transacción de 30k pendiente. Corrección: solo crear transacción "resto" cuando la suma de ingresos/egresos cliente ejecutados (tras esta ejecución) sigue siendo menor que mr/me. Se carga la lista de transacciones y se calculan sumIngresosClienteEjecutados y sumEgresosClienteEjecutados; faltaIngreso/faltaEgreso y diferencia = mr−suma (no mr−montoActual). En cambiarEstadoTransaccion la carga de transacciones se hace después del update para incluir esta transacción ya ejecutada. Aplicado en cambiarEstadoTransaccion, saveTransaccion (continuarFlujo) y guardarSoloMontoTransaccion.</v>
+        <v>En ARS-ARS (CHEQUE) las transacciones generadas con modo de pago Cheque no pueden cambiarse a otro modo. guardarSoloModoPagoTransaccion rechaza con toast y onFailure (revierte combo). Tabla wizard y panel: celda modo de pago en solo lectura para esas transacciones. Modal: select modo de pago deshabilitado cuando es orden CHEQUE y la transacción tiene modo cheque.</v>
       </c>
       <c r="E122" t="str">
         <v>Desarrollo</v>
@@ -2487,16 +2487,16 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C123" t="str">
-        <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
+        <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
       </c>
       <c r="D123" t="str">
-        <v>Al crear la transacción "Ganancia del acuerdo" (comisión Pandy) en ARS-ARS CHEQUE cuando el cliente completa, la instrumentación quedaba en 41k (30k+10k+1k) y rompía "A recibir 40.000". Se descuenta la comisión de una de las ingresos cliente→Pandy ejecutadas: se elige una con monto&gt;=comisión, se actualiza su monto (ej. 30k→29k), el movimiento de caja y el movimiento de CC (Cancelación) de esa transacción. Así instrumentación suma mr (40k). Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+        <v>Al ejecutar la última parte que cumple el cliente (suma de ingresos cliente ejecutados &gt;= mr y egresos a cliente ejecutados &gt;= me), se crea automáticamente la transacción "Ganancia del acuerdo" (monto = comisión Pandy de comisiones_orden), estado ejecutada, y su movimiento de caja. Aplicado en cambiarEstadoTransaccion y en saveTransaccion (continuarFlujo). Sincroniza instrumentación y CC con la comisión de Pandy.</v>
       </c>
       <c r="E123" t="str">
         <v>Desarrollo</v>
@@ -2504,16 +2504,16 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C124" t="str">
-        <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
+        <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
       </c>
       <c r="D124" t="str">
-        <v>El saldo de cuenta corriente intermediario solo consideraba movimientos ejecutados, por lo que no se mostraba la deuda pendiente (ej. 40.000 del cheque Pandy→Intermediario). Para que la regla sea la misma que con el cliente (saldo real): se cargan transacciones pendientes Pandy→Intermediario por intermediario y moneda; el saldo por moneda es el máximo entre lo que sale de movimientos y lo pendiente. loadCuentaCorriente con fetchPendingPandyIntermediario; buildCcResumenRows con saldosIntermediarioConPendientes; fetchMovimientosCcPorEntidad para intermediario también incorpora pendientes en el saldo del modal detalle.</v>
+        <v>Al ejecutar la transacción de 10k (resto del split 40k→30k) el sistema generaba erróneamente otra transacción de 30k pendiente. Corrección: solo crear transacción "resto" cuando la suma de ingresos/egresos cliente ejecutados (tras esta ejecución) sigue siendo menor que mr/me. Se carga la lista de transacciones y se calculan sumIngresosClienteEjecutados y sumEgresosClienteEjecutados; faltaIngreso/faltaEgreso y diferencia = mr−suma (no mr−montoActual). En cambiarEstadoTransaccion la carga de transacciones se hace después del update para incluir esta transacción ya ejecutada. Aplicado en cambiarEstadoTransaccion, saveTransaccion (continuarFlujo) y guardarSoloMontoTransaccion.</v>
       </c>
       <c r="E124" t="str">
         <v>Desarrollo</v>
@@ -2521,16 +2521,16 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C125" t="str">
-        <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
+        <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
       </c>
       <c r="D125" t="str">
-        <v>Para igualar la regla con cliente: al instrumentar CHEQUE con intermediario se inserta la fila de momento cero (Debe … nro orden N, monto negativo, pendiente). Al ejecutar el egreso Pandy→Intermediario (cheque) no se inserta una fila nueva; se busca si existe fila con ese transaccion_id y se actualiza a estado cerrado. Si no existe (órdenes sin momento cero), se inserta como antes. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
+        <v>Al crear la transacción "Ganancia del acuerdo" (comisión Pandy) en ARS-ARS CHEQUE cuando el cliente completa, la instrumentación quedaba en 41k (30k+10k+1k) y rompía "A recibir 40.000". Se descuenta la comisión de una de las ingresos cliente→Pandy ejecutadas: se elige una con monto&gt;=comisión, se actualiza su monto (ej. 30k→29k), el movimiento de caja y el movimiento de CC (Cancelación) de esa transacción. Así instrumentación suma mr (40k). Aplicado en cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
       </c>
       <c r="E125" t="str">
         <v>Desarrollo</v>
@@ -2538,16 +2538,16 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C126" t="str">
-        <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
+        <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
       </c>
       <c r="D126" t="str">
-        <v>Operaciones dos monedas (monR ≠ monE): cuando el cliente paga (ingreso ejecutada), se insertan dos movimientos CC: Cancelación de deuda (+monto en monR) y Contraparte cancelación (-monto en monR, -enMonE en monE). La suma da 0 en USD y solo queda Pandy debe ARS. Aplicado en guardarSoloMontoTransaccion, sincronizarCcYCajaDesdeOrden (Refrescar), saveTransaccion (!tieneMomentoCero). Al revertir se borran ambos conceptos (Cancelación y Contraparte cancelación) en saveTransaccion, guardarSoloMontoTransaccion y cambiarEstadoTransaccion.</v>
+        <v>El saldo de cuenta corriente intermediario solo consideraba movimientos ejecutados, por lo que no se mostraba la deuda pendiente (ej. 40.000 del cheque Pandy→Intermediario). Para que la regla sea la misma que con el cliente (saldo real): se cargan transacciones pendientes Pandy→Intermediario por intermediario y moneda; el saldo por moneda es el máximo entre lo que sale de movimientos y lo pendiente. loadCuentaCorriente con fetchPendingPandyIntermediario; buildCcResumenRows con saldosIntermediarioConPendientes; fetchMovimientosCcPorEntidad para intermediario también incorpora pendientes en el saldo del modal detalle.</v>
       </c>
       <c r="E126" t="str">
         <v>Desarrollo</v>
@@ -2555,16 +2555,16 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C127" t="str">
-        <v>CC regla simple: Compromiso y Compromiso Saldado</v>
+        <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
       </c>
       <c r="D127" t="str">
-        <v>Un registro por evento y por moneda. Momento cero: 2 filas Compromiso (una por moneda, solo esa moneda con valor); concepto "Compromiso - Orden Nro X y Trans Nro Y". Al ejecutar: 1 fila "Compromiso Saldado" por moneda pagada (una moneda por fila). Sin uso de estado para saldo (solo se excluye anulado). transaccion_numero en mov_cc y mov_cc_int (migración sql/migracion_cc_transaccion_numero_y_regla_simple.sql). Doc docs/REGLA_CC_SIMPLE.md. insertarMovimientosCcMomentoCero e Intermediario; sincronizarCcYCajaDesdeOrden con usarReglaSimpleCliente.</v>
+        <v>Para igualar la regla con cliente: al instrumentar CHEQUE con intermediario se inserta la fila de momento cero (Debe … nro orden N, monto negativo, pendiente). Al ejecutar el egreso Pandy→Intermediario (cheque) no se inserta una fila nueva; se busca si existe fila con ese transaccion_id y se actualiza a estado cerrado. Si no existe (órdenes sin momento cero), se inserta como antes. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion (continuarFlujo).</v>
       </c>
       <c r="E127" t="str">
         <v>Desarrollo</v>
@@ -2572,16 +2572,16 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C128" t="str">
-        <v>CC vista: saldo solo transacciones ejecutadas</v>
+        <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
       </c>
       <c r="D128" t="str">
-        <v>En la vista de Cuenta corriente (resumen y modal detalle) el saldo se calcula solo con movimientos que corresponden a transacciones ejecutadas. Si todas están pendientes, nadie le debe nada a nadie. Regla: Compromiso Saldado siempre cuenta; Compromiso solo si la transacción está ejecutada o la orden tiene al menos una ejecutada. loadCuentaCorriente y fetchMovimientosCcPorEntidad cargan transacciones e instrumentación para filtrar antes de sumar.</v>
+        <v>Operaciones dos monedas (monR ≠ monE): cuando el cliente paga (ingreso ejecutada), se insertan dos movimientos CC: Cancelación de deuda (+monto en monR) y Contraparte cancelación (-monto en monR, -enMonE en monE). La suma da 0 en USD y solo queda Pandy debe ARS. Aplicado en guardarSoloMontoTransaccion, sincronizarCcYCajaDesdeOrden (Refrescar), saveTransaccion (!tieneMomentoCero). Al revertir se borran ambos conceptos (Cancelación y Contraparte cancelación) en saveTransaccion, guardarSoloMontoTransaccion y cambiarEstadoTransaccion.</v>
       </c>
       <c r="E128" t="str">
         <v>Desarrollo</v>
@@ -2589,16 +2589,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C129" t="str">
-        <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
+        <v>CC regla simple: Compromiso y Compromiso Saldado</v>
       </c>
       <c r="D129" t="str">
-        <v>Reversa ejecutada→pendiente intermediario: ya no se hace flip monto en todas las filas. Solo filas de la transacción revocada: Debe (monto&lt;0) → UPDATE estado pendiente; cobro (monto&gt;0) → DELETE. Aplicado en cambiarEstadoTransaccion y saveTransaccion (revertCcInt). Relojería: dismissAllToasts() al cerrar modal orden y modal transacción; al cerrar modal orden se sincronizan montos de la tabla de instrumentación (guardarSoloMontoTransaccion por input) para no perder cambios sin blur. Doc DIAGNOSTICO_SINCRONIZACION_CC_Y_MODAL.md.</v>
+        <v>Un registro por evento y por moneda. Momento cero: 2 filas Compromiso (una por moneda, solo esa moneda con valor); concepto "Compromiso - Orden Nro X y Trans Nro Y". Al ejecutar: 1 fila "Compromiso Saldado" por moneda pagada (una moneda por fila). Sin uso de estado para saldo (solo se excluye anulado). transaccion_numero en mov_cc y mov_cc_int (migración sql/migracion_cc_transaccion_numero_y_regla_simple.sql). Doc docs/REGLA_CC_SIMPLE.md. insertarMovimientosCcMomentoCero e Intermediario; sincronizarCcYCajaDesdeOrden con usarReglaSimpleCliente.</v>
       </c>
       <c r="E129" t="str">
         <v>Desarrollo</v>
@@ -2606,16 +2606,16 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C130" t="str">
-        <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
+        <v>CC vista: saldo solo transacciones ejecutadas</v>
       </c>
       <c r="D130" t="str">
-        <v>Al instrumentar ARS-ARS (CHEQUE) con intermediario no se insertaban registros de momento cero en CC cliente; solo en CC intermediario. La regla debe ser única: en momento cero se cargan ambas cuentas corrientes (cliente con Pandy e intermediario con Pandy). En autoCompletarInstrumentacionChequeConIntermediario se llama ahora también a insertarMovimientosCcMomentoCero(ordenId, orden, ingresoClienteId, egresoClienteId) con las transacciones 1 y 2 (ingreso cliente→Pandy, egreso Pandy→cliente), además de insertarMovimientosCcMomentoCeroIntermediario.</v>
+        <v>En la vista de Cuenta corriente (resumen y modal detalle) el saldo se calcula solo con movimientos que corresponden a transacciones ejecutadas. Si todas están pendientes, nadie le debe nada a nadie. Regla: Compromiso Saldado siempre cuenta; Compromiso solo si la transacción está ejecutada o la orden tiene al menos una ejecutada. loadCuentaCorriente y fetchMovimientosCcPorEntidad cargan transacciones e instrumentación para filtrar antes de sumar.</v>
       </c>
       <c r="E130" t="str">
         <v>Desarrollo</v>
@@ -2623,16 +2623,16 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C131" t="str">
-        <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
+        <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
       </c>
       <c r="D131" t="str">
-        <v>El INSERT de momento cero fallaba por CHECK estado solo cerrado/anulado. Migración migracion_cc_intermediario_estado_pendiente.sql permite pendiente. Ejecutar en Supabase SQL Editor.</v>
+        <v>Reversa ejecutada→pendiente intermediario: ya no se hace flip monto en todas las filas. Solo filas de la transacción revocada: Debe (monto&lt;0) → UPDATE estado pendiente; cobro (monto&gt;0) → DELETE. Aplicado en cambiarEstadoTransaccion y saveTransaccion (revertCcInt). Relojería: dismissAllToasts() al cerrar modal orden y modal transacción; al cerrar modal orden se sincronizan montos de la tabla de instrumentación (guardarSoloMontoTransaccion por input) para no perder cambios sin blur. Doc DIAGNOSTICO_SINCRONIZACION_CC_Y_MODAL.md.</v>
       </c>
       <c r="E131" t="str">
         <v>Desarrollo</v>
@@ -2640,16 +2640,16 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C132" t="str">
-        <v>Reglas CC, caja e instrucciones: mejoras finales</v>
+        <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
       </c>
       <c r="D132" t="str">
-        <v>eliminarTransaccion: verificación de momento cero también en movimientos_cuenta_corriente_intermediario (no permitir baja si la transacción forma parte del momento cero en CC intermediario). Caja: comentarios que documentan que el saldo solo cuenta movimientos con estado cerrado (anulados no cuentan). guardarSoloModoPagoTransaccion: signo de caja correcto (signoCaja = cobrador===pandy ? 1 : -1) al reinsertar movimiento de caja. Regla conceptual de CC, caja e instrucciones alineada en todos los flujos.</v>
+        <v>Al instrumentar ARS-ARS (CHEQUE) con intermediario no se insertaban registros de momento cero en CC cliente; solo en CC intermediario. La regla debe ser única: en momento cero se cargan ambas cuentas corrientes (cliente con Pandy e intermediario con Pandy). En autoCompletarInstrumentacionChequeConIntermediario se llama ahora también a insertarMovimientosCcMomentoCero(ordenId, orden, ingresoClienteId, egresoClienteId) con las transacciones 1 y 2 (ingreso cliente→Pandy, egreso Pandy→cliente), además de insertarMovimientosCcMomentoCeroIntermediario.</v>
       </c>
       <c r="E132" t="str">
         <v>Desarrollo</v>
@@ -2657,16 +2657,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C133" t="str">
-        <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
+        <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
       </c>
       <c r="D133" t="str">
-        <v>Las tablas de CC cliente e intermediario deben ser idénticas. Migración añade monto_usd, monto_ars, monto_eur a movimientos_cuenta_corriente_intermediario. insertarMovimientosCcMomentoCeroIntermediario inserta con esas columnas; loadCuentaCorriente y fetchMovimientosCcPorEntidad las incluyen en el select. Reversa identifica momento cero por monto_usd/ars/eur no null.</v>
+        <v>El INSERT de momento cero fallaba por CHECK estado solo cerrado/anulado. Migración migracion_cc_intermediario_estado_pendiente.sql permite pendiente. Ejecutar en Supabase SQL Editor.</v>
       </c>
       <c r="E133" t="str">
         <v>Desarrollo</v>
@@ -2674,16 +2674,16 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C134" t="str">
-        <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
+        <v>Reglas CC, caja e instrucciones: mejoras finales</v>
       </c>
       <c r="D134" t="str">
-        <v>Al pasar a ejecutada el ingreso Intermediario→Pandy (efectivo) se debe marcar la fila Compensación de momento cero como cerrada y luego insertar el cobro. En insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion se hace primero UPDATE estado cerrado donde transaccion_id y estado pendiente, después INSERT del cobro.</v>
+        <v>eliminarTransaccion: verificación de momento cero también en movimientos_cuenta_corriente_intermediario (no permitir baja si la transacción forma parte del momento cero en CC intermediario). Caja: comentarios que documentan que el saldo solo cuenta movimientos con estado cerrado (anulados no cuentan). guardarSoloModoPagoTransaccion: signo de caja correcto (signoCaja = cobrador===pandy ? 1 : -1) al reinsertar movimiento de caja. Regla conceptual de CC, caja e instrucciones alineada en todos los flujos.</v>
       </c>
       <c r="E134" t="str">
         <v>Desarrollo</v>
@@ -2691,16 +2691,16 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C135" t="str">
-        <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
+        <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
       </c>
       <c r="D135" t="str">
-        <v>En momento cero las dos filas (Debe y Compensación) ya suman 0. Se quitó la capa de obligaciones pendientes (transacciones Pandy→Intermediario pendientes) que forzaba mostrar Pandy debe X. Resumen y modal detalle usan solo la suma de movimientos, igual que cliente. Eliminados fetchPendingPandyIntermediario y saldosIntermediarioConPendientes.</v>
+        <v>Las tablas de CC cliente e intermediario deben ser idénticas. Migración añade monto_usd, monto_ars, monto_eur a movimientos_cuenta_corriente_intermediario. insertarMovimientosCcMomentoCeroIntermediario inserta con esas columnas; loadCuentaCorriente y fetchMovimientosCcPorEntidad las incluyen en el select. Reversa identifica momento cero por monto_usd/ars/eur no null.</v>
       </c>
       <c r="E135" t="str">
         <v>Desarrollo</v>
@@ -2708,16 +2708,16 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C136" t="str">
-        <v>CC cliente: Cancelación alineada con monto de la transacción</v>
+        <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
       </c>
       <c r="D136" t="str">
-        <v>La Cancelación de deuda debe usar siempre el monto de la transacción (item.monto), no el total de la orden. Helper montosCancelacionDesdeOrden(item, orden). Al aplicar Ganancia del acuerdo se sincroniza la fila Cancelación del egreso Pandy→cliente con el monto actual de esa transacción. Script sql/corregir_cancelacion_cc_egreso_monto.sql para corregir datos existentes.</v>
+        <v>Al pasar a ejecutada el ingreso Intermediario→Pandy (efectivo) se debe marcar la fila Compensación de momento cero como cerrada y luego insertar el cobro. En insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion se hace primero UPDATE estado cerrado donde transaccion_id y estado pendiente, después INSERT del cobro.</v>
       </c>
       <c r="E136" t="str">
         <v>Desarrollo</v>
@@ -2725,16 +2725,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C137" t="str">
-        <v>CC intermediario: alta de comisión del intermediario</v>
+        <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
       </c>
       <c r="D137" t="str">
-        <v>Al completar el cliente (Ganancia del acuerdo) se inserta en movimientos_cuenta_corriente_intermediario un movimiento "Comisión del acuerdo" por la comisión con beneficiario=intermediario (comisiones_orden), con monto negativo (Pandy paga al intermediario). Una sola vez por orden. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>En momento cero las dos filas (Debe y Compensación) ya suman 0. Se quitó la capa de obligaciones pendientes (transacciones Pandy→Intermediario pendientes) que forzaba mostrar Pandy debe X. Resumen y modal detalle usan solo la suma de movimientos, igual que cliente. Eliminados fetchPendingPandyIntermediario y saldosIntermediarioConPendientes.</v>
       </c>
       <c r="E137" t="str">
         <v>Desarrollo</v>
@@ -2742,16 +2742,16 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C138" t="str">
-        <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
+        <v>CC cliente: Cancelación alineada con monto de la transacción</v>
       </c>
       <c r="D138" t="str">
-        <v>Al crear la transacción Ganancia del acuerdo se inserta también en movimientos_cuenta_corriente un movimiento con ese concepto y monto (montosCcPorMoneda) para que la CC cliente cierre correctamente. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>La Cancelación de deuda debe usar siempre el monto de la transacción (item.monto), no el total de la orden. Helper montosCancelacionDesdeOrden(item, orden). Al aplicar Ganancia del acuerdo se sincroniza la fila Cancelación del egreso Pandy→cliente con el monto actual de esa transacción. Script sql/corregir_cancelacion_cc_egreso_monto.sql para corregir datos existentes.</v>
       </c>
       <c r="E138" t="str">
         <v>Desarrollo</v>
@@ -2759,16 +2759,16 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C139" t="str">
-        <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
+        <v>CC intermediario: alta de comisión del intermediario</v>
       </c>
       <c r="D139" t="str">
-        <v>Todos los inserts en movimientos_cuenta_corriente_intermediario incluyen ...montosCcPorMoneda. Al ejecutar el ingreso Int→Pandy se asegura Comisión del acuerdo (comisiones_orden) si no existe. Script sql/corregir_cc_intermediario_montos_null.sql para datos existentes.</v>
+        <v>Al completar el cliente (Ganancia del acuerdo) se inserta en movimientos_cuenta_corriente_intermediario un movimiento "Comisión del acuerdo" por la comisión con beneficiario=intermediario (comisiones_orden), con monto negativo (Pandy paga al intermediario). Una sola vez por orden. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E139" t="str">
         <v>Desarrollo</v>
@@ -2776,16 +2776,16 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C140" t="str">
-        <v>CC intermediario: descuento y comisión al entregar cheques</v>
+        <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
       </c>
       <c r="D140" t="str">
-        <v>Al ejecutar ingreso Int→Pandy: se inserta movimiento "Descuento sobre cheque" (-monto) para que la CC cierre (nominal cheque vs efectivo recibido). Al ejecutar egreso Pandy→Int: se crea transacción "Comisión del acuerdo" (egreso Pandy→intermediario), movimiento de caja y movimiento en CC intermediario. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion.</v>
+        <v>Al crear la transacción Ganancia del acuerdo se inserta también en movimientos_cuenta_corriente un movimiento con ese concepto y monto (montosCcPorMoneda) para que la CC cliente cierre correctamente. Aplicado en cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E140" t="str">
         <v>Desarrollo</v>
@@ -2793,16 +2793,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C141" t="str">
-        <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
+        <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
       </c>
       <c r="D141" t="str">
-        <v>En saveTransaccion, esOrdenCheque se obtiene desde la orden (tipos_operacion.codigo === ARS-ARS) en lugar del DOM, para que al crear la transacción Ganancia del acuerdo se ejecute siempre el insert en movimientos_cuenta_corriente (movimiento positivo por la comisión) y cierre la CC con el cliente.</v>
+        <v>Todos los inserts en movimientos_cuenta_corriente_intermediario incluyen ...montosCcPorMoneda. Al ejecutar el ingreso Int→Pandy se asegura Comisión del acuerdo (comisiones_orden) si no existe. Script sql/corregir_cc_intermediario_montos_null.sql para datos existentes.</v>
       </c>
       <c r="E141" t="str">
         <v>Desarrollo</v>
@@ -2810,16 +2810,16 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C142" t="str">
-        <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
+        <v>CC intermediario: descuento y comisión al entregar cheques</v>
       </c>
       <c r="D142" t="str">
-        <v>Nueva tabla orden_comisiones_generadas (orden_id, tipo ganancia_pandy|comision_intermediario, transaccion_id, transaccion_id_reducida). Helpers asegurarGananciaPandy, revertirGananciaPandy, asegurarComisionIntermediario, revertirComisionIntermediario. Al crear: solo si no existe fila. Al pasar ejecutada→pendiente: se revierte comisión (borrar transacción, caja, CC, fila); ingreso Int→Pandy se revierte cobro+descuento y Compensación; si el cliente deja de completar se revierte Ganancia y se restaura ingreso reducido. Migración sql/migracion_orden_comisiones_generadas.sql. Doc FLUJOS_CC_REGLA.md §8.</v>
+        <v>Al ejecutar ingreso Int→Pandy: se inserta movimiento "Descuento sobre cheque" (-monto) para que la CC cierre (nominal cheque vs efectivo recibido). Al ejecutar egreso Pandy→Int: se crea transacción "Comisión del acuerdo" (egreso Pandy→intermediario), movimiento de caja y movimiento en CC intermediario. Aplicado en insertarMovimientosCcParaTransaccion, cambiarEstadoTransaccion y saveTransaccion.</v>
       </c>
       <c r="E142" t="str">
         <v>Desarrollo</v>
@@ -2827,16 +2827,16 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C143" t="str">
-        <v>Reajuste tests E2E y signos CC regla simple</v>
+        <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
       </c>
       <c r="D143" t="str">
-        <v>Tests orden-cc.spec.js: timeouts aumentados para vista CC (cc-loading hidden 45s, tbody primera fila 15s) por las consultas extra de transacciones e instrumentación. App: signos CC regla simple corregidos: Compromiso monE (Pandy debe) se guarda con -me; Compromiso Saldado egreso con +monto para que "Pandy debe" se muestre como valor negativo. Ejecutar npx playwright install si falta; app en marcha y .env.test para correr tests.</v>
+        <v>En saveTransaccion, esOrdenCheque se obtiene desde la orden (tipos_operacion.codigo === ARS-ARS) en lugar del DOM, para que al crear la transacción Ganancia del acuerdo se ejecute siempre el insert en movimientos_cuenta_corriente (movimiento positivo por la comisión) y cierre la CC con el cliente.</v>
       </c>
       <c r="E143" t="str">
         <v>Desarrollo</v>
@@ -2844,16 +2844,16 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C144" t="str">
-        <v>Refresh sin colapsar secciones expandidas</v>
+        <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
       </c>
       <c r="D144" t="str">
-        <v>El refresco automático (cada 30 s) y el criterio de no refrescar con modal abierto se extiende: si hay una sección expandida en la vista actual no se ejecuta el refresh para no colapsarla. Órdenes: detalle de transacciones expandido (transaccionesOrdenIdActual). Seguridad: menú o rol expandido. hasExpandedSectionInCurrentView(); refreshCurrentViewData() retorna sin recargar cuando hay expansión.</v>
+        <v>Nueva tabla orden_comisiones_generadas (orden_id, tipo ganancia_pandy|comision_intermediario, transaccion_id, transaccion_id_reducida). Helpers asegurarGananciaPandy, revertirGananciaPandy, asegurarComisionIntermediario, revertirComisionIntermediario. Al crear: solo si no existe fila. Al pasar ejecutada→pendiente: se revierte comisión (borrar transacción, caja, CC, fila); ingreso Int→Pandy se revierte cobro+descuento y Compensación; si el cliente deja de completar se revierte Ganancia y se restaura ingreso reducido. Migración sql/migracion_orden_comisiones_generadas.sql. Doc FLUJOS_CC_REGLA.md §8.</v>
       </c>
       <c r="E144" t="str">
         <v>Desarrollo</v>
@@ -2861,16 +2861,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C145" t="str">
-        <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
+        <v>Reajuste tests E2E y signos CC regla simple</v>
       </c>
       <c r="D145" t="str">
-        <v>En órdenes ARS-USD, USD-ARS y USD-USD (sin intermediario) el tipo tiene usa_intermediario=false y el wrap #orden-wrap-intermediario se oculta; el test intentaba selectOption en #orden-intermediario y fallaba por "element is not visible". Se espera a que el wrap esté hidden tras elegir el tipo y solo se selecciona intermediario cuando el wrap es visible.</v>
+        <v>Tests orden-cc.spec.js: timeouts aumentados para vista CC (cc-loading hidden 45s, tbody primera fila 15s) por las consultas extra de transacciones e instrumentación. App: signos CC regla simple corregidos: Compromiso monE (Pandy debe) se guarda con -me; Compromiso Saldado egreso con +monto para que "Pandy debe" se muestre como valor negativo. Ejecutar npx playwright install si falta; app en marcha y .env.test para correr tests.</v>
       </c>
       <c r="E145" t="str">
         <v>Desarrollo</v>
@@ -2878,16 +2878,16 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C146" t="str">
-        <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
+        <v>Refresh sin colapsar secciones expandidas</v>
       </c>
       <c r="D146" t="str">
-        <v>En los modales de Cliente e Intermediario el campo Activo pasa de checkbox a toggle switch (mismo estilo que en Tipos de operación). Clases form-group-toggle y label-with-toggle; mismo .toggle-switch con .slider. IDs cliente-activo e intermediario-activo sin cambios.</v>
+        <v>El refresco automático (cada 30 s) y el criterio de no refrescar con modal abierto se extiende: si hay una sección expandida en la vista actual no se ejecuta el refresh para no colapsarla. Órdenes: detalle de transacciones expandido (transaccionesOrdenIdActual). Seguridad: menú o rol expandido. hasExpandedSectionInCurrentView(); refreshCurrentViewData() retorna sin recargar cuando hay expansión.</v>
       </c>
       <c r="E146" t="str">
         <v>Desarrollo</v>
@@ -2895,16 +2895,16 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C147" t="str">
-        <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
+        <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
       </c>
       <c r="D147" t="str">
-        <v>En la tabla de Clientes y en la de Intermediarios la columna Activo muestra un toggle switch (como en Tipos de operación). Al cambiar el switch se actualiza activo en Supabase sin abrir el modal. Sin SQL: los datos ya están; solo cambia la UI.</v>
+        <v>En órdenes ARS-USD, USD-ARS y USD-USD (sin intermediario) el tipo tiene usa_intermediario=false y el wrap #orden-wrap-intermediario se oculta; el test intentaba selectOption en #orden-intermediario y fallaba por "element is not visible". Se espera a que el wrap esté hidden tras elegir el tipo y solo se selecciona intermediario cuando el wrap es visible.</v>
       </c>
       <c r="E147" t="str">
         <v>Desarrollo</v>
@@ -2912,16 +2912,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C148" t="str">
-        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
+        <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
       </c>
       <c r="D148" t="str">
-        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
+        <v>En los modales de Cliente e Intermediario el campo Activo pasa de checkbox a toggle switch (mismo estilo que en Tipos de operación). Clases form-group-toggle y label-with-toggle; mismo .toggle-switch con .slider. IDs cliente-activo e intermediario-activo sin cambios.</v>
       </c>
       <c r="E148" t="str">
         <v>Desarrollo</v>
@@ -2929,16 +2929,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C149" t="str">
-        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
+        <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
       </c>
       <c r="D149" t="str">
-        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
+        <v>En la tabla de Clientes y en la de Intermediarios la columna Activo muestra un toggle switch (como en Tipos de operación). Al cambiar el switch se actualiza activo en Supabase sin abrir el modal. Sin SQL: los datos ya están; solo cambia la UI.</v>
       </c>
       <c r="E149" t="str">
         <v>Desarrollo</v>
@@ -2946,16 +2946,16 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C150" t="str">
-        <v>Evitar updates de monto 0 en transacciones</v>
+        <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
       </c>
       <c r="D150" t="str">
-        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
+        <v>Al cerrar instrumentación (instrumentacion_cerrada_ejecucion) se llamaba a generarTransaccionesCompensacionPandyIntermediario, que creaba transacciones de compensación/comisión y movimientos en CC intermediario, duplicando la comisión ya creada con asegurarComisionIntermediario y pudiendo generar movimientos erróneos (ej. -51250). Para órdenes ARS-ARS con intermediario se omite esa llamada: el flujo correcto es momento cero + asegurarComisionIntermediario al ejecutar egreso Pandy→Int.</v>
       </c>
       <c r="E150" t="str">
         <v>Desarrollo</v>
@@ -2963,16 +2963,16 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C151" t="str">
-        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
+        <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
       </c>
       <c r="D151" t="str">
-        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
+        <v>Con intermediario se aplicaban dos veces el descuento de comisión: (1) split inline (debeDividir) bajaba el ingreso a monto_entregado y creaba Ganancia; (2) asegurarGananciaPandy creaba otra Ganancia y volvía a descontar del mismo ingreso, pudiendo llevar montos a 0. Correcciones: debeDividir solo cuando !intermediarioId; en asegurarGananciaPandy elegir para reducir la transacción de mayor monto estrictamente mayor que la comisión (nunca reducir una que quedaría en 0).</v>
       </c>
       <c r="E151" t="str">
         <v>Desarrollo</v>
@@ -2980,16 +2980,16 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C152" t="str">
-        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
+        <v>Evitar updates de monto 0 en transacciones</v>
       </c>
       <c r="D152" t="str">
-        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
+        <v>Protección en todos los flujos que escriben monto en transacciones: (1) asegurarGananciaPandy: no actualizar la transacción reducida si nuevoMonto &lt; 1e-6. (2) saveTransaccion split: solo update/insert transacción resto si diferencia &gt;= 1e-6. (3) cambiarEstadoTransaccion split: solo insertar transacción resto si diferencia &gt;= 1e-6. (4) guardarSoloMontoTransaccion: solo actualizar transacción resto si newRestoMonto &gt;= 1e-6. Así no se persiste monto 0 por descuento ni por split.</v>
       </c>
       <c r="E152" t="str">
         <v>Desarrollo</v>
@@ -2997,16 +2997,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C153" t="str">
-        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
+        <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
       </c>
       <c r="D153" t="str">
-        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
+        <v>Al pasar a ejecutada el egreso Pandy→intermediario (entrega de cheques), la CC intermediario debe reflejar que el intermediario le debe a Pandy (+montoEfectivoInt). En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→intermediario ejecutada y hay menos de 2 filas con monto ≈ +montoEfectivoInt, se insertan las que falten con concepto "Intermediario debe a Pandy" y estado cerrado. Misma lógica que CC cliente (dos -me cuando ingreso cliente ejecutada).</v>
       </c>
       <c r="E153" t="str">
         <v>Desarrollo</v>
@@ -3014,16 +3014,16 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C154" t="str">
-        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
+        <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
       </c>
       <c r="D154" t="str">
-        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
+        <v>Cuando Pandy paga al cliente (egreso Pandy→cliente ejecutada), el saldo debe pasar de -48.750 a 0. En sincronizarCcYCajaDesdeOrden se agrega bloque: si egreso Pandy→cliente ejecutada y no existe fila con monto ≈ +monto de esa transacción, se inserta una con concepto "Pago Pandy al cliente" y estado cerrado. Caja ya registraba el egreso en el forEach por transacción ejecutada.</v>
       </c>
       <c r="E154" t="str">
         <v>Desarrollo</v>
@@ -3031,16 +3031,16 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C155" t="str">
-        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
+        <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
       </c>
       <c r="D155" t="str">
-        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
+        <v>Regla sagrada: los 50.000 (monto_recibido) no se reemplazan por el monto reducido de la transacción. Cuando existe Ganancia del acuerdo, el ingreso cliente→Pandy puede estar en 48.750 en la transacción; en CC el Cobro debe seguir siendo +mr (50.000) para compensar con Comisión Pandy -1.250. En el forEach, al armar la fila Cobro para ingreso cliente→Pandy, si yaTieneGananciaTrx se usa mr y monR en lugar de t.monto y t.moneda.</v>
       </c>
       <c r="E155" t="str">
         <v>Desarrollo</v>
@@ -3048,16 +3048,16 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C156" t="str">
-        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
+        <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
       </c>
       <c r="D156" t="str">
-        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
+        <v>Cuando existe Ganancia del acuerdo no se inserta la fila "Ganancia del acuerdo" +1.250 en CC (esa suma ya está en el Cobro 50.000). Sí se inserta "Comisión Pandy" -1.250 para que el saldo cierre en 0: 50.000 - 1.250 - 48.750 - 48.750 + 48.750 = 0. El -1.250 es el movimiento que debe estar en la CC.</v>
       </c>
       <c r="E156" t="str">
         <v>Desarrollo</v>
@@ -3065,16 +3065,16 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C157" t="str">
-        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
+        <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
       </c>
       <c r="D157" t="str">
-        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
+        <v>Al ejecutarse el ingreso Intermediario→Pandy (49.250) no se duplica +49.250. Se deja de insertar el "Cobro" positivo en el forEach y se agrega un movimiento negativo -49.250 "Pago Intermediario a Pandy" para cerrar la CC en 0: +49.250 (Intermediario debe) - 49.250 (Pago) = 0. Mismo criterio que cliente (no duplicar, cerrar con el movimiento correcto).</v>
       </c>
       <c r="E157" t="str">
         <v>Desarrollo</v>
@@ -3082,16 +3082,16 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C158" t="str">
-        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
+        <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
       </c>
       <c r="D158" t="str">
-        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
+        <v>Solo debe haber una fila +49.250 "Intermediario debe a Pandy", no dos. Se corrige cuantasFaltanInt: de cuantasCobroInt &lt; 2 a cuantasCobroInt &lt; 1, y (2 - cuantasCobroInt) a (1 - cuantasCobroInt), para agregar como máximo una fila.</v>
       </c>
       <c r="E158" t="str">
         <v>Desarrollo</v>
@@ -3099,16 +3099,16 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C159" t="str">
-        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
+        <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
       </c>
       <c r="D159" t="str">
-        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
+        <v>Comisión Intermediario pasa a +750 (parte de los 50.000 que se queda el intermediario; -50.000 + 49.250 + 750 = 0). Las 3 líneas (-50.000, +750, +49.250) existen desde momento cero siempre que haya egreso Pandy→Int; la +49.250 "Intermediario debe a Pandy" estado pendiente/cerrado según si el ingreso Int→Pandy está ejecutada. Pasos: 0 = suma 0; 1 = egreso ejecutada, saldo +49.250; 2 = ingreso ejecutada, suma sigue 0 (no se agrega fila Pago -49.250: el cobro ya está en la +49.250).</v>
       </c>
       <c r="E159" t="str">
         <v>Desarrollo</v>
@@ -3116,16 +3116,16 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C160" t="str">
-        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
+        <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
       </c>
       <c r="D160" t="str">
-        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
+        <v>Las 3 líneas -50.000, +750, +49.250 ya suman 0. No se agrega movimiento "Pago Intermediario a Pandy" -49.250 al ejecutar el ingreso Int→Pandy; agregarlo duplicaba el 49.250 y daba suma -49.250. El cobro ya está reflejado en la línea +49.250.</v>
       </c>
       <c r="E160" t="str">
         <v>Desarrollo</v>
@@ -3133,16 +3133,16 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C161" t="str">
-        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
+        <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
       </c>
       <c r="D161" t="str">
-        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
+        <v>Cuando hay transacciones divididas (ej. ingreso 30k ejecutada + 20k pendiente), el sync no debe duplicar el Cobro nominal: si ya se agregó una fila Cobro con monto = mr (50.000), no se agrega otra para la segunda transacción del mismo leg. Así al cerrar una de las dos divididas el modelo responde bien (un Cobro 50.000, saldo coherente).</v>
       </c>
       <c r="E161" t="str">
         <v>Desarrollo</v>
@@ -3150,16 +3150,16 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C162" t="str">
-        <v>Reversar a pendiente: solo una vez por transacción</v>
+        <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
       </c>
       <c r="D162" t="str">
-        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
+        <v>El acuerdo es "cliente entrega cheques por 50.000": una transacción, no dos. Se deja de crear "Ganancia del acuerdo" y de reducir el ingreso a 48.750. La comisión se trata en CC desde los datos del acuerdo (Cobro +50.000, Comisión Pandy -1.250), como en CC intermediario. Quitados debeDividir (cambiarEstadoTransaccion), asegurarGananciaPandy y revertirGananciaPandy en flujos de ejecutada/pendiente. Sync: Cobro nominal (mr) cuando el acuerdo tiene comisión (comisionPandyOrden &gt;= 1e-6), no solo si existe transacción Ganancia.</v>
       </c>
       <c r="E162" t="str">
         <v>Desarrollo</v>
@@ -3167,16 +3167,16 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C163" t="str">
-        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
+        <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
       </c>
       <c r="D163" t="str">
-        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
+        <v>Al pasar a ejecutada la entrega Pandy→intermediario (cheques) la CC intermediario debe mostrar +49.250 (intermediario nos debe). Se agrega segunda fila +49.250 "Intermediario debe a Pandy" cuando el egreso está ejecutada (cuantasQueremos=2); al ejecutar el ingreso Int→Pandy se inserta -49.250 "Pago Intermediario a Pandy" para cerrar en 0. Estado de las filas +49.250: cerrado cuando egreso o ingreso ejecutada, pendiente si no.</v>
       </c>
       <c r="E163" t="str">
         <v>Desarrollo</v>
@@ -3184,16 +3184,16 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C164" t="str">
-        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
+        <v>Reversar a pendiente: solo una vez por transacción</v>
       </c>
       <c r="D164" t="str">
-        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
+        <v>Columna transacciones.revertida_una_vez (boolean). Al intentar reversar por segunda vez (ejecutada→pendiente) se muestra modal empático: "No se puede reversar de nuevo", mensaje claro y botones "Anular orden" (abre la orden para anular) y "Entendido". showConfirm acepta textoCancelar y tituloModal opcionales. sql/migracion_transaccion_revertida_una_vez.sql.</v>
       </c>
       <c r="E164" t="str">
         <v>Desarrollo</v>
@@ -3201,16 +3201,16 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C165" t="str">
-        <v>Número de transacción interno y convención movimientos de caja</v>
+        <v>Test E2E orden ARS-ARS y cuenta corriente</v>
       </c>
       <c r="D165" t="str">
-        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
+        <v>Nuevo archivo tests/e2e/orden-cc.spec.js: flujo completo crear orden ARS-ARS (tipo, cliente, importe cheque + tasa), ir a instrumentación, ejecutar las dos transacciones y verificar que la cuenta corriente refleja cada paso (cliente con saldo ARS tras primera ejecutada; tras segunda, saldo coherente). Guía docs/TESTING_E2E_GUIA.md actualizada con requisitos (tipo ARS-ARS activo, al menos un cliente, permisos).</v>
       </c>
       <c r="E165" t="str">
         <v>Desarrollo</v>
@@ -3218,16 +3218,16 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C166" t="str">
-        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
+        <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
       </c>
       <c r="D166" t="str">
-        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+        <v>En tests ARS-ARS, ARS-USD y USD-ARS se añade paso 6 Control de caja: abrir Cajas, comprobar vista y #cajas-saldos visible; en el log Excel se registra resultado esperado (Vista Cajas visible y saldos cargados) y estado OK o Fallo; si falla la comprobación el test falla y en Observaciones queda el error.</v>
       </c>
       <c r="E166" t="str">
         <v>Desarrollo</v>
@@ -3235,16 +3235,16 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C167" t="str">
-        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
+        <v>Número de transacción interno y convención movimientos de caja</v>
       </c>
       <c r="D167" t="str">
-        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
+        <v>Columna transacciones.numero (secuencia) para trazabilidad. Concepto de movimientos de caja por transacción: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Helpers conceptoCajaTransaccion y conceptoCajaTransaccionEspecial; todos los inserts de movimientos_caja con transaccion_id usan la convención. Panel de transacciones muestra columna Nro. SQL: sql/migracion_transacciones_numero.sql; truncate resetea transacciones_numero_seq.</v>
       </c>
       <c r="E167" t="str">
         <v>Desarrollo</v>
@@ -3252,16 +3252,16 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C168" t="str">
-        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
+        <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
       </c>
       <c r="D168" t="str">
-        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
+        <v>Log E2E: nueva hoja Caja con columnas por moneda y tipo (Efectivo/Banco): Saldo_Caja_*_Esp, Saldo_Caja_*_App, Resultado_Caja_* (OK/err). logCajaControl() en e2e-log-excel.js; tests llaman con saldos capturados. Movimientos de caja: migración orden_numero y transaccion_numero en movimientos_caja; todos los inserts rellenan estos campos; vista Cajas con columnas Fecha, Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Moneda, Monto, Caja, Concepto, Acciones. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
       </c>
       <c r="E168" t="str">
         <v>Desarrollo</v>
@@ -3269,16 +3269,16 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C169" t="str">
-        <v>Tipos de operación: Intermediario Sí/No</v>
+        <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
       </c>
       <c r="D169" t="str">
-        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
+        <v>Helper irACajasYLeerSaldos: va a Cajas, espera #cajas-loading hidden (20s) y lee saldos para que no queden –. En cada test se llama logCajaControl tras cada transacción ejecutada (una fila por paso) y una fila final. Hoja Caja en Excel: múltiples filas mostrando cómo se mueve la caja. Fix SheetNames para que la hoja Caja se persista al actualizar Excel existente.</v>
       </c>
       <c r="E169" t="str">
         <v>Desarrollo</v>
@@ -3286,16 +3286,16 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C170" t="str">
-        <v>Número de orden MAX+1 atómico en DB</v>
+        <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
       </c>
       <c r="D170" t="str">
-        <v>Función ordenes_insertar_con_proximo_numero en Supabase: asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones. La app llama a la RPC al crear orden nueva (wizard, saveOrden, chat); fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+        <v>En sincronizarCcYCajaDesdeOrden, cuando hay comisión Pandy (mr &gt; me, misma moneda), no hay transacción Ganancia y el ingreso cliente→Pandy está ejecutado, se agrega un movimiento de caja: ingreso efectivo por el monto de la comisión (transaccion_id null). Al re-sincronizar se borran movimientos de caja de la orden con transaccion_id null para no duplicar. Así la caja cierra en cero en operaciones de cobro de cheques.</v>
       </c>
       <c r="E170" t="str">
         <v>Desarrollo</v>
@@ -3303,101 +3303,101 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C171" t="str">
-        <v>v1.33 Despliegue</v>
+        <v>Tipos de operación: Intermediario Sí/No</v>
       </c>
       <c r="D171" t="str">
-        <v>CC ARS-ARS con intermediario: momento cero cliente (Compromiso -mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía TEST_BASE_URL cuando Vite usa otro puerto.</v>
+        <v>Columna usa_intermediario en tipos_operacion (migración sql). ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox Usa intermediario en modal. Modal de orden: si el tipo no usa intermediario se oculta el selector de intermediario y no se menciona; al guardar se fuerza intermediario_id = null. Tasa descuento intermediario y split comisión solo visibles cuando el tipo usa intermediario.</v>
       </c>
       <c r="E171" t="str">
-        <v>Despliegue</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C172" t="str">
-        <v>v1.34 Despliegue</v>
+        <v>Número de orden MAX+1 atómico en DB</v>
       </c>
       <c r="D172" t="str">
-        <v>CC regla simple: compromisos solo si al menos una transacción ejecutada; ambas pendientes → saldo 0.</v>
+        <v>Función ordenes_insertar_con_proximo_numero en Supabase: asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones. La app llama a la RPC al crear orden nueva (wizard, saveOrden, chat); fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
       <c r="E172" t="str">
-        <v>Despliegue</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C173" t="str">
-        <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
+        <v>v1.33 Despliegue</v>
       </c>
       <c r="D173" t="str">
-        <v>utils.js en raíz: formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda; main.js importa desde ./utils.js. RPC sync_cc_caja_orden en Supabase: front construye rows y llama RPC para delete+insert atómico; fallback a delete+insert en cliente si RPC no existe. sql/rpc_sync_cc_caja_orden.sql. Doc docs/FUNCIONES_CRITICAS_SUPABASE_VS_FRONT.md actualizado.</v>
+        <v>CC ARS-ARS con intermediario: momento cero cliente (Compromiso -mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía TEST_BASE_URL cuando Vite usa otro puerto.</v>
       </c>
       <c r="E173" t="str">
-        <v>Desarrollo</v>
+        <v>Despliegue</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C174" t="str">
-        <v>RPC transacciones_cambiar_estado</v>
+        <v>v1.34 Despliegue</v>
       </c>
       <c r="D174" t="str">
-        <v>Función PostgreSQL transacciones_cambiar_estado(p_transaccion_id, p_estado, p_fecha_ejecucion, p_usuario_id, p_revertida_una_vez). El front llama la RPC al cambiar pendiente↔ejecutada; si la RPC no existe usa UPDATE directo. sql/rpc_transacciones_cambiar_estado.sql. Sin Edge Functions: solo RPC (funciones en la DB).</v>
+        <v>CC regla simple: compromisos solo si al menos una transacción ejecutada; ambas pendientes → saldo 0.</v>
       </c>
       <c r="E174" t="str">
-        <v>Desarrollo</v>
+        <v>Despliegue</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C175" t="str">
-        <v>v1.35 Despliegue</v>
+        <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
       </c>
       <c r="D175" t="str">
-        <v>Regla de estilos de botones LyP: mismo estilo en toda la app; con leyenda icono a la izquierda; solo icono mismo estilo. Regla .cursor/rules/estilos-botones.mdc en Pandi y replicada en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
+        <v>utils.js en raíz: formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda; main.js importa desde ./utils.js. RPC sync_cc_caja_orden en Supabase: front construye rows y llama RPC para delete+insert atómico; fallback a delete+insert en cliente si RPC no existe. sql/rpc_sync_cc_caja_orden.sql. Doc docs/FUNCIONES_CRITICAS_SUPABASE_VS_FRONT.md actualizado.</v>
       </c>
       <c r="E175" t="str">
-        <v>Despliegue</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C176" t="str">
-        <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
+        <v>RPC transacciones_cambiar_estado</v>
       </c>
       <c r="D176" t="str">
-        <v>Vista Detalle de movimientos: se quitó el filtro Tipo "Todos"; solo Cliente e Intermediario. Columna Originante siempre visible: encabezado "Cliente" o "Intermediario" según el filtro y en cada fila el nombre del originante del movimiento. Export Excel incluye esa columna con el mismo criterio.</v>
+        <v>Función PostgreSQL transacciones_cambiar_estado(p_transaccion_id, p_estado, p_fecha_ejecucion, p_usuario_id, p_revertida_una_vez). El front llama la RPC al cambiar pendiente↔ejecutada; si la RPC no existe usa UPDATE directo. sql/rpc_transacciones_cambiar_estado.sql. Sin Edge Functions: solo RPC (funciones en la DB).</v>
       </c>
       <c r="E176" t="str">
         <v>Desarrollo</v>
@@ -3405,50 +3405,50 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C177" t="str">
-        <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
+        <v>v1.35 Despliegue</v>
       </c>
       <c r="D177" t="str">
-        <v>Originante en cada movimiento = Pagador de la transacción (nombre resuelto desde cliente/intermediario/Pandy). Leyendas concepto unificadas: Pago Realizado - Orden x y Trans x, Cobro Realizado - Orden x y Trans x, Compromiso de Pago - Orden x y Trans x, Compromiso a Cobrar - Orden x y Trans x. Vista Detalle: columnas Orden y Trans. (sin "Nro"); columnas Cliente/Intermediario y Originante. Helper conceptoCcLeyenda; sync e insertar momento cero usan nuevas leyendas.</v>
+        <v>Regla de estilos de botones LyP: mismo estilo en toda la app; con leyenda icono a la izquierda; solo icono mismo estilo. Regla .cursor/rules/estilos-botones.mdc en Pandi y replicada en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
       </c>
       <c r="E177" t="str">
-        <v>Desarrollo</v>
+        <v>Despliegue</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C178" t="str">
-        <v>v1.36 Despliegue</v>
+        <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
       </c>
       <c r="D178" t="str">
-        <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. bitacora-tareas.mdc y reglas-pandi.mdc actualizados con revisión RPC y adaptación de tests obligatorias.</v>
+        <v>Vista Detalle de movimientos: se quitó el filtro Tipo "Todos"; solo Cliente e Intermediario. Columna Originante siempre visible: encabezado "Cliente" o "Intermediario" según el filtro y en cada fila el nombre del originante del movimiento. Export Excel incluye esa columna con el mismo criterio.</v>
       </c>
       <c r="E178" t="str">
-        <v>Despliegue</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C179" t="str">
-        <v>CC: unificación de conceptos y transaccion_numero</v>
+        <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
       </c>
       <c r="D179" t="str">
-        <v>Conceptos CC intermediario y derivados unificados con conceptoCcLeyenda: Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo (tipo comision_acuerdo), siempre con " - Orden x y Trans x". transaccion_numero en todos los rows/inserts de CC (cliente e intermediario). asegurarComisionIntermediario con parámetro ordenNumero; filtros de reversa actualizados a "Compromiso a Cobrar". Doc REVISION_CC_INTERMEDIARIO_CONCEPTOS_Y_NRO_TRANS.md §4.</v>
+        <v>Originante en cada movimiento = Pagador de la transacción (nombre resuelto desde cliente/intermediario/Pandy). Leyendas concepto unificadas: Pago Realizado - Orden x y Trans x, Cobro Realizado - Orden x y Trans x, Compromiso de Pago - Orden x y Trans x, Compromiso a Cobrar - Orden x y Trans x. Vista Detalle: columnas Orden y Trans. (sin "Nro"); columnas Cliente/Intermediario y Originante. Helper conceptoCcLeyenda; sync e insertar momento cero usan nuevas leyendas.</v>
       </c>
       <c r="E179" t="str">
         <v>Desarrollo</v>
@@ -3456,33 +3456,33 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C180" t="str">
-        <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
+        <v>v1.36 Despliegue</v>
       </c>
       <c r="D180" t="str">
-        <v>Eliminado duplicado: una sola fila "Compromiso a Cobrar" por transacción (cuantasQueremos = 1). Doc FLUJOS_CC_REGLA.md: sección Revisión de impacto (RCA) y Objetivo actuar por transacción (no borrar/repoblar toda la orden). Regla en reglas-pandi.mdc: revisión de impacto RCA y regla por transacción (movimientos ligados a transacción; no depender de sync completo).</v>
+        <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. bitacora-tareas.mdc y reglas-pandi.mdc actualizados con revisión RPC y adaptación de tests obligatorias.</v>
       </c>
       <c r="E180" t="str">
-        <v>Desarrollo</v>
+        <v>Despliegue</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C181" t="str">
-        <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
+        <v>CC: unificación de conceptos y transaccion_numero</v>
       </c>
       <c r="D181" t="str">
-        <v>loadCuentaCorriente: solo lee mov_cc y mov_cc_int (sin sync previo). guardarSoloMontoTransaccion y hacerCierre: sin llamar a sincronizarCcYCajaDesdeOrden. autoCompletarInstrumentacionChequeConIntermediario: inserta momento cero (insertarMovimientosCcMomentoCero e Intermediario) en lugar de sync. cambiarEstadoTransaccion: actualizarEstadoSinSync (solo actualizarEstadoOrden). saveTransaccion revert: revertirCcYCajaPorTransaccion (borrar/actualizar solo movimientos de esa transacción) en lugar de sync. Base siempre bien relacionada; eficiente con alto volumen.</v>
+        <v>Conceptos CC intermediario y derivados unificados con conceptoCcLeyenda: Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo (tipo comision_acuerdo), siempre con " - Orden x y Trans x". transaccion_numero en todos los rows/inserts de CC (cliente e intermediario). asegurarComisionIntermediario con parámetro ordenNumero; filtros de reversa actualizados a "Compromiso a Cobrar". Doc REVISION_CC_INTERMEDIARIO_CONCEPTOS_Y_NRO_TRANS.md §4.</v>
       </c>
       <c r="E181" t="str">
         <v>Desarrollo</v>
@@ -3490,16 +3490,16 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C182" t="str">
-        <v>CC detalle movimientos: columna Tipo de operación</v>
+        <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
       </c>
       <c r="D182" t="str">
-        <v>En el modal Detalle de movimientos (cliente/intermediario) se agrega la columna Tipo op. con el código del tipo de operación de la orden (tipos_operacion.codigo). fetchMovimientosCcPorEntidad incluye tipo_operacion_id y tipos_operacion(codigo) en el select de órdenes; se enriquece cada movimiento con tipo_operacion; ordenamiento por esa columna. Trazabilidad visual completa (Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado).</v>
+        <v>Eliminado duplicado: una sola fila "Compromiso a Cobrar" por transacción (cuantasQueremos = 1). Doc FLUJOS_CC_REGLA.md: sección Revisión de impacto (RCA) y Objetivo actuar por transacción (no borrar/repoblar toda la orden). Regla en reglas-pandi.mdc: revisión de impacto RCA y regla por transacción (movimientos ligados a transacción; no depender de sync completo).</v>
       </c>
       <c r="E182" t="str">
         <v>Desarrollo</v>
@@ -3507,16 +3507,16 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C183" t="str">
-        <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
+        <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
       </c>
       <c r="D183" t="str">
-        <v>Tipo de operación visible en vista Detalle (página), modal detalle y export. Orden de columnas: Fecha, Tipo op., Orden, Trans., Concepto, … Columnas Fecha y Tipo op. ancladas en scroll horizontal (sticky left) en modal y vista detalle. loadCuentaCorriente carga tipos_operacion(codigo) en órdenes; buildCcResumenRows agrega tipo_operacion a detalleList. Export Excel incluye columna Tipo op. tras Fecha.</v>
+        <v>loadCuentaCorriente: solo lee mov_cc y mov_cc_int (sin sync previo). guardarSoloMontoTransaccion y hacerCierre: sin llamar a sincronizarCcYCajaDesdeOrden. autoCompletarInstrumentacionChequeConIntermediario: inserta momento cero (insertarMovimientosCcMomentoCero e Intermediario) en lugar de sync. cambiarEstadoTransaccion: actualizarEstadoSinSync (solo actualizarEstadoOrden). saveTransaccion revert: revertirCcYCajaPorTransaccion (borrar/actualizar solo movimientos de esa transacción) en lugar de sync. Base siempre bien relacionada; eficiente con alto volumen.</v>
       </c>
       <c r="E183" t="str">
         <v>Desarrollo</v>
@@ -3524,16 +3524,16 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C184" t="str">
-        <v>Modales: no cerrar al elegir opción de menú/select</v>
+        <v>CC detalle movimientos: columna Tipo de operación</v>
       </c>
       <c r="D184" t="str">
-        <v>Al abrir un desplegable (select o menú) y mover el mouse para elegir, el click a veces se reportaba en el backdrop y cerraba el modal. Helper setupBackdropCloseOnlyOnRealClick: solo cerrar si tanto mousedown como click fueron sobre el backdrop. Aplicado a todos los modales (órdenes, transacciones, CC, cliente, intermediario, tipo op., confirm, help, etc.).</v>
+        <v>En el modal Detalle de movimientos (cliente/intermediario) se agrega la columna Tipo op. con el código del tipo de operación de la orden (tipos_operacion.codigo). fetchMovimientosCcPorEntidad incluye tipo_operacion_id y tipos_operacion(codigo) en el select de órdenes; se enriquece cada movimiento con tipo_operacion; ordenamiento por esa columna. Trazabilidad visual completa (Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado).</v>
       </c>
       <c r="E184" t="str">
         <v>Desarrollo</v>
@@ -3541,16 +3541,16 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C185" t="str">
-        <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
+        <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
       </c>
       <c r="D185" t="str">
-        <v>El cierre por inactividad se disparaba al solo mover el mouse o el trackpad (sin clic) porque mousemove no actualizaba lastActivityTime. Se agregó mousemove a los eventos que llaman a updateSessionActivity (throttle 30 s); así mover el cursor mantiene la sesión viva y no se cierra la app al abrir un menú.</v>
+        <v>Tipo de operación visible en vista Detalle (página), modal detalle y export. Orden de columnas: Fecha, Tipo op., Orden, Trans., Concepto, … Columnas Fecha y Tipo op. ancladas en scroll horizontal (sticky left) en modal y vista detalle. loadCuentaCorriente carga tipos_operacion(codigo) en órdenes; buildCcResumenRows agrega tipo_operacion a detalleList. Export Excel incluye columna Tipo op. tras Fecha.</v>
       </c>
       <c r="E185" t="str">
         <v>Desarrollo</v>
@@ -3558,33 +3558,33 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C186" t="str">
-        <v>Despliegue v1.38</v>
+        <v>Modales: no cerrar al elegir opción de menú/select</v>
       </c>
       <c r="D186" t="str">
-        <v>Producción Vercel: XLSX desde CDN en index.html y main.js usa window.XLSX para que funcione sin bundler (fix "Failed to resolve module specifier xlsx").</v>
+        <v>Al abrir un desplegable (select o menú) y mover el mouse para elegir, el click a veces se reportaba en el backdrop y cerraba el modal. Helper setupBackdropCloseOnlyOnRealClick: solo cerrar si tanto mousedown como click fueron sobre el backdrop. Aplicado a todos los modales (órdenes, transacciones, CC, cliente, intermediario, tipo op., confirm, help, etc.).</v>
       </c>
       <c r="E186" t="str">
-        <v>Despliegue</v>
+        <v>Desarrollo</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C187" t="str">
-        <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
+        <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
       </c>
       <c r="D187" t="str">
-        <v>Tras cambiar transacción a "ejecutada" en el wizard, el test cerraba el modal y navegaba a Cuenta corriente antes de que el backend terminara; la transacción no se persistía y los asserts fallaban. Se agregó esperarActualizacionEstadoOrden(page): espera a que #orden-inst-actualizando-msg desaparezca (hasta 35 s) en los cuatro flujos (ARS-ARS, ARS-USD, USD-ARS, USD-USD).</v>
+        <v>El cierre por inactividad se disparaba al solo mover el mouse o el trackpad (sin clic) porque mousemove no actualizaba lastActivityTime. Se agregó mousemove a los eventos que llaman a updateSessionActivity (throttle 30 s); así mover el cursor mantiene la sesión viva y no se cierra la app al abrir un menú.</v>
       </c>
       <c r="E187" t="str">
         <v>Desarrollo</v>
@@ -3592,33 +3592,33 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C188" t="str">
-        <v>CC intermediario: estado pendiente en momento cero</v>
+        <v>Despliegue v1.38</v>
       </c>
       <c r="D188" t="str">
-        <v>En ARS-ARS con intermediario, insertarMovimientosCcMomentoCeroIntermediario no guardaba estado en las filas Debe/Compensación; si la tabla tiene estado NULL, el UPDATE en cambiarEstadoTransaccion (.eq(estado, pendiente)) no coincidía y la fila no se cerraba, dejando la CC del intermediario en cero tras ejecutar la 3.ª transacción. Se agrega estado: "pendiente" en ambas filas al insertar.</v>
+        <v>Producción Vercel: XLSX desde CDN en index.html y main.js usa window.XLSX para que funcione sin bundler (fix "Failed to resolve module specifier xlsx").</v>
       </c>
       <c r="E188" t="str">
-        <v>Desarrollo</v>
+        <v>Despliegue</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C189" t="str">
-        <v>Regla simple e infalible CC y caja</v>
+        <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
       </c>
       <c r="D189" t="str">
-        <v>Docs REGLA_CC_SIMPLE_INFALIBLE.md y actualización FLUJOS_CC_REGLA.md. Solo transacciones ejecutadas generan movimientos; signo por pagador/cobrador (pagador entidad → +monto, cobrador entidad → -monto); caja Pandy cobra + / paga -. Sin momento cero: no se insertan movimientos al crear la instrumentación; sync (sincronizarCcYCajaDesdeOrden) construye rows solo desde transacciones ejecutadas. cambiarEstadoTransaccion: tras RPC, reversas de ganancia/comisión si aplica y siempre sincronizarCcYCajaDesdeOrden(ordenId). App, tests y RPC alineados a la misma regla.</v>
+        <v>Tras cambiar transacción a "ejecutada" en el wizard, el test cerraba el modal y navegaba a Cuenta corriente antes de que el backend terminara; la transacción no se persistía y los asserts fallaban. Se agregó esperarActualizacionEstadoOrden(page): espera a que #orden-inst-actualizando-msg desaparezca (hasta 35 s) en los cuatro flujos (ARS-ARS, ARS-USD, USD-ARS, USD-USD).</v>
       </c>
       <c r="E189" t="str">
         <v>Desarrollo</v>
@@ -3626,16 +3626,16 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C190" t="str">
-        <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
+        <v>CC intermediario: estado pendiente en momento cero</v>
       </c>
       <c r="D190" t="str">
-        <v>En órdenes ARS-USD/USD-ARS el saldo debe cerrar en 0 tras ejecutar ambas transacciones. RPC sync_cc_caja_orden: COALESCE((r-&gt;&gt;'monto_usd')::numeric, 0) (y monto_ars, monto_eur) en inserts CC cliente e intermediario para no guardar NULL. Front: en sincronizarCcYCajaDesdeOrden los rows CC cliente llevan monto_usd, monto_ars, monto_eur explícitos con numCc(montos.*) en lugar de ...montos. sql/rpc_sync_cc_caja_orden.sql y main.js.</v>
+        <v>En ARS-ARS con intermediario, insertarMovimientosCcMomentoCeroIntermediario no guardaba estado en las filas Debe/Compensación; si la tabla tiene estado NULL, el UPDATE en cambiarEstadoTransaccion (.eq(estado, pendiente)) no coincidía y la fila no se cerraba, dejando la CC del intermediario en cero tras ejecutar la 3.ª transacción. Se agrega estado: "pendiente" en ambas filas al insertar.</v>
       </c>
       <c r="E190" t="str">
         <v>Desarrollo</v>
@@ -3643,16 +3643,16 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C191" t="str">
-        <v>CC: un movimiento = una moneda (la de la transacción)</v>
+        <v>Regla simple e infalible CC y caja</v>
       </c>
       <c r="D191" t="str">
-        <v>No puede haber valor en más de una moneda por movimiento. Sync: se usa montosCcPorMoneda(mon, monto) en lugar de montosCcPorOrden en todos los flujos (sincronizarCcYCajaDesdeOrden, insertarMovimientosCcParaTransaccion y fallbacks). Vista Detalle de movimientos: se muestra solo la columna de la moneda del movimiento (m.moneda); las demás "–". Aplica a vista principal y modal detalle.</v>
+        <v>Docs REGLA_CC_SIMPLE_INFALIBLE.md y actualización FLUJOS_CC_REGLA.md. Solo transacciones ejecutadas generan movimientos; signo por pagador/cobrador (pagador entidad → +monto, cobrador entidad → -monto); caja Pandy cobra + / paga -. Sin momento cero: no se insertan movimientos al crear la instrumentación; sync (sincronizarCcYCajaDesdeOrden) construye rows solo desde transacciones ejecutadas. cambiarEstadoTransaccion: tras RPC, reversas de ganancia/comisión si aplica y siempre sincronizarCcYCajaDesdeOrden(ordenId). App, tests y RPC alineados a la misma regla.</v>
       </c>
       <c r="E191" t="str">
         <v>Desarrollo</v>
@@ -3660,16 +3660,16 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C192" t="str">
-        <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
+        <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
       </c>
       <c r="D192" t="str">
-        <v>Por misma orden no puede haber resumen de CC con saldo en más de una moneda. Para órdenes en dos monedas (ARS-USD, USD-ARS) sin intermediario: cuando ingreso Cliente→Pandy y egreso Pandy→Cliente están ejecutados, se añaden dos movimientos de cierre en sync (concepto "Cierre orden N"): -monto recibido en monR y +monto entregado en monE. Así el saldo del cliente para esa orden queda 0 en cada moneda. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+        <v>En órdenes ARS-USD/USD-ARS el saldo debe cerrar en 0 tras ejecutar ambas transacciones. RPC sync_cc_caja_orden: COALESCE((r-&gt;&gt;'monto_usd')::numeric, 0) (y monto_ars, monto_eur) en inserts CC cliente e intermediario para no guardar NULL. Front: en sincronizarCcYCajaDesdeOrden los rows CC cliente llevan monto_usd, monto_ars, monto_eur explícitos con numCc(montos.*) en lugar de ...montos. sql/rpc_sync_cc_caja_orden.sql y main.js.</v>
       </c>
       <c r="E192" t="str">
         <v>Desarrollo</v>
@@ -3677,16 +3677,16 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C193" t="str">
-        <v>Regla CC: 4 premisas clave documentadas</v>
+        <v>CC: un movimiento = una moneda (la de la transacción)</v>
       </c>
       <c r="D193" t="str">
-        <v>Doc REGLA_CC_SIMPLE_INFALIBLE.md reordenado con las 4 premisas como base: (1) Siempre pagador y cobrador; (2) Siempre una única moneda; (3) Estado Pendiente o Ejecutada, solo Ejecutada genera movimientos; (4) Comisión implícita se administra según estado. Secciones del doc referencian cada premisa.</v>
+        <v>No puede haber valor en más de una moneda por movimiento. Sync: se usa montosCcPorMoneda(mon, monto) en lugar de montosCcPorOrden en todos los flujos (sincronizarCcYCajaDesdeOrden, insertarMovimientosCcParaTransaccion y fallbacks). Vista Detalle de movimientos: se muestra solo la columna de la moneda del movimiento (m.moneda); las demás "–". Aplica a vista principal y modal detalle.</v>
       </c>
       <c r="E193" t="str">
         <v>Desarrollo</v>
@@ -3694,16 +3694,16 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C194" t="str">
-        <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
+        <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
       </c>
       <c r="D194" t="str">
-        <v>Cliente pagó → movimiento -monto (saldo negativo = Pandy debe entregar). Pandy pagó al cliente → +monto. Así una sola transacción ejecutada (cliente pagó 3700) muestra -3700 (Pandy debe), no +3700. Ajustados sync, cierre dos monedas, ganancia Pandy e insertarMovimientosCcParaTransaccion. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+        <v>Por misma orden no puede haber resumen de CC con saldo en más de una moneda. Para órdenes en dos monedas (ARS-USD, USD-ARS) sin intermediario: cuando ingreso Cliente→Pandy y egreso Pandy→Cliente están ejecutados, se añaden dos movimientos de cierre en sync (concepto "Cierre orden N"): -monto recibido en monR y +monto entregado en monE. Así el saldo del cliente para esa orden queda 0 en cada moneda. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
       </c>
       <c r="E194" t="str">
         <v>Desarrollo</v>
@@ -3711,24 +3711,92 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>22:57</v>
+        <v>00:55</v>
       </c>
       <c r="C195" t="str">
+        <v>Regla CC: 4 premisas clave documentadas</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Doc REGLA_CC_SIMPLE_INFALIBLE.md reordenado con las 4 premisas como base: (1) Siempre pagador y cobrador; (2) Siempre una única moneda; (3) Estado Pendiente o Ejecutada, solo Ejecutada genera movimientos; (4) Comisión implícita se administra según estado. Secciones del doc referencian cada premisa.</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B196" t="str">
+        <v>00:55</v>
+      </c>
+      <c r="C196" t="str">
+        <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Cliente pagó → movimiento -monto (saldo negativo = Pandy debe entregar). Pandy pagó al cliente → +monto. Así una sola transacción ejecutada (cliente pagó 3700) muestra -3700 (Pandy debe), no +3700. Ajustados sync, cierre dos monedas, ganancia Pandy e insertarMovimientosCcParaTransaccion. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B197" t="str">
+        <v>00:55</v>
+      </c>
+      <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
       </c>
-      <c r="D195" t="str">
+      <c r="D197" t="str">
         <v>Cuando solo el egreso está ejecutada (Pandy pagó me) y el ingreso Cliente→Pandy está pendiente, el resumen debe mostrar lo que el cliente debe (mr), no me. En sync: egreso misma moneda con ingreso pendiente → movimiento +mr en CC cliente. Así ALFIE con ingreso 4933 pendiente y egreso 4849,14 ejecutada muestra "cliente debe 4933". Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
       </c>
-      <c r="E195" t="str">
+      <c r="E197" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B198" t="str">
+        <v>00:55</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Validación egreso cheques</v>
+      </c>
+      <c r="D198" t="str">
+        <v>No permitir marcar ejecutada la entrega de cheque (Pandy→Intermediario) si el ingreso del cheque (Cliente→Pandy) sigue pendiente. Validación en cambiarEstadoTransaccion; combo de estado con opción Ejecutada deshabilitada y tooltip en tabla de transacciones (expand y refresh).</v>
+      </c>
+      <c r="E198" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B199" t="str">
+        <v>00:55</v>
+      </c>
+      <c r="C199" t="str">
+        <v>CC resumen: color a favor / en contra de Pandy</v>
+      </c>
+      <c r="D199" t="str">
+        <v>Regla conceptual unificada para cliente e intermediario: verde = a favor de Pandy, rojo = en contra. Intermediario: se invierte el signo solo para el color (saldo en DB negativo = Pandy entregó = claim a favor = verde). Cliente: saldo en DB ya coincide (positivo = a Pandy le deben = verde).</v>
+      </c>
+      <c r="E199" t="str">
         <v>Desarrollo</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E195"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E199"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4229,7 +4297,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4252,7 +4320,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -4263,7 +4331,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -4274,7 +4342,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -4285,7 +4353,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -4296,7 +4364,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -4307,7 +4375,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -4318,7 +4386,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -4329,7 +4397,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -4340,7 +4408,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -4351,7 +4419,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -4362,7 +4430,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -4373,7 +4441,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -4384,7 +4452,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -4395,7 +4463,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -4406,7 +4474,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -4417,7 +4485,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -4428,7 +4496,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -4439,7 +4507,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -4450,7 +4518,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -4461,7 +4529,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -4472,7 +4540,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -4483,7 +4551,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -4494,7 +4562,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -4505,7 +4573,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -4516,7 +4584,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -4527,7 +4595,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -4538,7 +4606,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -4549,7 +4617,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -4560,7 +4628,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
@@ -4571,7 +4639,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
@@ -4582,7 +4650,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
@@ -4593,7 +4661,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
@@ -4604,7 +4672,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Switch Activo en tablas Clientes e Intermediarios; modales Cliente/Intermediario con toggle; centrado de botón y título en todas las pantallas con switch. Script truncar: orden correcto y orden_comisiones_generadas opcional. Tests E2E: intermediario solo si visible (tipos sin intermediario).</v>
@@ -4615,7 +4683,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>CC ARS-ARS con intermediario: momento cero cliente (-mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía testing con TEST_BASE_URL cuando Vite usa otro puerto.</v>
@@ -4626,7 +4694,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C36" t="str">
         <v>CC regla simple (USD-USD, 2 transacciones): compromisos solo cuando al menos una transacción está ejecutada; si ambas pendientes, saldo 0 (no figura deuda).</v>
@@ -4637,7 +4705,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Regla de estilos de botones LyP: mismo estilo (border-radius 8px, min-height); con leyenda = icono a la izquierda; solo icono mismo estilo; botón Excel verde. Regla estilos-botones.mdc en Pandi y en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
@@ -4648,7 +4716,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. Al completar tareas hay que actualizar bitácora, revisar RPC en sql/ si aplica y adaptar tests si afectan. bitacora-tareas.mdc y reglas-pandi.mdc.</v>
@@ -4659,7 +4727,7 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Modales: no cerrar al elegir en select (mousedown+click en backdrop). Sesión: mousemove cuenta como actividad para no cerrar por inactividad al mover mouse/trackpad. CC: Tipo op. después de Fecha, sticky y export Excel.</v>
@@ -4670,7 +4738,7 @@
         <v>1.38</v>
       </c>
       <c r="B40" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C40" t="str">
         <v>Producción Vercel: XLSX cargado desde CDN (script en index.html); main.js usa window.XLSX para evitar error "Failed to resolve module specifier xlsx" sin bundler.</v>
@@ -4681,15 +4749,26 @@
         <v>1.39</v>
       </c>
       <c r="B41" t="str">
-        <v>16/03/2026</v>
+        <v>17/03/2026</v>
       </c>
       <c r="C41" t="str">
         <v>CC regla infalible: ingreso misma moneda aporta -me (Pandy debe su transacción); egreso con ingreso pendiente aporta +mr (resumen muestra deuda del cliente). Sin movimiento extra ganancia Pandy en CC. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>1.40</v>
+      </c>
+      <c r="B42" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Validación egreso cheques: no ejecutar entrega al intermediario si ingreso Cliente→Pandy pendiente. CC resumen: color unificado (verde = a favor de Pandy, rojo = en contra) para cliente e intermediario.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.40: bitácora regenerada con Log y Versiones
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -433,7 +433,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>00:55</v>
+        <v>00:58</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>

</xml_diff>

<commit_message>
v1.41: CC modelo reglas (16 combinaciones), Tx1 SUMA_SALDO Y, comisiones pendientes, Compromiso 195k
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E199"/>
+  <dimension ref="A1:E206"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>00:58</v>
+        <v>15:36</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3794,9 +3794,128 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B200" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Tabla cc_modelo_reglas en Supabase</v>
+      </c>
+      <c r="D200" t="str">
+        <v>Tabla con todas las combinaciones del modelo CC: tipo_operacion_codigo, usa_intermediario, pagador, cobrador, tipo_transaccion, es_comision, estado_transaccion (pendiente/ejecutada), contrapartida_ejecutada, signos y flags (suma saldo, incluir en mov). 4 filas por tipo de transacción (ejecutada/pendiente × contrapartida sí/no). sql/cc_modelo_reglas_tabla.sql y migracion_cc_modelo_reglas_estado_transaccion.sql; docs/CC_MODELO_TABLA_REGLAS.md.</v>
+      </c>
+      <c r="E200" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B201" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C201" t="str">
+        <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Si Tx3 y Tx4 están ambas pendientes, ninguna transacción suma a saldo → detalle CC intermediario debe estar vacío y saldo 0. La comisión del acuerdo (-3.000) solo se incluye en el detalle cuando al menos una de Tx3 (egreso Pandy→Int) o Tx4 (ingreso Int→Pandy) está ejecutada. sincronizarCcYCajaDesdeOrden condiciona el push de la comisión a hayTx3Ejecutada || hayTx4Ejecutada. Doc CC_MODELO_REFERENCIA.md actualizado.</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B202" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Motor CC desde tabla cc_modelo_reglas</v>
+      </c>
+      <c r="D202" t="str">
+        <v>Sync CC consume la tabla: getReglasCcModelo(codigo, usa_intermediario). Si hay reglas, construye movimientos solo desde lookupRegla (transacciones + comisiones con condicion_estado_comision). Sin reglas → fallback ARS-ARS. Indiferente al tipo de operación. sql/migracion_cc_modelo_reglas_condicion_comision.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B203" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Reglas CC para todos los tipos activos</v>
+      </c>
+      <c r="D203" t="str">
+        <v>Reglas en cc_modelo_reglas para ARS-USD, USD-USD, USD-ARS (usa_intermediario false): par cliente↔pandy, 8 filas por código (24 total). Incluidas en cc_modelo_reglas_tabla.sql y sql/migracion_cc_modelo_reglas_tipos_sin_intermediario.sql para DB existentes.</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B204" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Reversión sin límite de veces</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Eliminada la restricción de cantidad de reversiones (ejecutada→pendiente). Ya no se consulta app_config reversar_max_veces ni la columna revertida_una_vez para bloquear; solo se pide confirmación al reversar. main.js cambiarEstadoTransaccion; docs/CONFIGURACION_REGLAS_NEGOCIO.md actualizado.</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B205" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Tabla CC alineada con Excel (regla madre completa)</v>
+      </c>
+      <c r="D205" t="str">
+        <v>Migración sql/migracion_cc_modelo_reglas_alinear_excel_completo.sql: Tx1 y Tx2 ejecutada con incluir_en_mov_cc_cliente = true; Tx4 ejecutada con incluir_en_mov_cc_intermediario = true; Comisión Pandy ejecutada siempre incluir en cliente. Tx4 pendiente sin incluir en detalle. Todas las combinaciones del Excel cubiertas en la tabla para que el motor sea infalible.</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="B206" t="str">
+        <v>15:36</v>
+      </c>
+      <c r="C206" t="str">
+        <v>v1.41 Despliegue</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Reglas CC: 16 combinaciones cubiertas por tabla (4 filas por tipo). Tx1 pendiente+contrapartida con SUMA_SALDO Y; comisiones pendientes con signo invertido e INCLUIR Y. Compromiso de Pago usa monto transacción (195k) no mr (200k). Docs y SQL actualizados.</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E199"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E206"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4297,7 +4416,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4766,9 +4885,20 @@
         <v>Validación egreso cheques: no ejecutar entrega al intermediario si ingreso Cliente→Pandy pendiente. CC resumen: color unificado (verde = a favor de Pandy, rojo = en contra) para cliente e intermediario.</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>1.41</v>
+      </c>
+      <c r="B43" t="str">
+        <v>17/03/2026</v>
+      </c>
+      <c r="C43" t="str">
+        <v>CC modelo reglas: 16 combinaciones cubiertas por tabla (4 filas por tipo). Tx1 pendiente+contrapartida ejecutada: SUMA_SALDO Y, signo -; comisiones pendientes con signo invertido e INCLUIR Y. Compromiso de Pago con monto de la transacción (195k) no mr (200k).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.41: CC reglas 16 combinaciones, Tx1 pendiente SUMA_SALDO Y, comisiones pendientes INCLUIR Y, Compromiso Pago 195k
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -433,7 +433,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>17/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>15:36</v>
+        <v>15:43</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>

</xml_diff>

<commit_message>
v1.42: Regla Tx1 (P,true) no sumar saldo cliente; E2E CC 12 combinaciones en verde
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E206"/>
+  <dimension ref="A1:E209"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2215,10 +2215,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2266,10 +2266,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2283,10 +2283,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2402,10 +2402,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2419,10 +2419,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2436,10 +2436,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2470,10 +2470,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2487,10 +2487,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2521,10 +2521,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2538,10 +2538,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2572,10 +2572,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2589,10 +2589,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2606,10 +2606,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2623,10 +2623,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2640,10 +2640,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2657,10 +2657,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2674,10 +2674,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2691,10 +2691,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2708,10 +2708,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2725,10 +2725,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2742,10 +2742,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2759,10 +2759,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2776,10 +2776,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2793,10 +2793,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2810,10 +2810,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2827,10 +2827,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2844,10 +2844,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2861,10 +2861,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2878,10 +2878,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2895,10 +2895,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2912,10 +2912,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2946,10 +2946,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2963,10 +2963,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2980,10 +2980,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2997,10 +2997,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3014,10 +3014,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3031,10 +3031,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3048,10 +3048,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3065,10 +3065,10 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3082,10 +3082,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3099,10 +3099,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3116,10 +3116,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3133,10 +3133,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3150,10 +3150,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3167,10 +3167,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3184,10 +3184,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3201,10 +3201,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3218,10 +3218,10 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3235,10 +3235,10 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3252,10 +3252,10 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3269,10 +3269,10 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3286,10 +3286,10 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3303,10 +3303,10 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3320,10 +3320,10 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3354,10 +3354,10 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3371,10 +3371,10 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3388,10 +3388,10 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3405,10 +3405,10 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3422,10 +3422,10 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3439,10 +3439,10 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3456,10 +3456,10 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3473,10 +3473,10 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3490,10 +3490,10 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3507,10 +3507,10 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3524,10 +3524,10 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3541,10 +3541,10 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3558,10 +3558,10 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3575,10 +3575,10 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3592,10 +3592,10 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3609,10 +3609,10 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3626,10 +3626,10 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3643,10 +3643,10 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3660,10 +3660,10 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3677,10 +3677,10 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3694,10 +3694,10 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3711,10 +3711,10 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3728,10 +3728,10 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3745,10 +3745,10 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3762,10 +3762,10 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3779,10 +3779,10 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3796,10 +3796,10 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3813,10 +3813,10 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3830,10 +3830,10 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3847,10 +3847,10 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3864,10 +3864,10 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3881,10 +3881,10 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3898,10 +3898,10 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>15:43</v>
+        <v>03:15</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3913,9 +3913,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B207" t="str">
+        <v>03:15</v>
+      </c>
+      <c r="C207" t="str">
+        <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
+      </c>
+      <c r="D207" t="str">
+        <v>Cada movimiento de CC guarda sumar_al_saldo e incluir_en_detalle (desde la regla al escribir). Saldo = suma solo de movimientos con sumar_al_saldo; detalle = solo filas con incluir_en_detalle. Sync escribe cliente e intermediario cuando incluir OR suma_saldo; comisión int solo si incluir OR suma_saldo. sql/migracion_cc_sumar_saldo_incluir_detalle.sql; main.js sync, fetchMovimientosCcPorEntidad, saldosDesdeMovimientosPorOrden y listado detalle.</v>
+      </c>
+      <c r="E207" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B208" t="str">
+        <v>03:15</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Cuando Tx1=P y Tx2=E (cliente aún no pagó, Pandy ya pagó): saldo cliente = +200k (cliente debe 200k), detalle +195k+5k. cc_modelo_reglas: Tx1 pendiente+contrapartida_ejecutada true → cc_cliente_suma_saldo false. sql/cc_modelo_reglas_todas_combinaciones.sql.</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B209" t="str">
+        <v>03:15</v>
+      </c>
+      <c r="C209" t="str">
+        <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Test tests/e2e/cc-combinaciones.spec.js valida 12 combinaciones Tx1..Tx4 (excl. P,P,E,P; P,E,E,E; Tx1=P y Tx3=E). Esperados en cc-combinaciones-esperado.js. Detalle cliente e int: esperar al menos 1 fila y leer las que haya (evitar timeout). test.step por combinación para ver fallo en reporte.</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E206"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E209"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4029,7 +4080,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de toda la tabla. Al editar transacción se respetan filas momento cero. Tabla detalle: Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
+        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de movimientos con sumar_al_saldo; detalle = solo movimientos con incluir_en_detalle (dos flags por movimiento desde cc_modelo_reglas). Tabla detalle: Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
       </c>
     </row>
     <row r="14">
@@ -4416,7 +4467,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4439,7 +4490,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -4450,7 +4501,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -4461,7 +4512,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -4472,7 +4523,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -4483,7 +4534,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -4494,7 +4545,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -4505,7 +4556,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -4516,7 +4567,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -4527,7 +4578,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -4538,7 +4589,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -4549,7 +4600,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -4560,7 +4611,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -4571,7 +4622,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -4582,7 +4633,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -4593,7 +4644,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -4604,7 +4655,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -4615,7 +4666,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -4626,7 +4677,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -4637,7 +4688,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -4648,7 +4699,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -4659,7 +4710,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -4670,7 +4721,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -4681,7 +4732,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -4692,7 +4743,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -4703,7 +4754,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -4714,7 +4765,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -4725,7 +4776,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -4736,7 +4787,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -4747,7 +4798,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
@@ -4758,7 +4809,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
@@ -4769,7 +4820,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
@@ -4780,7 +4831,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
@@ -4791,7 +4842,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Switch Activo en tablas Clientes e Intermediarios; modales Cliente/Intermediario con toggle; centrado de botón y título en todas las pantallas con switch. Script truncar: orden correcto y orden_comisiones_generadas opcional. Tests E2E: intermediario solo si visible (tipos sin intermediario).</v>
@@ -4802,7 +4853,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>CC ARS-ARS con intermediario: momento cero cliente (-mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía testing con TEST_BASE_URL cuando Vite usa otro puerto.</v>
@@ -4813,7 +4864,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C36" t="str">
         <v>CC regla simple (USD-USD, 2 transacciones): compromisos solo cuando al menos una transacción está ejecutada; si ambas pendientes, saldo 0 (no figura deuda).</v>
@@ -4824,7 +4875,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Regla de estilos de botones LyP: mismo estilo (border-radius 8px, min-height); con leyenda = icono a la izquierda; solo icono mismo estilo; botón Excel verde. Regla estilos-botones.mdc en Pandi y en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
@@ -4835,7 +4886,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. Al completar tareas hay que actualizar bitácora, revisar RPC en sql/ si aplica y adaptar tests si afectan. bitacora-tareas.mdc y reglas-pandi.mdc.</v>
@@ -4846,7 +4897,7 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Modales: no cerrar al elegir en select (mousedown+click en backdrop). Sesión: mousemove cuenta como actividad para no cerrar por inactividad al mover mouse/trackpad. CC: Tipo op. después de Fecha, sticky y export Excel.</v>
@@ -4857,7 +4908,7 @@
         <v>1.38</v>
       </c>
       <c r="B40" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C40" t="str">
         <v>Producción Vercel: XLSX cargado desde CDN (script en index.html); main.js usa window.XLSX para evitar error "Failed to resolve module specifier xlsx" sin bundler.</v>
@@ -4868,7 +4919,7 @@
         <v>1.39</v>
       </c>
       <c r="B41" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C41" t="str">
         <v>CC regla infalible: ingreso misma moneda aporta -me (Pandy debe su transacción); egreso con ingreso pendiente aporta +mr (resumen muestra deuda del cliente). Sin movimiento extra ganancia Pandy en CC. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
@@ -4879,7 +4930,7 @@
         <v>1.40</v>
       </c>
       <c r="B42" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C42" t="str">
         <v>Validación egreso cheques: no ejecutar entrega al intermediario si ingreso Cliente→Pandy pendiente. CC resumen: color unificado (verde = a favor de Pandy, rojo = en contra) para cliente e intermediario.</v>
@@ -4890,15 +4941,26 @@
         <v>1.41</v>
       </c>
       <c r="B43" t="str">
-        <v>17/03/2026</v>
+        <v>18/03/2026</v>
       </c>
       <c r="C43" t="str">
         <v>CC modelo reglas: 16 combinaciones cubiertas por tabla (4 filas por tipo). Tx1 pendiente+contrapartida ejecutada: SUMA_SALDO Y, signo -; comisiones pendientes con signo invertido e INCLUIR Y. Compromiso de Pago con monto de la transacción (195k) no mr (200k).</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>1.42</v>
+      </c>
+      <c r="B44" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Regla Tx1 (P,true) no sumar: saldo cliente +200k cuando Tx2=E. E2E CC combinaciones: 12 combinaciones, esperados y test resistente (detalle); test.step por combinación.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.43: E2E CC combinaciones esperados alineados; PASS saldo 0; Real desde vista Detalle de movimientos
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E209"/>
+  <dimension ref="A1:E213"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3918,7 +3918,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3935,7 +3935,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3952,7 +3952,7 @@
         <v>18/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>03:15</v>
+        <v>15:47</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3964,16 +3964,84 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B210" t="str">
+        <v>15:47</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Instrumentación: orden por numero 1,2,3,4</v>
+      </c>
+      <c r="D210" t="str">
+        <v>En el modal Nueva orden, paso Instrumentación, la tabla de transacciones se ordena por numero (ascendente) para que la fila 1 sea siempre Tx1, la 2 sea Tx2, etc. sortTransaccionesPorNumero en main.js; renderOrdenWizardInstrumentacion usa ese orden en lugar de sortTransaccionesIngresosPrimero. Así los tests E2E (nth(0)..nth(3)) aplican la combinación a las transacciones correctas.</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B211" t="str">
+        <v>15:47</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Regla: antes de asignar numero de transacción, el orden debe ser por pagador: 1) Cliente, 2) Pandy, 3) Intermediario. autoCompletarInstrumentacionChequeConIntermediario y autoCompletarInstrumentacionSinIntermediario insertan las filas en secuencia (reduce en lugar de Promise.all) para que la DB asigne numero 1,2,3,4 en ese orden. Así la combinación E,P,E,P coincide siempre con Tx1..Tx4.</v>
+      </c>
+      <c r="E211" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B212" t="str">
+        <v>15:47</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
+      </c>
+      <c r="D212" t="str">
+        <v>El test E2E ejecuta antes de iniciar: 1) Borrar clientes e intermediarios creados por los tests (E2E %). 2) Truncar órdenes, transacciones, instrumentación, CC y caja (mismo orden que truncar_ordenes_transacciones.sql). sql/rpc_limpiar_base_e2e.sql (RPC), scripts/limpiar-base-e2e.js (Node con Supabase), globalSetup en Playwright. Opcional: SUPABASE_URL y SUPABASE_SERVICE_ROLE_KEY en .env.test.</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="B213" t="str">
+        <v>15:47</v>
+      </c>
+      <c r="C213" t="str">
+        <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Fix combinación P,P,P,P (todo pendiente): (1) cc_modelo_reglas: Tx4 Int→Pandy pendiente+contrapartida false → incluir_en_mov_cc_intermediario false (evita que el front envíe el movimiento 197k). (2) RPC sync_cc_caja_orden: INSERT CC cliente e intermediario ahora incluye sumar_al_saldo e incluir_en_detalle desde el JSON (COALESCE a true si faltan). sql/cc_modelo_reglas_fix_pppp_saldo_cero.sql (UPDATE 4) y sql/rpc_sync_cc_caja_orden.sql. Test E2E P,P,P,P pasa sin errores.</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E209"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E213"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:E57"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4309,95 +4377,171 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
+        <v>Instrumentación: orden por numero 1,2,3,4</v>
       </c>
       <c r="B42" t="str">
-        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
+        <v>En el paso Instrumentación del modal de orden la tabla se ordena por numero (1, 2, 3, 4). Al crear transacciones (auto-completar) se insertan en secuencia por pagador: Cliente, Pandy, Intermediario, para que la DB asigne numero en ese orden y la combinación coincida con Tx1..Tx4.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Cargar orden por chat</v>
+        <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
       </c>
       <c r="B43" t="str">
-        <v>Botón Cargar por chat (estilo btn-chat, azul) en vista Órdenes y en Panel de Control (Accesos rápidos); visible solo con permiso ingresar_orden. Mensaje en lenguaje natural; con un monto y TC se calcula el otro. Al confirmar se crean orden e instrumentación.</v>
+        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Tests E2E (Playwright)</v>
+        <v>Cargar orden por chat</v>
       </c>
       <c r="B44" t="str">
-        <v>Tests en tests/e2e/: login (pantalla login, login con usuario de prueba, navegación a Panel). Orden ARS-ARS y cuenta corriente: flujo completo (nueva orden tipo ARS-ARS, cliente, importe cheque + tasa, instrumentación, ejecutar las dos transacciones) y verificación de que la CC refleja cada paso. Requisitos: tipo ARS-ARS activo, al menos un cliente, usuario con permisos. Guía docs/TESTING_E2E_GUIA.md.</v>
+        <v>Botón Cargar por chat (estilo btn-chat, azul) en vista Órdenes y en Panel de Control (Accesos rápidos); visible solo con permiso ingresar_orden. Mensaje en lenguaje natural; con un monto y TC se calcula el otro. Al confirmar se crean orden e instrumentación.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Número de transacción y convención caja</v>
+        <v>Tests E2E (Playwright)</v>
       </c>
       <c r="B45" t="str">
-        <v>Transacciones tienen número interno (transacciones.numero, secuencia) para trazabilidad. Movimientos de caja originados por transacción usan concepto: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Panel de transacciones muestra columna Nro. sql/migracion_transacciones_numero.sql.</v>
+        <v>Tests en tests/e2e/: login (pantalla login, login con usuario de prueba, navegación a Panel). Orden ARS-ARS y cuenta corriente: flujo completo (nueva orden tipo ARS-ARS, cliente, importe cheque + tasa, instrumentación, ejecutar las dos transacciones) y verificación de que la CC refleja cada paso. Requisitos: tipo ARS-ARS activo, al menos un cliente, usuario con permisos. Guía docs/TESTING_E2E_GUIA.md.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Log E2E hoja Caja</v>
+        <v>Número de transacción y convención caja</v>
       </c>
       <c r="B46" t="str">
-        <v>Hoja Caja en Excel: una fila por transacción (y una final) con columnas Saldo_Caja_EF/BA por moneda (Esp, App, Resultado). irACajasYLeerSaldos espera fin de carga para que los saldos no queden en blanco. tests/e2e/orden-cc.spec.js y e2e-log-excel.js.</v>
+        <v>Transacciones tienen número interno (transacciones.numero, secuencia) para trazabilidad. Movimientos de caja originados por transacción usan concepto: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Panel de transacciones muestra columna Nro. sql/migracion_transacciones_numero.sql.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Movimientos de caja estructurados</v>
+        <v>Log E2E hoja Caja</v>
       </c>
       <c r="B47" t="str">
-        <v>Tabla movimientos_caja con orden_numero y transaccion_numero; vista Cajas: columnas Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Caja, Concepto. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+        <v>Hoja Caja en Excel: una fila por transacción (y una final) con columnas Saldo_Caja_EF/BA por moneda (Esp, App, Resultado). irACajasYLeerSaldos espera fin de carga para que los saldos no queden en blanco. tests/e2e/orden-cc.spec.js y e2e-log-excel.js.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Caja: movimiento por comisión Pandy</v>
+        <v>Movimientos de caja estructurados</v>
       </c>
       <c r="B48" t="str">
-        <v>Cuando hay comisión Pandy (misma moneda, sin transacción Ganancia) la sincronización agrega un movimiento de caja (ingreso efectivo por la comisión) para que la caja cierre en cero en operaciones de cobro de cheques. transaccion_id null; al re-sincronizar se borran esos movimientos por orden.</v>
+        <v>Tabla movimientos_caja con orden_numero y transaccion_numero; vista Cajas: columnas Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Caja, Concepto. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Tipos de operación: Intermediario Sí/No</v>
+        <v>Caja: movimiento por comisión Pandy</v>
       </c>
       <c r="B49" t="str">
-        <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
+        <v>Cuando hay comisión Pandy (misma moneda, sin transacción Ganancia) la sincronización agrega un movimiento de caja (ingreso efectivo por la comisión) para que la caja cierre en cero en operaciones de cobro de cheques. transaccion_id null; al re-sincronizar se borran esos movimientos por orden.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Número de orden atómico (MAX+1)</v>
+        <v>Tipos de operación: Intermediario Sí/No</v>
       </c>
       <c r="B50" t="str">
-        <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+        <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Utils y RPC sync CC/caja</v>
+        <v>Número de orden atómico (MAX+1)</v>
       </c>
       <c r="B51" t="str">
-        <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
+        <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
+        <v>Utils y RPC sync CC/caja</v>
+      </c>
+      <c r="B52" t="str">
+        <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
         <v>Conceptos CC unificados y número de transacción</v>
       </c>
-      <c r="B52" t="str">
+      <c r="B53" t="str">
         <v>Todos los movimientos CC (cliente e intermediario) usan leyendas unificadas (Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo) con sufijo " - Orden x y Trans x". transaccion_numero se guarda en todos los inserts/rows para que la columna Trans. del detalle nunca quede en blanco cuando hay transacción de referencia. Incluye movimientos derivados (pago/cobro de comisiones).</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="B54" t="str">
+        <v>__AHORA__</v>
+      </c>
+      <c r="C54" t="str">
+        <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Ajuste de 6 combinaciones en tests/e2e/cc-combinaciones-esperado.js: P,E,P,P y E,E,P,P int 0 y detalle []; E,P,P,P cliente -200k y [-200k], int 0 y []; E,P,P,E, E,P,E,P, E,P,E,E cliente -200k y [-200k] (sin 5k cuando Tx2=P). Doc docs/CC_COMBINACIONES_ESPERADO_DERIVACION.md reescrita con las 12 combinaciones y tabla resumen final.</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="B55" t="str">
+        <v>__AHORA__</v>
+      </c>
+      <c r="C55" t="str">
+        <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Si saldo esperado es 0 la app no muestra fila en resumen → no se abre modal. El test marca PASS en detalle (no N/A). Detalle se lee solo del modal Ver detalle (#cc-detalle-tbody), no de la vista Detalle de movimientos. tests/e2e/cc-combinaciones.spec.js.</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="B56" t="str">
+        <v>__AHORA__</v>
+      </c>
+      <c r="C56" t="str">
+        <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Cuando no hay fila en Resumen (saldo 0) el test hace clic en Detalle de movimientos (Tipo Cliente o Intermediario) y lee la tabla para rellenar Real en el log Excel. Mismo criterio para cliente e intermediario. tests/e2e/cc-combinaciones.spec.js.</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="B57" t="str">
+        <v>__AHORA__</v>
+      </c>
+      <c r="C57" t="str">
+        <v>v1.43 Despliegue</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Versión 1.43: E2E CC combinaciones esperados alineados con tabla SQL; PASS en detalle cuando saldo 0; Real desde vista Detalle de movimientos (Cliente e Int).</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4467,7 +4611,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4958,9 +5102,20 @@
         <v>Regla Tx1 (P,true) no sumar: saldo cliente +200k cuando Tx2=E. E2E CC combinaciones: 12 combinaciones, esperados y test resistente (detalle); test.step por combinación.</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>1.43</v>
+      </c>
+      <c r="B45" t="str">
+        <v>18/03/2026</v>
+      </c>
+      <c r="C45" t="str">
+        <v>E2E CC combinaciones: esperados alineados con tabla SQL (6 combinaciones); PASS en detalle cuando saldo 0; Real rellenado desde vista Detalle de movimientos (Cliente e Intermediario) cuando no hay fila en Resumen.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.44: CHEQUE-ARS canónico, modal tipo op iconos, E2E/SQL y docs
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E230"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -447,10 +447,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -464,10 +464,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -481,10 +481,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -498,10 +498,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -515,10 +515,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -532,10 +532,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -549,10 +549,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -566,10 +566,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -583,10 +583,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -600,10 +600,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -617,10 +617,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -634,10 +634,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -651,10 +651,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -668,10 +668,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -685,10 +685,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -719,10 +719,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -736,10 +736,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -753,10 +753,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -770,10 +770,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -787,10 +787,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -821,10 +821,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -838,10 +838,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -855,10 +855,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -889,10 +889,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -906,10 +906,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -957,10 +957,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -974,10 +974,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -991,10 +991,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1008,10 +1008,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1025,10 +1025,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1042,10 +1042,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1059,10 +1059,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1110,10 +1110,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1127,10 +1127,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1178,10 +1178,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1195,10 +1195,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1212,10 +1212,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1229,10 +1229,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1246,10 +1246,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1280,10 +1280,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1297,10 +1297,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1314,10 +1314,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1331,10 +1331,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1348,10 +1348,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1365,10 +1365,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1382,10 +1382,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1399,10 +1399,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1416,10 +1416,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1450,10 +1450,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1467,10 +1467,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1484,10 +1484,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1501,10 +1501,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1535,10 +1535,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1552,10 +1552,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1569,10 +1569,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1586,10 +1586,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1637,10 +1637,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1654,10 +1654,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1671,10 +1671,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1705,10 +1705,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1722,10 +1722,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1739,10 +1739,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1756,10 +1756,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1807,10 +1807,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1824,10 +1824,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1858,10 +1858,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1875,10 +1875,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1892,10 +1892,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1926,10 +1926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1943,10 +1943,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1960,10 +1960,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1994,10 +1994,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2011,10 +2011,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2028,10 +2028,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2045,10 +2045,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2062,10 +2062,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2079,10 +2079,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2113,10 +2113,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2130,10 +2130,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2164,10 +2164,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2198,10 +2198,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2215,10 +2215,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2232,10 +2232,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2249,10 +2249,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2266,10 +2266,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2283,10 +2283,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2300,10 +2300,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2317,10 +2317,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2351,10 +2351,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2368,10 +2368,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2385,10 +2385,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2402,10 +2402,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2419,10 +2419,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2436,10 +2436,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2470,10 +2470,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2487,10 +2487,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2521,10 +2521,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2538,10 +2538,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2555,10 +2555,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2572,10 +2572,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2589,10 +2589,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2606,10 +2606,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2623,10 +2623,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2640,10 +2640,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2657,10 +2657,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2674,10 +2674,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2691,10 +2691,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2708,10 +2708,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2725,10 +2725,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2742,10 +2742,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2759,10 +2759,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2776,10 +2776,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2793,10 +2793,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2810,10 +2810,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2827,10 +2827,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2844,10 +2844,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2861,10 +2861,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2878,10 +2878,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2895,10 +2895,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2912,10 +2912,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2929,10 +2929,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2946,10 +2946,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2963,10 +2963,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2980,10 +2980,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -2997,10 +2997,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3014,10 +3014,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3031,10 +3031,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3048,10 +3048,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3065,10 +3065,10 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3082,10 +3082,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3099,10 +3099,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3116,10 +3116,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3133,10 +3133,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3150,10 +3150,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3167,10 +3167,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3184,10 +3184,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3201,10 +3201,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3218,10 +3218,10 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3235,10 +3235,10 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3252,10 +3252,10 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3269,10 +3269,10 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3286,10 +3286,10 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3303,10 +3303,10 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3320,10 +3320,10 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3354,10 +3354,10 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3371,10 +3371,10 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3388,10 +3388,10 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3405,10 +3405,10 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3422,10 +3422,10 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3439,10 +3439,10 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3456,10 +3456,10 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3473,10 +3473,10 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3490,10 +3490,10 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3507,10 +3507,10 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3524,10 +3524,10 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3541,10 +3541,10 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3558,10 +3558,10 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3575,10 +3575,10 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3592,10 +3592,10 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3609,10 +3609,10 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3626,10 +3626,10 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3643,10 +3643,10 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3660,10 +3660,10 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3677,10 +3677,10 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3694,10 +3694,10 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3711,10 +3711,10 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3728,10 +3728,10 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3745,10 +3745,10 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3762,10 +3762,10 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3779,10 +3779,10 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3796,10 +3796,10 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3813,10 +3813,10 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3830,10 +3830,10 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3847,10 +3847,10 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3864,10 +3864,10 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3881,10 +3881,10 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3898,10 +3898,10 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3915,10 +3915,10 @@
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3932,10 +3932,10 @@
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3949,10 +3949,10 @@
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3966,10 +3966,10 @@
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B210" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C210" t="str">
         <v>Instrumentación: orden por numero 1,2,3,4</v>
@@ -3983,10 +3983,10 @@
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B211" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C211" t="str">
         <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
@@ -4000,10 +4000,10 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B212" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C212" t="str">
         <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
@@ -4017,10 +4017,10 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="B213" t="str">
-        <v>15:47</v>
+        <v>10:03</v>
       </c>
       <c r="C213" t="str">
         <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
@@ -4032,16 +4032,305 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B214" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C214" t="str">
+        <v>E2E CC combinaciones: subir timeout global</v>
+      </c>
+      <c r="D214" t="str">
+        <v>tests/e2e/cc-combinaciones.spec.js ajusta timeouts para evitar corte por sync CC/caja más lento en combinaciones como E,E,E,P (timeout global y espera de #orden-inst-actualizando-msg).</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B215" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Doc respaldo E2E CC + RPC null-safe</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Comentario en sql/rpc_sync_cc_caja_orden.sql sobre -&gt;&gt; y null. Docs: TESTING_E2E_GUIA §1.6–1.7, CONTEXTO_TEST_CC_COMBINACIONES, INVESTIGACION_CC_COMBINACIONES_FUENTE_VERDAD §7, FUNCIONES_CRITICAS_SUPABASE_VS_FRONT, DONDE_QUEDAMOS. Eliminado console.log debug en main.js (sync CC).</v>
+      </c>
+      <c r="E215" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B216" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Panel y Cajas: mismos permisos en cards + Cheque ARS</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Tarjetas Efectivo/Banco/Cheque en Panel de Control gobernadas por ver_cajas_efectivo, ver_cajas_banco, ver_cajas_cheque (igual que vista Cajas). Nueva card Cheque en Panel (solo ARS: saldo inicial, actual, variación). Card Cheque en Cajas solo ARS; icono /assets/Icono_Cheques.png. Seguridad: bloque Panel sin ver_inicio_efectivo/banco (solo ver_inicio y pendientes). sql/migracion_panel_tarjetas_mismos_permisos_ver_cajas.sql. docs/PERMISOS_POR_MENU.md.</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B217" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C217" t="str">
+        <v>UI card Cheque compacta y alineada</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Clase inicio-caja-card-cheque-compact: ancho max-content/justify-self start en desktop; columna ARS minmax(max-content) y encabezado flex-end alineado con importes. Vista Cajas misma clase. Móvil ≤768: card a ancho disponible.</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B218" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Tipo de operación: iconos moneda y cheque</v>
+      </c>
+      <c r="D218" t="str">
+        <v>utils.js: htmlTipoOperacionIconos (par monedas con →; código con CHEQUE → Icono_Cheques.png), htmlIconoMonedaTipoOp. Órdenes, órdenes pendientes, CC detalle (vista y modal), ABM tipos (columna Tipo + IN/OUT con icono). Modal orden: preview junto al select. Export Excel sigue con código texto.</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B219" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Tipos de operación: icono configurable (auto / cheques / imagen)</v>
+      </c>
+      <c r="D219" t="str">
+        <v>Columnas icono_modo e icono_url_publica en tipos_operacion. ABM: modo automático, siempre cheques o personalizado (URL https o subida a Storage bucket tipo-operacion-iconos). htmlTipoOperacionIconos con opts; listados órdenes, pendientes, CC y preview en modal orden. sql/migracion_tipos_operacion_icono.sql, sql/storage_bucket_tipo_operacion_iconos.sql, docs/TIPOS_OPERACION_ICONO.md.</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B220" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C220" t="str">
+        <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Ajuste de 6 combinaciones en tests/e2e/cc-combinaciones-esperado.js: P,E,P,P y E,E,P,P int 0 y detalle []; E,P,P,P cliente -200k y [-200k], int 0 y []; E,P,P,E, E,P,E,P, E,P,E,E cliente -200k y [-200k] (sin 5k cuando Tx2=P). Doc docs/CC_COMBINACIONES_ESPERADO_DERIVACION.md reescrita con las 12 combinaciones y tabla resumen final.</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B221" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C221" t="str">
+        <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
+      </c>
+      <c r="D221" t="str">
+        <v>Si saldo esperado es 0 la app no muestra fila en resumen → no se abre modal. El test marca PASS en detalle (no N/A). Detalle se lee solo del modal Ver detalle (#cc-detalle-tbody), no de la vista Detalle de movimientos. tests/e2e/cc-combinaciones.spec.js.</v>
+      </c>
+      <c r="E221" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B222" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C222" t="str">
+        <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
+      </c>
+      <c r="D222" t="str">
+        <v>Cuando no hay fila en Resumen (saldo 0) el test hace clic en Detalle de movimientos (Tipo Cliente o Intermediario) y lee la tabla para rellenar Real en el log Excel. Mismo criterio para cliente e intermediario. tests/e2e/cc-combinaciones.spec.js.</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B223" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C223" t="str">
+        <v>v1.43 Despliegue</v>
+      </c>
+      <c r="D223" t="str">
+        <v>Versión 1.43: E2E CC combinaciones esperados alineados con tabla SQL; PASS en detalle cuando saldo 0; Real desde vista Detalle de movimientos (Cliente e Int).</v>
+      </c>
+      <c r="E223" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B224" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C224" t="str">
+        <v>CC sync: dedupe por (entidad, orden, monto)</v>
+      </c>
+      <c r="D224" t="str">
+        <v>Evitar doble -200k en E,P,P,E y E,P,E,P: el dedupe antes de sync_cc_caja_orden usa clave (cliente_id/intermediario_id, orden_id, monto) sin concepto ni transaccion_id, una sola fila por (orden, entidad, monto). Sin cambios en tablas ni RPC.</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B225" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C225" t="str">
+        <v>Tipo operación: moneda Cheque (CHEQUE–ARS)</v>
+      </c>
+      <c r="D225" t="str">
+        <v>ABM tipos: opción Cheque en Moneda IN/OUT (solo con ARS del otro lado). En órdenes moneda_recibida/entregada siguen ARS. Helpers esTipoOperacionChequeArs / monedaCatalogoParaOrden: mismo flujo que ARS-ARS legacy (4 transacciones, comisión ARS, reglas cc_modelo como ARS-ARS, sync CC, wizard, validaciones). Listas órdenes/pendientes cargan moneda_in/out en mapa tipos. index.html selects; main.js; docs/TIPOS_OPERACION_MONEDA_CHEQUE.md.</v>
+      </c>
+      <c r="E225" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B226" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C226" t="str">
+        <v>E2E: tipo CHEQUE-ARS en tests CC</v>
+      </c>
+      <c r="D226" t="str">
+        <v>tests/e2e/cc-combinaciones.spec.js y orden-cc.spec.js seleccionan option[data-codigo="CHEQUE-ARS"]. sql/seed_tipo_operacion_cheque_ars.sql para crear el catálogo en Supabase. docs/TESTING_E2E_GUIA.md §1.5 actualizado.</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B227" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Fix SQL CHEQUE en checks de moneda</v>
+      </c>
+      <c r="D227" t="str">
+        <v>migracion_cc_modelo_reglas_canonico_cheque_ars.sql y seed_tipo_operacion_cheque_ars.sql ahora recrean checks tipos_operacion_moneda_in/out para permitir CHEQUE antes de setear moneda_in/out=CHEQUE,ARS. Evita error 23514 en Supabase.</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B228" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Canónico CHEQUE-ARS en tabla de verdad</v>
+      </c>
+      <c r="D228" t="str">
+        <v>SQL y motor CC alineados a CHEQUE-ARS como código canónico: migración sql/migracion_cc_modelo_reglas_canonico_cheque_ars.sql (migra reglas y catálogo), scripts cc_modelo_* actualizados, main.js prioriza reglas CHEQUE-ARS con fallback ARS-ARS. seed desactiva ARS-ARS-CHEQUE legacy en dev.</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B229" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Modal orden: tipo de operación con iconos</v>
+      </c>
+      <c r="D229" t="str">
+        <v>Nueva orden / Editar: listbox custom con mismos iconos que la tabla (monedas IN→OUT, cheque, custom URL). El &lt;select id="orden-tipo-operacion"&gt; sigue en el DOM (oculto) con las mismas &lt;option data-codigo&gt;; Playwright sigue usando selectOption y option[data-codigo=…]. Escape cierra solo el desplegable antes que el modal. index.html + main.js (rebuildOrdenTipoOperacionListbox, closeOrdenTipoOperacionListbox).</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B230" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Fix listbox tipo operación en modal orden</v>
+      </c>
+      <c r="D230" t="str">
+        <v>El desplegable quedaba recortado por overflow-y del .modal-body y overflow del .modal; al abrir se posiciona con position:fixed según getBoundingClientRect del botón, z-index alto, reposición en scroll/resize. Modal orden min-height 220px para la vista inicial compacta.</v>
+      </c>
+      <c r="E230" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E230"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:B53"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4108,7 +4397,7 @@
         <v>Vista Cajas</v>
       </c>
       <c r="B8" t="str">
-        <v>Dos cards como Panel: Efectivo y Banco (visibles según ver_cajas_efectivo y ver_cajas_banco). Permisos granulares Ver Efectivo / Ver Banco; al desactivar Ver u Operar en Seguridad se muestra mensaje aclaratorio. Filtro por moneda y tabla de movimientos; ABM movimientos y tipos según permisos.</v>
+        <v>Cards Efectivo, Banco y Cheque (Cheque solo saldo ARS; icono Icono_Cheques.png). Visibilidad según ver_cajas_efectivo, ver_cajas_banco, ver_cajas_cheque (mismos permisos que en Panel de Control). Filtro por moneda y tabla de movimientos; ABM movimientos y tipos según permisos.</v>
       </c>
     </row>
     <row r="9">
@@ -4132,7 +4421,7 @@
         <v>Vista Órdenes</v>
       </c>
       <c r="B11" t="str">
-        <v>Listado, Nueva orden y Editar. Estados: cotización, cerrada, concertada. Al concertar se generan movimientos de caja y cuenta corriente (evita doble concertación).</v>
+        <v>Listado con columna tipo de operación como iconos (monedas IN→OUT, cheque por código o por configuración del tipo, o imagen personalizada https). Nueva orden y Editar: selector de tipo como listbox con iconos + nombre; el select nativo permanece oculto para E2E y datos. Estados: cotización, cerrada, concertada. Al concertar se generan movimientos de caja y cuenta corriente.</v>
       </c>
     </row>
     <row r="12">
@@ -4148,7 +4437,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Momento cero: 2 filas (Debe X monR de nro orden N + Compensación de nro orden N) con ambas monedas; el concepto usa siempre el número interno de orden (no el id de Supabase). Al ejecutar se marca la fila cerrado y se inserta Cancelación de deuda (sin invertir signos). Saldo = suma de movimientos con sumar_al_saldo; detalle = solo movimientos con incluir_en_detalle (dos flags por movimiento desde cc_modelo_reglas). Tabla detalle: Fecha, Orden, Trans., Tipo op., Concepto, USD, ARS, EUR, Estado. Filtro Cliente/Intermediario; Refrescar; modal detalle. Script sql/truncar_ordenes_transacciones.sql incluye reset de secuencia (próxima orden nº 1).</v>
+        <v>Momento cero: 2 filas (Debe + Compensación) con ambas monedas; concepto con número interno de orden. Saldo = suma con sumar_al_saldo; detalle con incluir_en_detalle. Tabla detalle: Tipo op. como iconos (incluye icono configurable por tipo); export Excel con código en texto. Filtro Cliente/Intermediario; modal detalle. sql/truncar_ordenes_transacciones.sql.</v>
       </c>
     </row>
     <row r="14">
@@ -4172,7 +4461,7 @@
         <v>Panel de Control (Inicio)</v>
       </c>
       <c r="B16" t="str">
-        <v>Tarjetas Efectivo y Banco: Saldo Inicial, Saldo Actual (fila destacada), Var. con icono tendencia; USD/ARS/EUR (Efectivo) y USD/ARS (Banco); iconos por moneda. Cards Órdenes pendientes (por estado, ojo por fila y en título) y Transacciones pendientes (cantidad en círculo); mismo ancho que Efectivo.</v>
+        <v>Tarjetas Efectivo, Banco y Cheque (Cheque solo ARS, misma lógica inicial/actual/var. que las otras; icono Icono_Cheques.png). Visibilidad de las tres cards con ver_cajas_efectivo, ver_cajas_banco, ver_cajas_cheque. Cards Órdenes pendientes y Transacciones pendientes (ver_inicio_pendientes).</v>
       </c>
     </row>
     <row r="17">
@@ -4252,7 +4541,7 @@
         <v>Panel de Control parametrizable</v>
       </c>
       <c r="B26" t="str">
-        <v>Tres permisos: ver_inicio_efectivo, ver_inicio_banco, ver_inicio_pendientes. En Inicio se muestran/ocultan tarjetas Efectivo, Banco y bloque Pendientes según permiso. Por defecto visor solo tarjetas de pendientes.</v>
+        <v>ver_inicio y ver_inicio_pendientes en bloque Panel en Seguridad. Tarjetas de cajas en Panel usan los mismos permisos que Cajas: ver_cajas_efectivo, ver_cajas_banco, ver_cajas_cheque. Migración opcional sql/migracion_panel_tarjetas_mismos_permisos_ver_cajas.sql para roles con solo permisos legacy ver_inicio_efectivo/banco.</v>
       </c>
     </row>
     <row r="27">
@@ -4388,7 +4677,7 @@
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
       </c>
       <c r="B43" t="str">
-        <v>Tabla tipos_operacion con moneda_in y moneda_out (fuente de verdad). Lógica de orden y transacción usa esas columnas; fallback a parsear código. ABM Tipos de operación: vista en menú (permiso abm_tipos_operacion), listado, Nuevo/Editar con código, nombre, moneda IN, moneda OUT, activo. Migración sql/migracion_tipos_operacion_moneda_abm.sql.</v>
+        <v>Tabla tipos_operacion con moneda_in y moneda_out (USD, EUR, ARS, CHEQUE). Cheque solo con ARS; en órdenes se persiste ARS. Código canónico de reglas y catálogo: CHEQUE-ARS (con fallback legacy ARS-ARS en motor). ABM: columna Tipo con iconos; Moneda IN/OUT. Migraciones: sql/migracion_cc_modelo_reglas_canonico_cheque_ars.sql, sql/seed_tipo_operacion_cheque_ars.sql, sql/migracion_tipos_operacion_icono.sql.</v>
       </c>
     </row>
     <row r="44">
@@ -4471,77 +4760,9 @@
         <v>Todos los movimientos CC (cliente e intermediario) usan leyendas unificadas (Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo) con sufijo " - Orden x y Trans x". transaccion_numero se guarda en todos los inserts/rows para que la columna Trans. del detalle nunca quede en blanco cuando hay transacción de referencia. Incluye movimientos derivados (pago/cobro de comisiones).</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>__HOY__</v>
-      </c>
-      <c r="B54" t="str">
-        <v>__AHORA__</v>
-      </c>
-      <c r="C54" t="str">
-        <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
-      </c>
-      <c r="D54" t="str">
-        <v>Ajuste de 6 combinaciones en tests/e2e/cc-combinaciones-esperado.js: P,E,P,P y E,E,P,P int 0 y detalle []; E,P,P,P cliente -200k y [-200k], int 0 y []; E,P,P,E, E,P,E,P, E,P,E,E cliente -200k y [-200k] (sin 5k cuando Tx2=P). Doc docs/CC_COMBINACIONES_ESPERADO_DERIVACION.md reescrita con las 12 combinaciones y tabla resumen final.</v>
-      </c>
-      <c r="E54" t="str">
-        <v>Desarrollo</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>__HOY__</v>
-      </c>
-      <c r="B55" t="str">
-        <v>__AHORA__</v>
-      </c>
-      <c r="C55" t="str">
-        <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
-      </c>
-      <c r="D55" t="str">
-        <v>Si saldo esperado es 0 la app no muestra fila en resumen → no se abre modal. El test marca PASS en detalle (no N/A). Detalle se lee solo del modal Ver detalle (#cc-detalle-tbody), no de la vista Detalle de movimientos. tests/e2e/cc-combinaciones.spec.js.</v>
-      </c>
-      <c r="E55" t="str">
-        <v>Desarrollo</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>__HOY__</v>
-      </c>
-      <c r="B56" t="str">
-        <v>__AHORA__</v>
-      </c>
-      <c r="C56" t="str">
-        <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
-      </c>
-      <c r="D56" t="str">
-        <v>Cuando no hay fila en Resumen (saldo 0) el test hace clic en Detalle de movimientos (Tipo Cliente o Intermediario) y lee la tabla para rellenar Real en el log Excel. Mismo criterio para cliente e intermediario. tests/e2e/cc-combinaciones.spec.js.</v>
-      </c>
-      <c r="E56" t="str">
-        <v>Desarrollo</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>__HOY__</v>
-      </c>
-      <c r="B57" t="str">
-        <v>__AHORA__</v>
-      </c>
-      <c r="C57" t="str">
-        <v>v1.43 Despliegue</v>
-      </c>
-      <c r="D57" t="str">
-        <v>Versión 1.43: E2E CC combinaciones esperados alineados con tabla SQL; PASS en detalle cuando saldo 0; Real desde vista Detalle de movimientos (Cliente e Int).</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Despliegue</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B53"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4611,7 +4832,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -4634,7 +4855,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C2" t="str">
         <v>Setup: estructura repo, reglas de trabajo, script bitácora, package.json, Vercel, config.example.</v>
@@ -4645,7 +4866,7 @@
         <v>1.1</v>
       </c>
       <c r="B3" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C3" t="str">
         <v>Mensajería propia (toast en lugar de alert), tasa descuento intermediario solo coma decimal, movimientos caja efectivo/banco, conceptos CC más claros (Conversión de moneda, Comisión del acuerdo), layout extendido (max-width 1600px), responsive móvil reforzado (safe area, tablas, toasts, form actions).</v>
@@ -4656,7 +4877,7 @@
         <v>1.2</v>
       </c>
       <c r="B4" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C4" t="str">
         <v>Quitar título redundante "Panel de Control" en vista Inicio (solo se muestra en el header).</v>
@@ -4667,7 +4888,7 @@
         <v>1.3</v>
       </c>
       <c r="B5" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C5" t="str">
         <v>Permisos granulares: editar_orden y cambiar_estado_transaccion. SQL migración (app_permission, RLS), frontend: botones Editar orden y combo estado transacción según permiso; guardar orden con validación de permisos.</v>
@@ -4678,7 +4899,7 @@
         <v>1.4</v>
       </c>
       <c r="B6" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C6" t="str">
         <v>Logo y favicon: Emoji-de-WhatsApp-panda como base. Recorte correcto (cropOffset Y X = 0 262) para cuadrado central; PNG 192/32/16 y favicon; logo en header/login con contenedor circular; z-index para que sidebar no tape logo; cache-bust ?v=2 en favicon.</v>
@@ -4689,7 +4910,7 @@
         <v>1.5</v>
       </c>
       <c r="B7" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C7" t="str">
         <v>Nueva orden: tipo de operación define monedas (primera = recibida, segunda = entregada). Monedas recibida/entregada se rellenan y deshabilitan según tipo; estilo gris para selects deshabilitados.</v>
@@ -4700,7 +4921,7 @@
         <v>1.6</v>
       </c>
       <c r="B8" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C8" t="str">
         <v>Instrumentación sin intermediario: auto-generación de transacciones para USD-USD, ARS-USD, USD-ARS y ARS-ARS. Al abrir instrumentación vacía se crean dos transacciones (ingreso/egreso efectivo).</v>
@@ -4711,7 +4932,7 @@
         <v>1.7</v>
       </c>
       <c r="B9" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C9" t="str">
         <v>CC intermediario: conciliación por moneda (Debe ≤ Haber), un movimiento Comisión cuando hay tope. Transacciones: moneda/tipo según tipo operación. Orden: distribución comisión visible y editable con intermediario; alerta si 0% intermediario (todos los tipos); ARS-USD en split y validaciones.</v>
@@ -4722,7 +4943,7 @@
         <v>1.8</v>
       </c>
       <c r="B10" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C10" t="str">
         <v>ARS-USD/USD-ARS (sin comisión, montos desde TC). Anulación de órdenes y baja de transacciones. Mensajería interna: showConfirm. Estado de orden se actualiza al instrumentar (auto-complete). ARS-DOLAR eliminado.</v>
@@ -4733,7 +4954,7 @@
         <v>1.9</v>
       </c>
       <c r="B11" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C11" t="str">
         <v>Permisos reordenados: 7 granulares (Ingresar/Editar/Anular Orden, Editar Estado Orden, Ingresar/Editar/Eliminar Transacciones). Eliminado abm_ordenes. Migración SQL y RLS; frontend solo usa los 7 permisos.</v>
@@ -4744,7 +4965,7 @@
         <v>1.10</v>
       </c>
       <c r="B12" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C12" t="str">
         <v>Panel de Control: tarjetas Efectivo/Banco (Saldo Inicial, Saldo Actual destacado, Var. con tendencia); Órdenes pendientes por estado con ojo por fila; Transacciones pendientes con número en círculo; mismo ancho que Efectivo.</v>
@@ -4755,7 +4976,7 @@
         <v>1.11</v>
       </c>
       <c r="B13" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C13" t="str">
         <v>Permisos de vistas por perfil (ver_inicio, ver_ordenes, etc.). Panel parametrizable: tarjetas Efectivo/Banco/Pendientes por permiso (por defecto visor solo pendientes). Seguridad: agrupación Vistas/ABM, subpermisos con sangría e iconos, roles colapsados al iniciar.</v>
@@ -4766,7 +4987,7 @@
         <v>1.12</v>
       </c>
       <c r="B14" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C14" t="str">
         <v>Presentación comercial: barra azul (#0d2137), logo con fondo transparente y contorno blanco, paginado "actual / total", interlineados y leyendas mejorados.</v>
@@ -4777,7 +4998,7 @@
         <v>1.13</v>
       </c>
       <c r="B15" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C15" t="str">
         <v>Filtros en modal Órdenes pendientes: Cliente, Intermediario y Estado. Regla de despliegue sin generación de PPT.</v>
@@ -4788,7 +5009,7 @@
         <v>1.14</v>
       </c>
       <c r="B16" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C16" t="str">
         <v>Tiempo de inactividad: cierre de sesión automático tras X minutos sin actividad (clic, teclado, scroll). Solo Admin configura en Seguridad. Tabla app_config (sql/app_config_session_timeout.sql).</v>
@@ -4799,7 +5020,7 @@
         <v>1.15</v>
       </c>
       <c r="B17" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C17" t="str">
         <v>Sidebar colapsado más visible: borde derecho, botón con fondo y flecha grande para expandir/contraer; aria-label y title dinámicos.</v>
@@ -4810,7 +5031,7 @@
         <v>1.16</v>
       </c>
       <c r="B18" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C18" t="str">
         <v>Iconos cash/Banco en tarjetas Efectivo y Banco. Reorganización: carpeta assets/ con todos los logos e iconos; rutas /assets/ en app y script PPT; regla estructura-proyecto actualizada.</v>
@@ -4821,7 +5042,7 @@
         <v>1.17</v>
       </c>
       <c r="B19" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C19" t="str">
         <v>Cuenta corriente: tabla por moneda (USD/EUR/ARS) con iconos del Panel, Positivo/Negativo, filtro Cliente/Intermediario, solo entidades con saldo; columna Acción; modales ampliados al máximo y arrastrables por el header; icono Ver detalle sin contorno/relleno; regla Modales en .cursor/rules.</v>
@@ -4832,7 +5053,7 @@
         <v>1.18</v>
       </c>
       <c r="B20" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C20" t="str">
         <v>Intermediario: revisión guardado y visualización en órdenes y modales pendientes; intermediario_id en todos los selects de orden para consistencia (refresco detalle, validación totales, actualizar estado).</v>
@@ -4843,7 +5064,7 @@
         <v>1.19</v>
       </c>
       <c r="B21" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C21" t="str">
         <v>Wizard nueva orden: corrección paso instrumentación; al guardar la primera transacción se puede seguir agregando en el mismo paso (fix canEditarTr en renderWizardList).</v>
@@ -4854,7 +5075,7 @@
         <v>1.20</v>
       </c>
       <c r="B22" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C22" t="str">
         <v>Cuenta corriente: todos los movimientos en cualquier estado; Caja solo ejecutada. Auto-complete instrumentación genera CC; doc CUENTA_CORRIENTE_Y_CAJA.md.</v>
@@ -4865,7 +5086,7 @@
         <v>1.21</v>
       </c>
       <c r="B23" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C23" t="str">
         <v>Permisos por menú: menús colapsables (por defecto cerrados), encabezado rol sticky, toggles on/off clicables. Cajas: Ver Efectivo/Banco granular (ver_cajas_efectivo, ver_cajas_banco); tarjetas solo con permiso específico. Intermediarios: Operar (abm_intermediarios) en Seguridad. Cascada: al desactivar acceso al menú se desactivan también los hijos de ese ítem.</v>
@@ -4876,7 +5097,7 @@
         <v>1.22</v>
       </c>
       <c r="B24" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C24" t="str">
         <v>Cuenta corriente: compromiso solo por órdenes no ejecutadas (ganancia no como saldo del cliente). Refresh del modal con saldos y operaciones; botón Refrescar. Lista incluye todos los clientes/intermediarios y quienes tengan compromiso; misma lógica para intermediario.</v>
@@ -4887,7 +5108,7 @@
         <v>1.23</v>
       </c>
       <c r="B25" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C25" t="str">
         <v>Cuenta corriente: concilia sin doble conteo. Movimientos "Transacción pendiente" no se restan del compromiso (solo ejecutados/cierre y manuales), para que saldos por moneda se mantengan visibles cuando falta ejecutar una pata. Leyenda y doc actualizadas.</v>
@@ -4898,7 +5119,7 @@
         <v>1.24</v>
       </c>
       <c r="B26" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C26" t="str">
         <v>Ayudas (help): popovers expandibles para textos largos (scroll), cierre con Escape. Regla .cursor/rules/help-popovers.mdc para mantener el patrón en próximos helps.</v>
@@ -4909,7 +5130,7 @@
         <v>1.25</v>
       </c>
       <c r="B27" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C27" t="str">
         <v>Ayudas (help): los íconos de ayuda ahora abren un modal de Help (en lugar de popover) para mostrar textos largos de forma legible. Regla actualizada para el patrón modal.</v>
@@ -4920,7 +5141,7 @@
         <v>1.26</v>
       </c>
       <c r="B28" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C28" t="str">
         <v>Cargar orden por chat: botón azul (btn-chat) en Órdenes y Panel de Control; tipo de cambio y cálculo del otro monto; al confirmar se crean orden, instrumentación y transacciones automáticas; desde Panel redirige a Órdenes al finalizar.</v>
@@ -4931,7 +5152,7 @@
         <v>1.27</v>
       </c>
       <c r="B29" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C29" t="str">
         <v>Modal Cargar por chat: icono en el título, botón Enviar con estilo unificado y a la derecha del campo de texto.</v>
@@ -4942,7 +5163,7 @@
         <v>1.28</v>
       </c>
       <c r="B30" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C30" t="str">
         <v>Vista Órdenes: filtros Cliente, Intermediario y Estado. Combos de filtros con estilo moderno (select-filtro, puntas redondeadas). Quitar Cotización y Concertada del filtro Estado.</v>
@@ -4953,7 +5174,7 @@
         <v>1.29</v>
       </c>
       <c r="B31" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C31" t="str">
         <v>Tipos de operación: columna usa_intermediario (Intermediario Sí/No). ABM con columnas Intermediario y Activo como switches (mismo estilo que Seguridad). Modal de orden: si el tipo no usa intermediario no se muestra el selector de intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
@@ -4964,7 +5185,7 @@
         <v>1.30</v>
       </c>
       <c r="B32" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C32" t="str">
         <v>Número de orden atómico: función ordenes_insertar_con_proximo_numero en DB (MAX+1 con lock). La app llama a la RPC al crear orden nueva; sin huecos ni colisiones por concurrencia. sql/ordenes_insertar_con_proximo_numero.sql.</v>
@@ -4975,7 +5196,7 @@
         <v>1.31</v>
       </c>
       <c r="B33" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C33" t="str">
         <v>Reajuste tests E2E (timeouts CC) y signos CC regla simple (Pandy debe = negativo). Refresh automático no se ejecuta si hay sección expandida (detalle transacciones en Órdenes o menú/rol en Seguridad) para no colapsar.</v>
@@ -4986,7 +5207,7 @@
         <v>1.32</v>
       </c>
       <c r="B34" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C34" t="str">
         <v>Switch Activo en tablas Clientes e Intermediarios; modales Cliente/Intermediario con toggle; centrado de botón y título en todas las pantallas con switch. Script truncar: orden correcto y orden_comisiones_generadas opcional. Tests E2E: intermediario solo si visible (tipos sin intermediario).</v>
@@ -4997,7 +5218,7 @@
         <v>1.33</v>
       </c>
       <c r="B35" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C35" t="str">
         <v>CC ARS-ARS con intermediario: momento cero cliente (-mr/-me, Compromiso Saldado +me); sin fila Comisión Pandy en sync para que saldo cierre en 0. Mensajes de error login E2E; guía testing con TEST_BASE_URL cuando Vite usa otro puerto.</v>
@@ -5008,7 +5229,7 @@
         <v>1.34</v>
       </c>
       <c r="B36" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C36" t="str">
         <v>CC regla simple (USD-USD, 2 transacciones): compromisos solo cuando al menos una transacción está ejecutada; si ambas pendientes, saldo 0 (no figura deuda).</v>
@@ -5019,7 +5240,7 @@
         <v>1.35</v>
       </c>
       <c r="B37" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C37" t="str">
         <v>Regla de estilos de botones LyP: mismo estilo (border-radius 8px, min-height); con leyenda = icono a la izquierda; solo icono mismo estilo; botón Excel verde. Regla estilos-botones.mdc en Pandi y en Fornitalia, MiGusto, Everfit, Sistema-Contable.</v>
@@ -5030,7 +5251,7 @@
         <v>1.36</v>
       </c>
       <c r="B38" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C38" t="str">
         <v>Reglas que no pueden omitirse: Bitácora, RPC/Supabase y Tests. Al completar tareas hay que actualizar bitácora, revisar RPC en sql/ si aplica y adaptar tests si afectan. bitacora-tareas.mdc y reglas-pandi.mdc.</v>
@@ -5041,7 +5262,7 @@
         <v>1.37</v>
       </c>
       <c r="B39" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C39" t="str">
         <v>Modales: no cerrar al elegir en select (mousedown+click en backdrop). Sesión: mousemove cuenta como actividad para no cerrar por inactividad al mover mouse/trackpad. CC: Tipo op. después de Fecha, sticky y export Excel.</v>
@@ -5052,7 +5273,7 @@
         <v>1.38</v>
       </c>
       <c r="B40" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C40" t="str">
         <v>Producción Vercel: XLSX cargado desde CDN (script en index.html); main.js usa window.XLSX para evitar error "Failed to resolve module specifier xlsx" sin bundler.</v>
@@ -5063,7 +5284,7 @@
         <v>1.39</v>
       </c>
       <c r="B41" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C41" t="str">
         <v>CC regla infalible: ingreso misma moneda aporta -me (Pandy debe su transacción); egreso con ingreso pendiente aporta +mr (resumen muestra deuda del cliente). Sin movimiento extra ganancia Pandy en CC. Doc REGLA_CC_SIMPLE_INFALIBLE.md actualizado.</v>
@@ -5074,7 +5295,7 @@
         <v>1.40</v>
       </c>
       <c r="B42" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C42" t="str">
         <v>Validación egreso cheques: no ejecutar entrega al intermediario si ingreso Cliente→Pandy pendiente. CC resumen: color unificado (verde = a favor de Pandy, rojo = en contra) para cliente e intermediario.</v>
@@ -5085,7 +5306,7 @@
         <v>1.41</v>
       </c>
       <c r="B43" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C43" t="str">
         <v>CC modelo reglas: 16 combinaciones cubiertas por tabla (4 filas por tipo). Tx1 pendiente+contrapartida ejecutada: SUMA_SALDO Y, signo -; comisiones pendientes con signo invertido e INCLUIR Y. Compromiso de Pago con monto de la transacción (195k) no mr (200k).</v>
@@ -5096,7 +5317,7 @@
         <v>1.42</v>
       </c>
       <c r="B44" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C44" t="str">
         <v>Regla Tx1 (P,true) no sumar: saldo cliente +200k cuando Tx2=E. E2E CC combinaciones: 12 combinaciones, esperados y test resistente (detalle); test.step por combinación.</v>
@@ -5107,15 +5328,26 @@
         <v>1.43</v>
       </c>
       <c r="B45" t="str">
-        <v>18/03/2026</v>
+        <v>19/03/2026</v>
       </c>
       <c r="C45" t="str">
         <v>E2E CC combinaciones: esperados alineados con tabla SQL (6 combinaciones); PASS en detalle cuando saldo 0; Real rellenado desde vista Detalle de movimientos (Cliente e Intermediario) cuando no hay fila en Resumen.</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>1.44</v>
+      </c>
+      <c r="B46" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C46" t="str">
+        <v>CHEQUE-ARS canónico (SQL/motor/E2E); modal Nueva orden: selector de tipo con iconos (select oculto para Playwright); listbox position fixed para no recortar por overflow del modal; min-height modal orden; checks moneda CHEQUE en migración/seed; docs y guía E2E.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.45: CC modelo moneda/monto exposición en tabla y motor
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E230"/>
+  <dimension ref="A1:E232"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3918,7 +3918,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3935,7 +3935,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3952,7 +3952,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3969,7 +3969,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B210" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C210" t="str">
         <v>Instrumentación: orden por numero 1,2,3,4</v>
@@ -3986,7 +3986,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B211" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C211" t="str">
         <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
@@ -4003,7 +4003,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B212" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C212" t="str">
         <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
@@ -4020,7 +4020,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B213" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C213" t="str">
         <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
@@ -4037,7 +4037,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B214" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C214" t="str">
         <v>E2E CC combinaciones: subir timeout global</v>
@@ -4054,7 +4054,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B215" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C215" t="str">
         <v>Doc respaldo E2E CC + RPC null-safe</v>
@@ -4071,7 +4071,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B216" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C216" t="str">
         <v>Panel y Cajas: mismos permisos en cards + Cheque ARS</v>
@@ -4088,7 +4088,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B217" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C217" t="str">
         <v>UI card Cheque compacta y alineada</v>
@@ -4105,7 +4105,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B218" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C218" t="str">
         <v>Tipo de operación: iconos moneda y cheque</v>
@@ -4122,7 +4122,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B219" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C219" t="str">
         <v>Tipos de operación: icono configurable (auto / cheques / imagen)</v>
@@ -4139,7 +4139,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B220" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C220" t="str">
         <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
@@ -4156,7 +4156,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B221" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C221" t="str">
         <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
@@ -4173,7 +4173,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B222" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C222" t="str">
         <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
@@ -4190,7 +4190,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B223" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C223" t="str">
         <v>v1.43 Despliegue</v>
@@ -4207,7 +4207,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B224" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C224" t="str">
         <v>CC sync: dedupe por (entidad, orden, monto)</v>
@@ -4224,7 +4224,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B225" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C225" t="str">
         <v>Tipo operación: moneda Cheque (CHEQUE–ARS)</v>
@@ -4241,7 +4241,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B226" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C226" t="str">
         <v>E2E: tipo CHEQUE-ARS en tests CC</v>
@@ -4258,7 +4258,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B227" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C227" t="str">
         <v>Fix SQL CHEQUE en checks de moneda</v>
@@ -4275,7 +4275,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B228" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C228" t="str">
         <v>Canónico CHEQUE-ARS en tabla de verdad</v>
@@ -4292,7 +4292,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B229" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C229" t="str">
         <v>Modal orden: tipo de operación con iconos</v>
@@ -4309,7 +4309,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B230" t="str">
-        <v>10:03</v>
+        <v>10:54</v>
       </c>
       <c r="C230" t="str">
         <v>Fix listbox tipo operación en modal orden</v>
@@ -4321,16 +4321,50 @@
         <v>Desarrollo</v>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B231" t="str">
+        <v>10:54</v>
+      </c>
+      <c r="C231" t="str">
+        <v>CC modelo: moneda y monto de exposición en tabla</v>
+      </c>
+      <c r="D231" t="str">
+        <v>Nuevas columnas en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion (orden_recibida|orden_entregada|transaccion) y *_monto_referencia (mr|me|monto_transaccion|monto_efectivo_intermediario). Motor main.js resolverMonedaYMontoCc*; NULL en ambas = legacy. ARS-USD/USD-USD/USD-ARS: ingreso Cliente→Pandy expone orden_entregada+me (deuda en moneda a entregar). sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; cc_modelo_reglas_tabla.sql y cc_modelo_reglas_todas_combinaciones.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+      <c r="E231" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B232" t="str">
+        <v>10:54</v>
+      </c>
+      <c r="C232" t="str">
+        <v>Despliegue producción v1.45</v>
+      </c>
+      <c r="D232" t="str">
+        <v>Push a main y Vercel --prod: CC exposición configurable en cc_modelo_reglas; sidebar v1.45.</v>
+      </c>
+      <c r="E232" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E232"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4754,15 +4788,23 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
+        <v>CC modelo: moneda e importe de exposición</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Por fila en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion y *_monto_referencia definen en qué moneda y con qué monto se registra el movimiento (orden recibida/entregada, transacción; mr/me/monto_transacción, etc.). Válido para cualquier combinación de monedas configurada en la tabla. NULL en ambas columnas del lado = comportamiento legacy. sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
         <v>Conceptos CC unificados y número de transacción</v>
       </c>
-      <c r="B53" t="str">
+      <c r="B54" t="str">
         <v>Todos los movimientos CC (cliente e intermediario) usan leyendas unificadas (Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo) con sufijo " - Orden x y Trans x". transaccion_numero se guarda en todos los inserts/rows para que la columna Trans. del detalle nunca quede en blanco cuando hay transacción de referencia. Incluye movimientos derivados (pago/cobro de comisiones).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4832,7 +4874,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5345,9 +5387,20 @@
         <v>CHEQUE-ARS canónico (SQL/motor/E2E); modal Nueva orden: selector de tipo con iconos (select oculto para Playwright); listbox position fixed para no recortar por overflow del modal; min-height modal orden; checks moneda CHEQUE en migración/seed; docs y guía E2E.</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>1.45</v>
+      </c>
+      <c r="B47" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C47" t="str">
+        <v>CC modelo: moneda e importe de exposición por fila en cc_modelo_reglas (cliente/intermediario); motor main.js con resolvers; migración SQL y scripts tabla/combinaciones; doc CC_MODELO_ENGINE_TABLA; bitácora y prerrequisito en migración CHEQUE-ARS.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C47"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.46: CC espejo ARS-USD, filtros Movimientos grid, modal orden, montos instrumentación
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E232"/>
+  <dimension ref="A1:E245"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3918,7 +3918,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3935,7 +3935,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3952,7 +3952,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3969,7 +3969,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B210" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C210" t="str">
         <v>Instrumentación: orden por numero 1,2,3,4</v>
@@ -3986,7 +3986,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B211" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C211" t="str">
         <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
@@ -4003,7 +4003,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B212" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C212" t="str">
         <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
@@ -4020,7 +4020,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B213" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C213" t="str">
         <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
@@ -4037,7 +4037,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B214" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C214" t="str">
         <v>E2E CC combinaciones: subir timeout global</v>
@@ -4054,7 +4054,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B215" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C215" t="str">
         <v>Doc respaldo E2E CC + RPC null-safe</v>
@@ -4071,7 +4071,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B216" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C216" t="str">
         <v>Panel y Cajas: mismos permisos en cards + Cheque ARS</v>
@@ -4088,7 +4088,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B217" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C217" t="str">
         <v>UI card Cheque compacta y alineada</v>
@@ -4105,7 +4105,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B218" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C218" t="str">
         <v>Tipo de operación: iconos moneda y cheque</v>
@@ -4122,7 +4122,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B219" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C219" t="str">
         <v>Tipos de operación: icono configurable (auto / cheques / imagen)</v>
@@ -4139,7 +4139,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B220" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C220" t="str">
         <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
@@ -4156,7 +4156,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B221" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C221" t="str">
         <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
@@ -4173,7 +4173,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B222" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C222" t="str">
         <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
@@ -4190,7 +4190,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B223" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C223" t="str">
         <v>v1.43 Despliegue</v>
@@ -4207,7 +4207,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B224" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C224" t="str">
         <v>CC sync: dedupe por (entidad, orden, monto)</v>
@@ -4224,7 +4224,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B225" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C225" t="str">
         <v>Tipo operación: moneda Cheque (CHEQUE–ARS)</v>
@@ -4241,7 +4241,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B226" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C226" t="str">
         <v>E2E: tipo CHEQUE-ARS en tests CC</v>
@@ -4258,7 +4258,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B227" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C227" t="str">
         <v>Fix SQL CHEQUE en checks de moneda</v>
@@ -4275,7 +4275,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B228" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C228" t="str">
         <v>Canónico CHEQUE-ARS en tabla de verdad</v>
@@ -4292,7 +4292,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B229" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C229" t="str">
         <v>Modal orden: tipo de operación con iconos</v>
@@ -4309,7 +4309,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B230" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C230" t="str">
         <v>Fix listbox tipo operación en modal orden</v>
@@ -4326,7 +4326,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B231" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C231" t="str">
         <v>CC modelo: moneda y monto de exposición en tabla</v>
@@ -4343,7 +4343,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B232" t="str">
-        <v>10:54</v>
+        <v>13:11</v>
       </c>
       <c r="C232" t="str">
         <v>Despliegue producción v1.45</v>
@@ -4355,9 +4355,230 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B233" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C233" t="str">
+        <v>CC dos monedas: no duplicar cierre con exposición</v>
+      </c>
+      <c r="D233" t="str">
+        <v>Con reglas que definen cc_cliente_moneda_exposicion/monto_referencia, el motor ya cierra en una moneda; el bloque legacy "Cierre orden" (+monR/-monE) ya no corre (evita saldo USD y ARS simultáneo tras las dos patas). main.js; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B234" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C234" t="str">
+        <v>CC detalle: línea espejo moneda transacción + egreso suma saldo par cerrado</v>
+      </c>
+      <c r="D234" t="str">
+        <v>Sin intermediario y dos monedas: tras movimiento de exposición (p. ej. Cobro en USD), si la transacción es en otra moneda se inserta fila espejo solo detalle (ARS, no suma saldo). Regla egreso ejecutada+contrapartida: cc_cliente_suma_saldo true para cerrar saldo. sql/migracion_cc_modelo_reglas_egreso_par_cerrado_suma_saldo.sql; cc_modelo_reglas_todas_combinaciones / tabla.</v>
+      </c>
+      <c r="E234" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B235" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C235" t="str">
+        <v>CC UI: solapas Saldos y Movimientos</v>
+      </c>
+      <c r="D235" t="str">
+        <v>Vista Cuenta corriente: filtro Tipo Cliente/Intermediario arriba; solapas con iconos (Saldos = mini gráfico barras, Movimientos = lista). Panel Saldos: Refrescar + Exportar Excel + tabla resumen. Panel Movimientos: fechas Desde/Hasta + Refrescar + Exportar + tabla detalle. data-vista resumen/detalle sin cambios (E2E). syncCcPestañasYPaneles en main.js; estilos .cc-solapas/.cc-solapa.</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B236" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C236" t="str">
+        <v>CC Movimientos: columnas al contenido y filtro entidad</v>
+      </c>
+      <c r="D236" t="str">
+        <v>Tabla detalle con clase tabla-cc-detalle-movimientos: table-layout auto, width max-content, celdas white-space nowrap (sin saltos de línea); sticky lateral desactivado en esa vista para no solapar columnas. Combo Cliente/Intermediario (Todos + lista desde movimientos) según tipo; ccDetalleFiltroEntidadId; export Excel respeta filtro.</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B237" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C237" t="str">
+        <v>CC Movimientos: toolbar filtros espaciado y fechas</v>
+      </c>
+      <c r="D237" t="str">
+        <v>Panel Movimientos: toolbar en grid 3 columnas (.cc-toolbar-mov-filtros-grid: Cliente | fechas 1fr | acciones); column-gap clamp; ≤720px columna única; inputs cc-input-fecha; select-filtro; móvil 44px en fechas.</v>
+      </c>
+      <c r="E237" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B238" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C238" t="str">
+        <v>SPA: gesto trackpad horizontal no dispara atrás</v>
+      </c>
+      <c r="D238" t="str">
+        <v>index.html: overscroll-behavior-x none en html/body; contain en .main-content, .tabla-clientes-wrap, .tabla-movimientos-wrap, .modal .modal-body, inicio-caja-tabla y wraps en ≤768px. Evita que el scroll horizontal en CC Movimientos (y otras tablas) cierre la app por navegación atrás. Regla .cursor/rules/gestos-trackpad-overscroll-spa.mdc y mención en reglas-pandi.</v>
+      </c>
+      <c r="E238" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B239" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C239" t="str">
+        <v>USD-USD: comisión visible en CC + E2E ajustado</v>
+      </c>
+      <c r="D239" t="str">
+        <v>Reglas cc_modelo para USD-USD sin intermediario incluyen es_comision (Comisión del acuerdo) visible en Movimientos (incluir_en_detalle=true) sin impactar saldo (sumar_al_saldo=false). Archivos SQL: cc_modelo_reglas_todas_combinaciones, cc_modelo_reglas_tabla y migracion_cc_modelo_reglas_comision_usd_usd_sin_intermediario.sql. E2E orden-cc agrega validación de esa comisión en vista Movimientos.</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B240" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C240" t="str">
+        <v>CC sin int: Cobro Realizado visible + comisión con nro trans.</v>
+      </c>
+      <c r="D240" t="str">
+        <v>cc_modelo_reglas: ingreso Cliente→Pandy con par cerrado pasa incluir_en_mov_cc_cliente=true (ARS-USD, USD-USD, USD-ARS). Migración migracion_cc_modelo_reglas_sin_int_incluir_cobro_par_cerrado.sql. main.js: concepto Comisión del acuerdo usa número de la trans. de ingreso cliente→Pandy (evita Trans ?). Doc CC_MODELO_ENGINE_TABLA.</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B241" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Modal orden: sin duplicar moneda/montos (bloque azul)</v>
+      </c>
+      <c r="D241" t="str">
+        <v>USD-USD y CHEQUE-ARS (primeros datos): ocultas las filas Moneda recibimos + Monto y Moneda entregamos + Monto en la zona blanca (inputs siguen en DOM para guardado y E2E; ids orden-row-moneda-monto-* para que insertBefore de dos monedas no rompa el toggle). Más aire en caja azul entre importe/tasa y Monto a Recibir/Entregar (margin-top, padding-top, separador). index.html + main.js adaptarFormularioOrden.</v>
+      </c>
+      <c r="E241" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B242" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Instrumentación: ancho columna Monto</v>
+      </c>
+      <c r="D242" t="str">
+        <v>Inputs .input-monto-transaccion-tabla: se quitó max-width 8rem (cortaba ARS grandes). min-width 11rem, max-width none, border-radius 8px, tabular-nums. Columna Monto min-width 15rem en #orden-inst-tabla y #tabla-transacciones. Wrap mantiene scroll horizontal si hace falta.</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B243" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C243" t="str">
+        <v>CC ARS-USD: espejo Compromiso en moneda recibida</v>
+      </c>
+      <c r="D243" t="str">
+        <v>Con ambas transacciones ejecutadas, el detalle mostraba -mr ARS en Cobro (espejo ingreso) sin fila compensatoria en ARS con originante Pandy. Se agrega línea espejo en egreso Pandy→Cliente: moneda = moneda recibida del acuerdo, monto = signo*mr, transaccion_id del egreso, solo detalle (no suma saldo). Simétrico a USD-ARS (espejo en USD). main.js sincronizarCcYCajaDesdeOrden; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B244" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C244" t="str">
+        <v>CC Movimientos: toolbar grid 3 columnas</v>
+      </c>
+      <c r="D244" t="str">
+        <v>Filtros ya no usan .vista-toolbar: .cc-toolbar-mov-filtros-grid con Cliente | fechas (1fr) | Refrescar/Excel; column-gap clamp; ≤720px una columna. Evita encimar combo con Desde (sin conflicto gap global tablet).</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B245" t="str">
+        <v>13:11</v>
+      </c>
+      <c r="C245" t="str">
+        <v>v1.46 Despliegue</v>
+      </c>
+      <c r="D245" t="str">
+        <v>Producción Vercel: versión sidebar 1.46; CC Movimientos grid; espejo compromiso ARS-USD; modal orden y montos instrumentación; docs y bitácora al día.</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E232"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E245"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4471,7 +4692,7 @@
         <v>Vista Cuenta corriente</v>
       </c>
       <c r="B13" t="str">
-        <v>Momento cero: 2 filas (Debe + Compensación) con ambas monedas; concepto con número interno de orden. Saldo = suma con sumar_al_saldo; detalle con incluir_en_detalle. Tabla detalle: Tipo op. como iconos (incluye icono configurable por tipo); export Excel con código en texto. Filtro Cliente/Intermediario; modal detalle. sql/truncar_ordenes_transacciones.sql.</v>
+        <v>Solapas Saldos y Movimientos; en Movimientos barra de filtros en grid 3 columnas (Cliente | fechas Desde/Hasta | Refrescar/Excel), sin flex vista-toolbar. Filtro por entidad; columnas del listado al ancho del contenido (scroll horizontal). Filtro Tipo compartido. Saldo = sumar_al_saldo; detalle = incluir_en_detalle. Export Excel. Modal por fila.</v>
       </c>
     </row>
     <row r="14">
@@ -4599,7 +4820,7 @@
         <v>Tipo de operación y monedas en orden</v>
       </c>
       <c r="B29" t="str">
-        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris).</v>
+        <v>En Nueva orden / Editar orden, el tipo de operación define monedas: primera = recibida, segunda = entregada. Los selects se rellenan y deshabilitan (gris). En USD-USD y CHEQUE-ARS con bloque azul no se muestran de nuevo moneda/montos debajo de la fecha (solo lectura arriba); más separación visual entre filas del bloque azul.</v>
       </c>
     </row>
     <row r="30">
@@ -4791,7 +5012,7 @@
         <v>CC modelo: moneda e importe de exposición</v>
       </c>
       <c r="B53" t="str">
-        <v>Por fila en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion y *_monto_referencia definen en qué moneda y con qué monto se registra el movimiento (orden recibida/entregada, transacción; mr/me/monto_transacción, etc.). Válido para cualquier combinación de monedas configurada en la tabla. NULL en ambas columnas del lado = comportamiento legacy. sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+        <v>Por fila en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion y *_monto_referencia definen en qué moneda y con qué monto se registra el movimiento (orden recibida/entregada, transacción; mr/me/monto_transacción, etc.). Sin intermediario y dos monedas: espejo en ingreso (moneda transacción) y espejo en egreso (mr en moneda recibida, originante Pandy) solo detalle. sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
       </c>
     </row>
     <row r="54">
@@ -4874,7 +5095,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5398,9 +5619,20 @@
         <v>CC modelo: moneda e importe de exposición por fila en cc_modelo_reglas (cliente/intermediario); motor main.js con resolvers; migración SQL y scripts tabla/combinaciones; doc CC_MODELO_ENGINE_TABLA; bitácora y prerrequisito en migración CHEQUE-ARS.</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>1.46</v>
+      </c>
+      <c r="B48" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Modal orden (primeros datos): sin duplicar moneda/montos; más aire bloque azul. Instrumentación: columna Monto ancha para ARS. CC ARS-USD: espejo Compromiso en moneda recibida (detalle). CC Movimientos: filtros en grid 3 columnas. Trackpad overscroll SPA; reglas SQL CC sin int cobro par cerrado; comisión USD-USD; E2E ajustes.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.47: alinear CC por tabla y cerrar E2E activos
Consolida cc_modelo_reglas como fuente de verdad para P,E y USD-USD: ingreso pendiente con contrapartida usa orden_recibida+mr, y USD-USD refleja cobro bruto con cierre final por comisión al par cerrado. Actualiza migraciones/documentación y deja verdes los E2E de combinaciones activas.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E245"/>
+  <dimension ref="A1:E249"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3918,7 +3918,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3935,7 +3935,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3952,7 +3952,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3969,7 +3969,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B210" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C210" t="str">
         <v>Instrumentación: orden por numero 1,2,3,4</v>
@@ -3986,7 +3986,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B211" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C211" t="str">
         <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
@@ -4003,7 +4003,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B212" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C212" t="str">
         <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
@@ -4020,7 +4020,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B213" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C213" t="str">
         <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
@@ -4037,7 +4037,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B214" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C214" t="str">
         <v>E2E CC combinaciones: subir timeout global</v>
@@ -4054,7 +4054,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B215" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C215" t="str">
         <v>Doc respaldo E2E CC + RPC null-safe</v>
@@ -4071,7 +4071,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B216" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C216" t="str">
         <v>Panel y Cajas: mismos permisos en cards + Cheque ARS</v>
@@ -4088,7 +4088,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B217" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C217" t="str">
         <v>UI card Cheque compacta y alineada</v>
@@ -4105,7 +4105,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B218" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C218" t="str">
         <v>Tipo de operación: iconos moneda y cheque</v>
@@ -4122,7 +4122,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B219" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C219" t="str">
         <v>Tipos de operación: icono configurable (auto / cheques / imagen)</v>
@@ -4139,7 +4139,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B220" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C220" t="str">
         <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
@@ -4156,7 +4156,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B221" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C221" t="str">
         <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
@@ -4173,7 +4173,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B222" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C222" t="str">
         <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
@@ -4190,7 +4190,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B223" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C223" t="str">
         <v>v1.43 Despliegue</v>
@@ -4207,7 +4207,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B224" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C224" t="str">
         <v>CC sync: dedupe por (entidad, orden, monto)</v>
@@ -4224,7 +4224,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B225" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C225" t="str">
         <v>Tipo operación: moneda Cheque (CHEQUE–ARS)</v>
@@ -4241,7 +4241,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B226" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C226" t="str">
         <v>E2E: tipo CHEQUE-ARS en tests CC</v>
@@ -4258,7 +4258,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B227" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C227" t="str">
         <v>Fix SQL CHEQUE en checks de moneda</v>
@@ -4275,7 +4275,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B228" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C228" t="str">
         <v>Canónico CHEQUE-ARS en tabla de verdad</v>
@@ -4292,7 +4292,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B229" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C229" t="str">
         <v>Modal orden: tipo de operación con iconos</v>
@@ -4309,7 +4309,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B230" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C230" t="str">
         <v>Fix listbox tipo operación en modal orden</v>
@@ -4326,7 +4326,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B231" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C231" t="str">
         <v>CC modelo: moneda y monto de exposición en tabla</v>
@@ -4343,7 +4343,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B232" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C232" t="str">
         <v>Despliegue producción v1.45</v>
@@ -4360,7 +4360,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B233" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C233" t="str">
         <v>CC dos monedas: no duplicar cierre con exposición</v>
@@ -4377,7 +4377,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B234" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C234" t="str">
         <v>CC detalle: línea espejo moneda transacción + egreso suma saldo par cerrado</v>
@@ -4394,7 +4394,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B235" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C235" t="str">
         <v>CC UI: solapas Saldos y Movimientos</v>
@@ -4411,7 +4411,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B236" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C236" t="str">
         <v>CC Movimientos: columnas al contenido y filtro entidad</v>
@@ -4428,7 +4428,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B237" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C237" t="str">
         <v>CC Movimientos: toolbar filtros espaciado y fechas</v>
@@ -4445,7 +4445,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B238" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C238" t="str">
         <v>SPA: gesto trackpad horizontal no dispara atrás</v>
@@ -4462,7 +4462,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B239" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C239" t="str">
         <v>USD-USD: comisión visible en CC + E2E ajustado</v>
@@ -4479,7 +4479,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B240" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C240" t="str">
         <v>CC sin int: Cobro Realizado visible + comisión con nro trans.</v>
@@ -4496,7 +4496,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B241" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C241" t="str">
         <v>Modal orden: sin duplicar moneda/montos (bloque azul)</v>
@@ -4513,7 +4513,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B242" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C242" t="str">
         <v>Instrumentación: ancho columna Monto</v>
@@ -4530,7 +4530,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B243" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C243" t="str">
         <v>CC ARS-USD: espejo Compromiso en moneda recibida</v>
@@ -4547,7 +4547,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B244" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C244" t="str">
         <v>CC Movimientos: toolbar grid 3 columnas</v>
@@ -4564,7 +4564,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B245" t="str">
-        <v>13:11</v>
+        <v>15:14</v>
       </c>
       <c r="C245" t="str">
         <v>v1.46 Despliegue</v>
@@ -4576,16 +4576,84 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B246" t="str">
+        <v>15:14</v>
+      </c>
+      <c r="C246" t="str">
+        <v>E2E CC tipos 2 transacciones (combinaciones)</v>
+      </c>
+      <c r="D246" t="str">
+        <v>Nuevo test tests/e2e/cc-tipos-activos-combinaciones.spec.js: 4 combinaciones P/E por ARS-USD, USD-ARS y USD-USD con montos enteros fijos; expectativas en cc-tipos-activos-esperado.js; log test-results/cc-tipos-activos-log.xlsx. Scripts npm test:e2e-cc-tipos-2tx y test:e2e-cc-activos-completo (con cc-combinaciones). CHEQUE-ARS sigue en cc-combinaciones.spec.js. docs/TESTING_E2E_GUIA.md §1.8.</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B247" t="str">
+        <v>15:14</v>
+      </c>
+      <c r="C247" t="str">
+        <v>CC sin int P,E: regla tabla única fuente de verdad</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Ingreso Cliente→Pandy pendiente + contrapartida ejecutada: cc_modelo_reglas con orden_recibida+mr, compromiso_cobrar, suma saldo e incluir mov. Evita neto 0 por −me USD vs +me egreso en ARS-USD/USD-ARS/USD-USD. SQL: cc_modelo_reglas_tabla/todas_combinaciones, migracion_cc_modelo_reglas_ingreso_pendiente_par_exposicion_mr.sql, migracion tipos_sin_intermediario y moneda_exposicion (excepción). E2E cc-tipos-activos-esperado P,E actualizado. Doc CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B248" t="str">
+        <v>15:14</v>
+      </c>
+      <c r="C248" t="str">
+        <v>E2E USD-USD E,P: expectativa alineada a tabla</v>
+      </c>
+      <c r="D248" t="str">
+        <v>cc-tipos-activos-esperado: saldo USD −9.700 (exposición me tras cobro Tx1); caja +10.000. Antes +10.000 confundía importe bruto con posición CC; los 300 USD son margen/comisión Pandy respecto de 10.000 vs 9.700.</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="B249" t="str">
+        <v>15:14</v>
+      </c>
+      <c r="C249" t="str">
+        <v>USD-USD: cobro bruto -10000 en CC y cierre E,E con comisión</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Ajuste fuente de verdad cc_modelo_reglas: ingreso Cliente→Pandy (sin intermediario, USD-USD) expone transaccion+monto_transaccion (cobro bruto -10000). Para cerrar E,E en 0, comisión ejecutada+contrapartida true suma saldo (+300). SQL: cc_modelo_reglas_tabla, cc_modelo_reglas_todas_combinaciones, migracion_cc_modelo_reglas_tipos_sin_intermediario, migracion_cc_modelo_reglas_moneda_exposicion, migracion_cc_modelo_reglas_comision_usd_usd_sin_intermediario y nueva migracion_cc_modelo_reglas_usd_usd_cobro_bruto_y_cierre_comision.sql. E2E esperado actualizado.</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Desarrollo</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E245"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E249"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B55"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -4953,79 +5021,87 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Número de transacción y convención caja</v>
+        <v>E2E CC combinaciones (tipos 2 tx)</v>
       </c>
       <c r="B46" t="str">
-        <v>Transacciones tienen número interno (transacciones.numero, secuencia) para trazabilidad. Movimientos de caja originados por transacción usan concepto: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Panel de transacciones muestra columna Nro. sql/migracion_transacciones_numero.sql.</v>
+        <v>cc-tipos-activos-combinaciones.spec.js: combinaciones Tx1/Tx2 para ARS-USD, USD-ARS y USD-USD; cliente E2E CC TiposActivos; npm run test:e2e-cc-tipos-2tx o test:e2e-cc-activos-completo junto a cc-combinaciones (CHEQUE-ARS).</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Log E2E hoja Caja</v>
+        <v>Número de transacción y convención caja</v>
       </c>
       <c r="B47" t="str">
-        <v>Hoja Caja en Excel: una fila por transacción (y una final) con columnas Saldo_Caja_EF/BA por moneda (Esp, App, Resultado). irACajasYLeerSaldos espera fin de carga para que los saldos no queden en blanco. tests/e2e/orden-cc.spec.js y e2e-log-excel.js.</v>
+        <v>Transacciones tienen número interno (transacciones.numero, secuencia) para trazabilidad. Movimientos de caja originados por transacción usan concepto: "Ingreso/Egreso de [moneda], por [monto], nro orden [nro], nro transacción [nro]". Panel de transacciones muestra columna Nro. sql/migracion_transacciones_numero.sql.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Movimientos de caja estructurados</v>
+        <v>Log E2E hoja Caja</v>
       </c>
       <c r="B48" t="str">
-        <v>Tabla movimientos_caja con orden_numero y transaccion_numero; vista Cajas: columnas Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Caja, Concepto. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
+        <v>Hoja Caja en Excel: una fila por transacción (y una final) con columnas Saldo_Caja_EF/BA por moneda (Esp, App, Resultado). irACajasYLeerSaldos espera fin de carga para que los saldos no queden en blanco. tests/e2e/orden-cc.spec.js y e2e-log-excel.js.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Caja: movimiento por comisión Pandy</v>
+        <v>Movimientos de caja estructurados</v>
       </c>
       <c r="B49" t="str">
-        <v>Cuando hay comisión Pandy (misma moneda, sin transacción Ganancia) la sincronización agrega un movimiento de caja (ingreso efectivo por la comisión) para que la caja cierre en cero en operaciones de cobro de cheques. transaccion_id null; al re-sincronizar se borran esos movimientos por orden.</v>
+        <v>Tabla movimientos_caja con orden_numero y transaccion_numero; vista Cajas: columnas Origen, Nro orden, Nro transacción, Tipo (Ingreso/Egreso), Caja, Concepto. sql/migracion_movimientos_caja_orden_transaccion_numero.sql.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Tipos de operación: Intermediario Sí/No</v>
+        <v>Caja: movimiento por comisión Pandy</v>
       </c>
       <c r="B50" t="str">
-        <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
+        <v>Cuando hay comisión Pandy (misma moneda, sin transacción Ganancia) la sincronización agrega un movimiento de caja (ingreso efectivo por la comisión) para que la caja cierre en cero en operaciones de cobro de cheques. transaccion_id null; al re-sincronizar se borran esos movimientos por orden.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Número de orden atómico (MAX+1)</v>
+        <v>Tipos de operación: Intermediario Sí/No</v>
       </c>
       <c r="B51" t="str">
-        <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
+        <v>Columna usa_intermediario en tipos_operacion. En ABM Tipos de operación: columna Intermediario (Sí/No) y checkbox "Usa intermediario" en modal Nuevo/Editar. En modal de orden: si el tipo no usa intermediario, el selector de intermediario no se muestra ni se menciona; si usa intermediario se muestra como antes. Al guardar orden se fuerza intermediario_id = null cuando el tipo no usa intermediario. sql/migracion_tipos_operacion_usa_intermediario.sql.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Utils y RPC sync CC/caja</v>
+        <v>Número de orden atómico (MAX+1)</v>
       </c>
       <c r="B52" t="str">
-        <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
+        <v>Al crear orden nueva la app llama a la RPC ordenes_insertar_con_proximo_numero: en la DB se asigna numero = MAX(numero)+1 bajo pg_advisory_xact_lock para evitar huecos y colisiones por concurrencia. Fallback a INSERT sin numero si la columna no existe. sql/ordenes_insertar_con_proximo_numero.sql.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>CC modelo: moneda e importe de exposición</v>
+        <v>Utils y RPC sync CC/caja</v>
       </c>
       <c r="B53" t="str">
-        <v>Por fila en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion y *_monto_referencia definen en qué moneda y con qué monto se registra el movimiento (orden recibida/entregada, transacción; mr/me/monto_transacción, etc.). Sin intermediario y dos monedas: espejo en ingreso (moneda transacción) y espejo en egreso (mr en moneda recibida, originante Pandy) solo detalle. sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+        <v>utils.js en raíz con formatMonto, formatImporteDisplay, formatImporteParaInput, formatearCeldaMoneda. RPC sync_cc_caja_orden: front construye rows de CC y caja, backend hace delete+insert en una transacción. Fallback en cliente si la RPC no está desplegada. sql/rpc_sync_cc_caja_orden.sql.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
+        <v>CC modelo: moneda e importe de exposición</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Por fila en cc_modelo_reglas: cc_cliente/intermediario_moneda_exposicion y *_monto_referencia definen en qué moneda y con qué monto se registra el movimiento (orden recibida/entregada, transacción; mr/me/monto_transacción, etc.). Sin intermediario y dos monedas: espejo en ingreso (moneda transacción) y espejo en egreso (mr en moneda recibida, originante Pandy) solo detalle. sql/migracion_cc_modelo_reglas_moneda_exposicion.sql; docs/CC_MODELO_ENGINE_TABLA.md.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
         <v>Conceptos CC unificados y número de transacción</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B55" t="str">
         <v>Todos los movimientos CC (cliente e intermediario) usan leyendas unificadas (Pago Realizado, Cobro Realizado, Compromiso de Pago, Compromiso a Cobrar, Comisión del acuerdo) con sufijo " - Orden x y Trans x". transaccion_numero se guarda en todos los inserts/rows para que la columna Trans. del detalle nunca quede en blanco cuando hay transacción de referencia. Incluye movimientos derivados (pago/cobro de comisiones).</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5095,7 +5171,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5630,9 +5706,20 @@
         <v>Modal orden (primeros datos): sin duplicar moneda/montos; más aire bloque azul. Instrumentación: columna Monto ancha para ARS. CC ARS-USD: espejo Compromiso en moneda recibida (detalle). CC Movimientos: filtros en grid 3 columnas. Trackpad overscroll SPA; reglas SQL CC sin int cobro par cerrado; comisión USD-USD; E2E ajustes.</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>1.47</v>
+      </c>
+      <c r="B49" t="str">
+        <v>19/03/2026</v>
+      </c>
+      <c r="C49" t="str">
+        <v>CC tabla única fuente de verdad: ajuste P,E (ingreso pendiente + contrapartida ejecutada) en dos monedas con orden_recibida+mr; USD-USD cobro bruto -10000 (monto_transaccion) y cierre E,E con comisión +300 al saldo cuando par cerrado. Nuevas migraciones SQL puntuales, documentación del motor y E2E completos (cc-combinaciones + tipos 2tx) en verde.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v1.48: ajuste visual iconos y entrega insumo presentación
Actualiza a v1.48 con iconos de moneda en círculo gris sutil manteniendo el estilo previo de botones, y agrega el insumo HTML/PDF de main.js para IA de presentaciones. Se actualiza bitácora y versión de despliegue.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E249"/>
+  <dimension ref="A1:E253"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B2" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C2" t="str">
         <v>Setup Pandi</v>
@@ -450,7 +450,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B3" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C3" t="str">
         <v>SQL tablas y seguridad</v>
@@ -467,7 +467,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B4" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C4" t="str">
         <v>UI base y login</v>
@@ -484,7 +484,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B5" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C5" t="str">
         <v>ABM Clientes</v>
@@ -501,7 +501,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B6" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C6" t="str">
         <v>Vista Cajas</v>
@@ -518,7 +518,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B7" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C7" t="str">
         <v>ABM Tipos de movimiento de caja</v>
@@ -535,7 +535,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B8" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C8" t="str">
         <v>Iconos y regla botones</v>
@@ -552,7 +552,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B9" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C9" t="str">
         <v>Importes y formato</v>
@@ -569,7 +569,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B10" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C10" t="str">
         <v>Vista Órdenes</v>
@@ -586,7 +586,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B11" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C11" t="str">
         <v>Edición movimientos de caja</v>
@@ -603,7 +603,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B12" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C12" t="str">
         <v>Vista Cuenta corriente</v>
@@ -620,7 +620,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B13" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C13" t="str">
         <v>Vista Inicio</v>
@@ -637,7 +637,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B14" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C14" t="str">
         <v>Convención cuenta corriente</v>
@@ -654,7 +654,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B15" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C15" t="str">
         <v>Edición movimientos cuenta corriente</v>
@@ -671,7 +671,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B16" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C16" t="str">
         <v>Responsividad móvil</v>
@@ -688,7 +688,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B17" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C17" t="str">
         <v>Mensajería propia (toast)</v>
@@ -705,7 +705,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B18" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C18" t="str">
         <v>Tasa descuento intermediario y caja banco</v>
@@ -722,7 +722,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B19" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C19" t="str">
         <v>Conceptos CC y layout</v>
@@ -739,7 +739,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B20" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C20" t="str">
         <v>Responsive móvil reforzado</v>
@@ -756,7 +756,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B21" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C21" t="str">
         <v>Panel de Control sin título redundante</v>
@@ -773,7 +773,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B22" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C22" t="str">
         <v>Permisos editar orden y cambiar estado transacción</v>
@@ -790,7 +790,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B23" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C23" t="str">
         <v>Logo y favicon desde Emoji-de-WhatsApp-panda</v>
@@ -807,7 +807,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B24" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C24" t="str">
         <v>Tipo operación define monedas en Nueva orden</v>
@@ -824,7 +824,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B25" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C25" t="str">
         <v>Transacciones auto sin intermediario</v>
@@ -841,7 +841,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B26" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C26" t="str">
         <v>v1.7: CC intermediario, transacciones y orden</v>
@@ -858,7 +858,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B27" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C27" t="str">
         <v>v1.8: ARS-USD/USD-ARS, anulación, mensajería interna, estado al instrumentar</v>
@@ -875,7 +875,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B28" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C28" t="str">
         <v>v1.9: Permisos reordenados (7 granulares, sin abm_ordenes)</v>
@@ -892,7 +892,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B29" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C29" t="str">
         <v>v1.10: Panel de Control rediseñado</v>
@@ -909,7 +909,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B30" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C30" t="str">
         <v>Permisos de vistas por perfil</v>
@@ -926,7 +926,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B31" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C31" t="str">
         <v>Panel de Control parametrizable</v>
@@ -943,7 +943,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B32" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C32" t="str">
         <v>Seguridad: agrupación y subpermisos</v>
@@ -960,7 +960,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B33" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C33" t="str">
         <v>Seguridad: roles colapsados</v>
@@ -977,7 +977,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B34" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C34" t="str">
         <v>Presentación comercial PPT</v>
@@ -994,7 +994,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B35" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C35" t="str">
         <v>Filtros en Órdenes pendientes</v>
@@ -1011,7 +1011,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B36" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C36" t="str">
         <v>Regla de despliegue sin PPT</v>
@@ -1028,7 +1028,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B37" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C37" t="str">
         <v>Tiempo de inactividad</v>
@@ -1045,7 +1045,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B38" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C38" t="str">
         <v>Sidebar colapsado más visible</v>
@@ -1062,7 +1062,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B39" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C39" t="str">
         <v>Iconos y carpeta assets</v>
@@ -1079,7 +1079,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B40" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C40" t="str">
         <v>Ajustes modal Nueva transacción</v>
@@ -1096,7 +1096,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B41" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C41" t="str">
         <v>Modal transacción: moneda del tipo y conversión inversa</v>
@@ -1113,7 +1113,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B42" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C42" t="str">
         <v>Tipos de operación: moneda_in/moneda_out y ABM</v>
@@ -1130,7 +1130,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B43" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C43" t="str">
         <v>Cuenta corriente: vista Todos y modal detalle</v>
@@ -1147,7 +1147,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B44" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C44" t="str">
         <v>v1.17: Cuenta corriente y modales</v>
@@ -1164,7 +1164,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B45" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C45" t="str">
         <v>v1.18: Intermediario en órdenes y transacciones</v>
@@ -1181,7 +1181,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B46" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C46" t="str">
         <v>v1.19: Wizard instrumentación</v>
@@ -1198,7 +1198,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B47" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C47" t="str">
         <v>v1.20: Cuenta corriente y Caja</v>
@@ -1215,7 +1215,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B48" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C48" t="str">
         <v>Cards Cajas como Panel de Control</v>
@@ -1232,7 +1232,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B49" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C49" t="str">
         <v>Propuesta permisos por menú</v>
@@ -1249,7 +1249,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B50" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C50" t="str">
         <v>Permisos por opción de menú (UI)</v>
@@ -1266,7 +1266,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B51" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C51" t="str">
         <v>Cajas: Ver granular y mensajes al desactivar</v>
@@ -1283,7 +1283,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B52" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C52" t="str">
         <v>Seguridad: anclaje y toggles</v>
@@ -1300,7 +1300,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B53" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C53" t="str">
         <v>Seguridad: menús colapsables</v>
@@ -1317,7 +1317,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B54" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C54" t="str">
         <v>Cajas: tarjeta solo por permiso específico</v>
@@ -1334,7 +1334,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B55" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C55" t="str">
         <v>Intermediarios: Operar en permisos</v>
@@ -1351,7 +1351,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B56" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C56" t="str">
         <v>Seguridad: cascada al desactivar padre</v>
@@ -1368,7 +1368,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B57" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C57" t="str">
         <v>CC: refresh con nueva lógica y botón Refrescar</v>
@@ -1385,7 +1385,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B58" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C58" t="str">
         <v>CC: compromiso solo órdenes no ejecutadas</v>
@@ -1402,7 +1402,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B59" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C59" t="str">
         <v>CC: evitar doble conteo pendientes</v>
@@ -1419,7 +1419,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B60" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C60" t="str">
         <v>v1.22 Despliegue</v>
@@ -1436,7 +1436,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B61" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C61" t="str">
         <v>v1.23 Despliegue</v>
@@ -1453,7 +1453,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B62" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C62" t="str">
         <v>Help: popovers expandibles y texto CC</v>
@@ -1470,7 +1470,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B63" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C63" t="str">
         <v>Help: leyendas colapsadas por defecto</v>
@@ -1487,7 +1487,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B64" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C64" t="str">
         <v>Help: modal en toda la app</v>
@@ -1504,7 +1504,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B65" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C65" t="str">
         <v>v1.24 Despliegue</v>
@@ -1521,7 +1521,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B66" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C66" t="str">
         <v>v1.25 Despliegue</v>
@@ -1538,7 +1538,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B67" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C67" t="str">
         <v>Cargar orden por chat (MVP local)</v>
@@ -1555,7 +1555,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B68" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C68" t="str">
         <v>Chat orden: tipo de cambio y alta directa</v>
@@ -1572,7 +1572,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B69" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C69" t="str">
         <v>Chat orden: un monto + TC calcula el otro</v>
@@ -1589,7 +1589,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B70" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C70" t="str">
         <v>Botón Cargar por chat: estilo y Panel de Control</v>
@@ -1606,7 +1606,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B71" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C71" t="str">
         <v>Chat orden: auto-generar transacciones al confirmar</v>
@@ -1623,7 +1623,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B72" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C72" t="str">
         <v>Modal chat: icono en título, Enviar a la derecha del input</v>
@@ -1640,7 +1640,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B73" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C73" t="str">
         <v>Filtros vista Órdenes y estilo combos</v>
@@ -1657,7 +1657,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B74" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C74" t="str">
         <v>Cuenta corriente: solo ejecutadas y Pandy-Intermediario</v>
@@ -1674,7 +1674,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B75" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C75" t="str">
         <v>Cuenta corriente: saldo solo movimientos ejecutados</v>
@@ -1691,7 +1691,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B76" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C76" t="str">
         <v>Cuenta corriente: saldo neto con transacciones pendientes</v>
@@ -1708,7 +1708,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B77" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C77" t="str">
         <v>Split ingreso cliente→Pandy: ganancia explícita</v>
@@ -1725,7 +1725,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B78" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C78" t="str">
         <v>CC: cuando una parte cumplió, el resto participa</v>
@@ -1742,7 +1742,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B79" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C79" t="str">
         <v>Conceptos CC y columnas Pagador/Cobrador</v>
@@ -1759,7 +1759,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B80" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C80" t="str">
         <v>Orden: numero legible y orden_id obligatorio en CC</v>
@@ -1776,7 +1776,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B81" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C81" t="str">
         <v>Orden: fallback sin numero, borrador y botón Instrumentación</v>
@@ -1793,7 +1793,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B82" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C82" t="str">
         <v>Modal orden dos monedas: El cliente compra primero, TC, resto calculado</v>
@@ -1810,7 +1810,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B83" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C83" t="str">
         <v>Órdenes: número visible al volver; carga instrumentación</v>
@@ -1827,7 +1827,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B84" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C84" t="str">
         <v>Cuenta corriente: Cobro/Deuda, sin Debe-Haber, deuda pendiente</v>
@@ -1844,7 +1844,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B85" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C85" t="str">
         <v>CC momento cero: registros pendientes por moneda</v>
@@ -1861,7 +1861,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B86" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C86" t="str">
         <v>CC: invertir signos al cerrar; saldo = suma de toda la tabla</v>
@@ -1878,7 +1878,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B87" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C87" t="str">
         <v>CC momento cero: signos correctos y solo invertir moneda ejecutada</v>
@@ -1895,7 +1895,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B88" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C88" t="str">
         <v>Editar transacción y CC: respetar momento cero</v>
@@ -1912,7 +1912,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B89" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C89" t="str">
         <v>CC nueva lógica: Debe/Compensación y Cancelación de deuda</v>
@@ -1929,7 +1929,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B90" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C90" t="str">
         <v>CC momento cero: concepto con número interno de orden</v>
@@ -1946,7 +1946,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B91" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C91" t="str">
         <v>Script truncado y reset secuencia orden</v>
@@ -1963,7 +1963,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B92" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C92" t="str">
         <v>CC: sin movimientos Conversión de moneda</v>
@@ -1980,7 +1980,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B93" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C93" t="str">
         <v>CC Cancelación: ambos montos por orden</v>
@@ -1997,7 +1997,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B94" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C94" t="str">
         <v>CC Resumen: saldo desde movimientos + moneda compromiso</v>
@@ -2014,7 +2014,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B95" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C95" t="str">
         <v>CC: revisión regla en todos los flujos</v>
@@ -2031,7 +2031,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B96" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C96" t="str">
         <v>CC: auto-compensación al ejecutar con monto distinto al de la orden</v>
@@ -2048,7 +2048,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B97" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C97" t="str">
         <v>Modal instrumentación: Monto, Estado y Modo de pago editables en tabla; Editar solo para el resto</v>
@@ -2065,7 +2065,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B98" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C98" t="str">
         <v>Split CC: no duplicar al ejecutar la transacción diferencia</v>
@@ -2082,7 +2082,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B99" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C99" t="str">
         <v>CC intermediario: deuda Pandy en rojo y regla de oro</v>
@@ -2099,7 +2099,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B100" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C100" t="str">
         <v>CC: regla unificada y una sola carga de pendientes</v>
@@ -2116,7 +2116,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B101" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C101" t="str">
         <v>CC intermediario: insertarMovimientosCcParaTransaccion alineado</v>
@@ -2133,7 +2133,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B102" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C102" t="str">
         <v>CC intermediario y truncate: número de orden y setval</v>
@@ -2150,7 +2150,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B103" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C103" t="str">
         <v>Paso 3 CC cliente: Cancelación por monto real y sin doble comisión</v>
@@ -2167,7 +2167,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B104" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C104" t="str">
         <v>CC cliente: comisión como resultado del split y saldo 0</v>
@@ -2184,7 +2184,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B105" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C105" t="str">
         <v>CC cliente: no zeroar originales y comisión visible (+1.250 y -1.250)</v>
@@ -2201,7 +2201,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B106" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C106" t="str">
         <v>Sincronización CC y caja desde orden + transacciones</v>
@@ -2218,7 +2218,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B107" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C107" t="str">
         <v>Split egreso CC: moneda correcta en Debe/Compensación</v>
@@ -2235,7 +2235,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B108" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C108" t="str">
         <v>CC resumen: agrupar por orden_id para una sola moneda</v>
@@ -2252,7 +2252,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B109" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C109" t="str">
         <v>CC Cancelación por monto de la transacción</v>
@@ -2269,7 +2269,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B110" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C110" t="str">
         <v>Split CC: diferencia desde fila, no desde orden</v>
@@ -2286,7 +2286,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B111" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C111" t="str">
         <v>Tarea de análisis: modal transacción con ejecutadas</v>
@@ -2303,7 +2303,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B112" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C112" t="str">
         <v>Modal transacción ejecutada: solo concepto editable</v>
@@ -2320,7 +2320,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B113" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C113" t="str">
         <v>Edición transacción: sin restricción; re-estructurar regla al editar</v>
@@ -2337,7 +2337,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B114" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C114" t="str">
         <v>Reajuste CC y caja al editar monto o modo de pago</v>
@@ -2354,7 +2354,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B115" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C115" t="str">
         <v>Split al pasar a ejecutada: sincronizar monto desde tabla</v>
@@ -2371,7 +2371,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B116" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C116" t="str">
         <v>CC: evitar movimientos con monto_usd/ars/eur en null</v>
@@ -2388,7 +2388,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B117" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C117" t="str">
         <v>CC: no mostrar comisión Pandy como deuda del cliente</v>
@@ -2405,7 +2405,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B118" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C118" t="str">
         <v>Tasas de descuento: reconocer coma decimal</v>
@@ -2422,7 +2422,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B119" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C119" t="str">
         <v>Modal orden más ancho</v>
@@ -2439,7 +2439,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B120" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C120" t="str">
         <v>Split sin momento cero (ARS-ARS CHEQUE)</v>
@@ -2456,7 +2456,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B121" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C121" t="str">
         <v>Split + CC + caja para cualquier tipo de operación</v>
@@ -2473,7 +2473,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B122" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C122" t="str">
         <v>Operación CHEQUE: no cambiar modo de pago en transacciones con Cheque</v>
@@ -2490,7 +2490,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B123" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C123" t="str">
         <v>ARS-ARS CHEQUE: generar Ganancia del acuerdo cuando el cliente completa</v>
@@ -2507,7 +2507,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B124" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C124" t="str">
         <v>Split sin momento cero: no crear resto cuando el cliente ya completó</v>
@@ -2524,7 +2524,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B125" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C125" t="str">
         <v>Ganancia del acuerdo: descontar comisión de una ingreso cliente→Pandy</v>
@@ -2541,7 +2541,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B126" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C126" t="str">
         <v>CC Intermediario: incluir obligaciones pendientes (misma regla que cliente)</v>
@@ -2558,7 +2558,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B127" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C127" t="str">
         <v>CC Intermediario momento cero: actualizar fila al ejecutar egreso Pandy→Intermediario</v>
@@ -2575,7 +2575,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B128" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C128" t="str">
         <v>CC USD-ARS: dos registros (Cancelación + Contraparte) en todos los flujos</v>
@@ -2592,7 +2592,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B129" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C129" t="str">
         <v>CC regla simple: Compromiso y Compromiso Saldado</v>
@@ -2609,7 +2609,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B130" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C130" t="str">
         <v>CC vista: saldo solo transacciones ejecutadas</v>
@@ -2626,7 +2626,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B131" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C131" t="str">
         <v>CC Intermediario reversa y relojería: misma regla que cliente + sync al cerrar</v>
@@ -2643,7 +2643,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B132" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C132" t="str">
         <v>Momento cero CHEQUE: misma regla para todos los tipos de operación</v>
@@ -2660,7 +2660,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B133" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C133" t="str">
         <v>CC intermediario momento cero: permitir estado pendiente en DB</v>
@@ -2677,7 +2677,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B134" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C134" t="str">
         <v>Reglas CC, caja e instrucciones: mejoras finales</v>
@@ -2694,7 +2694,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B135" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C135" t="str">
         <v>CC intermediario: misma estructura que CC cliente (monto_usd, monto_ars, monto_eur)</v>
@@ -2711,7 +2711,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B136" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C136" t="str">
         <v>CC intermediario: cerrar fila Compensación al ejecutar ingreso Int→Pandy</v>
@@ -2728,7 +2728,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B137" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C137" t="str">
         <v>CC intermediario: saldo solo desde movimientos (sin capa pendientes)</v>
@@ -2745,7 +2745,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B138" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C138" t="str">
         <v>CC cliente: Cancelación alineada con monto de la transacción</v>
@@ -2762,7 +2762,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B139" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C139" t="str">
         <v>CC intermediario: alta de comisión del intermediario</v>
@@ -2779,7 +2779,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B140" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C140" t="str">
         <v>CC cliente: movimiento por Ganancia del acuerdo para cerrar saldo</v>
@@ -2796,7 +2796,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B141" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C141" t="str">
         <v>CC intermediario: nunca null en monto_usd/ars/eur; comisión al ejecutar cobro</v>
@@ -2813,7 +2813,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B142" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C142" t="str">
         <v>CC intermediario: descuento y comisión al entregar cheques</v>
@@ -2830,7 +2830,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B143" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C143" t="str">
         <v>CC cliente: movimiento Ganancia desde datos de la orden</v>
@@ -2847,7 +2847,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B144" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C144" t="str">
         <v>Tabla orden_comisiones_generadas y CC a prueba de re-ejecución</v>
@@ -2864,7 +2864,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B145" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C145" t="str">
         <v>Reajuste tests E2E y signos CC regla simple</v>
@@ -2881,7 +2881,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B146" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C146" t="str">
         <v>Refresh sin colapsar secciones expandidas</v>
@@ -2898,7 +2898,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B147" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C147" t="str">
         <v>Tests E2E: intermediario solo si visible (tipos sin intermediario)</v>
@@ -2915,7 +2915,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B148" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C148" t="str">
         <v>Modales Cliente e Intermediario: Activo como switch on/off</v>
@@ -2932,7 +2932,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B149" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C149" t="str">
         <v>Tablas Clientes e Intermediarios: columna Activo con switch on/off</v>
@@ -2949,7 +2949,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B150" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C150" t="str">
         <v>ARS-ARS CHEQUE: no ejecutar compensación legacy al cerrar instrumentación</v>
@@ -2966,7 +2966,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B151" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C151" t="str">
         <v>Montos a cero al cambiar estado (ARS-ARS con intermediario)</v>
@@ -2983,7 +2983,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B152" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C152" t="str">
         <v>Evitar updates de monto 0 en transacciones</v>
@@ -3000,7 +3000,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B153" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C153" t="str">
         <v>CC intermediario: segundo +49.250 cuando Pandy entrega cheques</v>
@@ -3017,7 +3017,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B154" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C154" t="str">
         <v>CC cliente: +monto Pago Pandy al cliente cuando egreso Pandy→cliente ejecutada</v>
@@ -3034,7 +3034,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B155" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C155" t="str">
         <v>CC cliente: Cobro nominal 50.000 no se toca (compensa con comisión)</v>
@@ -3051,7 +3051,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B156" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C156" t="str">
         <v>CC cliente: solo Comisión Pandy -1.250 cuando hay Ganancia (saldo 0)</v>
@@ -3068,7 +3068,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B157" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C157" t="str">
         <v>CC intermediario: ingreso Int→Pandy con signo negativo (Pago Intermediario a Pandy)</v>
@@ -3085,7 +3085,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B158" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C158" t="str">
         <v>CC intermediario: una sola fila Intermediario debe a Pandy</v>
@@ -3102,7 +3102,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B159" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C159" t="str">
         <v>CC intermediario: Comisión +750 y 3 líneas desde momento cero</v>
@@ -3119,7 +3119,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B160" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C160" t="str">
         <v>CC intermediario: no agregar Pago Intermediario a Pandy -49.250</v>
@@ -3136,7 +3136,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B161" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C161" t="str">
         <v>CC cliente: split de transacciones (un solo Cobro nominal)</v>
@@ -3153,7 +3153,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B162" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C162" t="str">
         <v>No dividir transacción por comisión: acuerdo = una instrucción</v>
@@ -3170,7 +3170,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B163" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C163" t="str">
         <v>CC intermediario: saldo +49.250 al ejecutar egreso Pandy→Int</v>
@@ -3187,7 +3187,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B164" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C164" t="str">
         <v>Reversar a pendiente: solo una vez por transacción</v>
@@ -3204,7 +3204,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B165" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C165" t="str">
         <v>Test E2E orden ARS-ARS y cuenta corriente</v>
@@ -3221,7 +3221,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B166" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C166" t="str">
         <v>E2E pruebas 4, 5 y 6: control de caja en log y test</v>
@@ -3238,7 +3238,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B167" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C167" t="str">
         <v>Número de transacción interno y convención movimientos de caja</v>
@@ -3255,7 +3255,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B168" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C168" t="str">
         <v>Log E2E hoja Caja y movimientos de caja estructurados</v>
@@ -3272,7 +3272,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B169" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C169" t="str">
         <v>Log E2E Caja: transacción por transacción y saldos no en blanco</v>
@@ -3289,7 +3289,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B170" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C170" t="str">
         <v>Caja: movimiento por comisión Pandy (sin transacción Ganancia)</v>
@@ -3306,7 +3306,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B171" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C171" t="str">
         <v>Tipos de operación: Intermediario Sí/No</v>
@@ -3323,7 +3323,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B172" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C172" t="str">
         <v>Número de orden MAX+1 atómico en DB</v>
@@ -3340,7 +3340,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B173" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C173" t="str">
         <v>v1.33 Despliegue</v>
@@ -3357,7 +3357,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B174" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C174" t="str">
         <v>v1.34 Despliegue</v>
@@ -3374,7 +3374,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B175" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C175" t="str">
         <v>Utils y RPC sync CC/caja (modelo Sistema-Contable)</v>
@@ -3391,7 +3391,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B176" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C176" t="str">
         <v>RPC transacciones_cambiar_estado</v>
@@ -3408,7 +3408,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B177" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C177" t="str">
         <v>v1.35 Despliegue</v>
@@ -3425,7 +3425,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B178" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C178" t="str">
         <v>CC Detalle movimientos: Originante siempre visible, sin filtro Todos</v>
@@ -3442,7 +3442,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B179" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C179" t="str">
         <v>CC: Originante = Pagador, leyendas concepto y columnas cortas</v>
@@ -3459,7 +3459,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B180" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C180" t="str">
         <v>v1.36 Despliegue</v>
@@ -3476,7 +3476,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B181" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C181" t="str">
         <v>CC: unificación de conceptos y transaccion_numero</v>
@@ -3493,7 +3493,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B182" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C182" t="str">
         <v>CC intermediario: sin duplicado Compromiso a Cobrar; regla RCA y por transacción</v>
@@ -3510,7 +3510,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B183" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C183" t="str">
         <v>CC y caja eficientes: actuar solo por transacción, sin borrar/repoblar</v>
@@ -3527,7 +3527,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B184" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C184" t="str">
         <v>CC detalle movimientos: columna Tipo de operación</v>
@@ -3544,7 +3544,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B185" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C185" t="str">
         <v>CC: Tipo op. después de Fecha, sticky y export Excel</v>
@@ -3561,7 +3561,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B186" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C186" t="str">
         <v>Modales: no cerrar al elegir opción de menú/select</v>
@@ -3578,7 +3578,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B187" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C187" t="str">
         <v>Sesión: movimiento de mouse/trackpad cuenta como actividad</v>
@@ -3595,7 +3595,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B188" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C188" t="str">
         <v>Despliegue v1.38</v>
@@ -3612,7 +3612,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B189" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C189" t="str">
         <v>Tests E2E: esperar actualización estado antes de ir a CC</v>
@@ -3629,7 +3629,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B190" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C190" t="str">
         <v>CC intermediario: estado pendiente en momento cero</v>
@@ -3646,7 +3646,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B191" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C191" t="str">
         <v>Regla simple e infalible CC y caja</v>
@@ -3663,7 +3663,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B192" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C192" t="str">
         <v>CC dos monedas: RPC COALESCE y front montos explícitos</v>
@@ -3680,7 +3680,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B193" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C193" t="str">
         <v>CC: un movimiento = una moneda (la de la transacción)</v>
@@ -3697,7 +3697,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B194" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C194" t="str">
         <v>CC: cierre orden dos monedas para saldo 0 en resumen</v>
@@ -3714,7 +3714,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B195" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C195" t="str">
         <v>Regla CC: 4 premisas clave documentadas</v>
@@ -3731,7 +3731,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B196" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C196" t="str">
         <v>CC cliente: corrección signos (positivo=cliente debe, negativo=Pandy debe)</v>
@@ -3748,7 +3748,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B197" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C197" t="str">
         <v>CC: resumen con ingreso pendiente muestra deuda del cliente (mr)</v>
@@ -3765,7 +3765,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B198" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C198" t="str">
         <v>Validación egreso cheques</v>
@@ -3782,7 +3782,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B199" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C199" t="str">
         <v>CC resumen: color a favor / en contra de Pandy</v>
@@ -3799,7 +3799,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B200" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C200" t="str">
         <v>Tabla cc_modelo_reglas en Supabase</v>
@@ -3816,7 +3816,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B201" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C201" t="str">
         <v>CC intermediario: comisión solo si Tx3 o Tx4 ejecutada</v>
@@ -3833,7 +3833,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B202" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C202" t="str">
         <v>Motor CC desde tabla cc_modelo_reglas</v>
@@ -3850,7 +3850,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B203" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C203" t="str">
         <v>Reglas CC para todos los tipos activos</v>
@@ -3867,7 +3867,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B204" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C204" t="str">
         <v>Reversión sin límite de veces</v>
@@ -3884,7 +3884,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B205" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C205" t="str">
         <v>Tabla CC alineada con Excel (regla madre completa)</v>
@@ -3901,7 +3901,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B206" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C206" t="str">
         <v>v1.41 Despliegue</v>
@@ -3918,7 +3918,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B207" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C207" t="str">
         <v>CC: dos flags por movimiento (sumar_al_saldo / incluir_en_detalle)</v>
@@ -3935,7 +3935,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B208" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C208" t="str">
         <v>Regla Tx1 (P,true): no sumar al saldo cliente</v>
@@ -3952,7 +3952,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B209" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C209" t="str">
         <v>E2E CC combinaciones: 12 combinaciones y test resistente</v>
@@ -3969,7 +3969,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B210" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C210" t="str">
         <v>Instrumentación: orden por numero 1,2,3,4</v>
@@ -3986,7 +3986,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B211" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C211" t="str">
         <v>Orden por pagador al crear transacciones (1 Cliente, 2 Pandy, 3 Int)</v>
@@ -4003,7 +4003,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B212" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C212" t="str">
         <v>Limpieza base E2E antes de tests (solo desarrollo)</v>
@@ -4020,7 +4020,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B213" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C213" t="str">
         <v>P,P,P,P saldo 0: regla Tx4 + RPC sumar_al_saldo/incluir_en_detalle</v>
@@ -4037,7 +4037,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B214" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C214" t="str">
         <v>E2E CC combinaciones: subir timeout global</v>
@@ -4054,7 +4054,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B215" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C215" t="str">
         <v>Doc respaldo E2E CC + RPC null-safe</v>
@@ -4071,7 +4071,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B216" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C216" t="str">
         <v>Panel y Cajas: mismos permisos en cards + Cheque ARS</v>
@@ -4088,7 +4088,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B217" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C217" t="str">
         <v>UI card Cheque compacta y alineada</v>
@@ -4105,7 +4105,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B218" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C218" t="str">
         <v>Tipo de operación: iconos moneda y cheque</v>
@@ -4122,7 +4122,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B219" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C219" t="str">
         <v>Tipos de operación: icono configurable (auto / cheques / imagen)</v>
@@ -4139,7 +4139,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B220" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C220" t="str">
         <v>E2E CC combinaciones: esperados alineados con tabla SQL</v>
@@ -4156,7 +4156,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B221" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C221" t="str">
         <v>E2E CC combinaciones: PASS cuando saldo 0 y sin fila en resumen</v>
@@ -4173,7 +4173,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B222" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C222" t="str">
         <v>E2E CC combinaciones: Real desde vista Detalle de movimientos</v>
@@ -4190,7 +4190,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B223" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C223" t="str">
         <v>v1.43 Despliegue</v>
@@ -4207,7 +4207,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B224" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C224" t="str">
         <v>CC sync: dedupe por (entidad, orden, monto)</v>
@@ -4224,7 +4224,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B225" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C225" t="str">
         <v>Tipo operación: moneda Cheque (CHEQUE–ARS)</v>
@@ -4241,7 +4241,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B226" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C226" t="str">
         <v>E2E: tipo CHEQUE-ARS en tests CC</v>
@@ -4258,7 +4258,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B227" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C227" t="str">
         <v>Fix SQL CHEQUE en checks de moneda</v>
@@ -4275,7 +4275,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B228" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C228" t="str">
         <v>Canónico CHEQUE-ARS en tabla de verdad</v>
@@ -4292,7 +4292,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B229" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C229" t="str">
         <v>Modal orden: tipo de operación con iconos</v>
@@ -4309,7 +4309,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B230" t="str">
-        <v>15:14</v>
+        <v>15:57</v>
       </c>
       <c r="C230" t="str">
         <v>Fix listbox tipo operación en modal orden</v>
@@ -4326,7 +4326,7 @@
         <v>19/03/2026</v>
       </c>
       <c r="B231" t=